<commit_message>
T1.8: test infra — coverage gate, proptest, fuzz, bot agent, traceability, 50 fixture dossiers
Demo: just demo T1.8 + docs/demos/T1.8/fixtures-contact-sheet.png. just verify now runs coverage, pytest, frontend, traceability.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/space-compute-gantt-v3.xlsx
+++ b/docs/space-compute-gantt-v3.xlsx
@@ -1518,7 +1518,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Test infra: coverage, fuzz, Playwright+axe, bot-…</t>
+          <t>Test infra: coverage gate, proptest, fuzz, bot-a…</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1541,7 +1541,7 @@
         </is>
       </c>
       <c r="I18" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J18">
         <f>IF(I18&gt;=1,"Done",IF(TODAY()&gt;F18,"Late",IF(I18&gt;0,"In progress","Not started")))</f>
@@ -3656,7 +3656,7 @@
         </is>
       </c>
       <c r="I63" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J63">
         <f>IF(I63&gt;=1,"Done",IF(TODAY()&gt;F63,"Late",IF(I63&gt;0,"In progress","Not started")))</f>

</xml_diff>

<commit_message>
plan: Phase 1 progress — 13/14 foundation tasks done, T1.7 rendering (30%); add owner task T8.14 (R2 bucket)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/space-compute-gantt-v3.xlsx
+++ b/docs/space-compute-gantt-v3.xlsx
@@ -600,7 +600,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF100"/>
+  <dimension ref="A1:AF101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1259,7 +1259,7 @@
         </is>
       </c>
       <c r="I12" s="4" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="J12">
         <f>IF(I12&gt;=1,"Done",IF(TODAY()&gt;F12,"Late",IF(I12&gt;0,"In progress","Not started")))</f>
@@ -4657,7 +4657,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>T8.1</t>
+          <t>T8.14</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -4667,26 +4667,26 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Staging deploy, deploy workflow, snapshots, cycl…</t>
+          <t>Create Cloudflare R2 bucket + API token + custom…</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>sonnet-5</t>
+          <t>human</t>
         </is>
       </c>
       <c r="E85" s="3" t="n">
-        <v>46407</v>
+        <v>46316</v>
       </c>
       <c r="F85" s="3" t="n">
-        <v>46408</v>
+        <v>46316</v>
       </c>
       <c r="G85" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>T7.1</t>
+          <t>T1.7</t>
         </is>
       </c>
       <c r="I85" s="4" t="n">
@@ -4704,7 +4704,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>T8.2</t>
+          <t>T8.1</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -4714,26 +4714,26 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Upload subjects/protocol/honeypots to staging</t>
+          <t>Staging deploy, deploy workflow, snapshots, cycl…</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>haiku-4.5</t>
+          <t>sonnet-5</t>
         </is>
       </c>
       <c r="E86" s="3" t="n">
-        <v>46409</v>
+        <v>46407</v>
       </c>
       <c r="F86" s="3" t="n">
-        <v>46409</v>
+        <v>46408</v>
       </c>
       <c r="G86" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>T8.1,T7.6</t>
+          <t>T7.1</t>
         </is>
       </c>
       <c r="I86" s="4" t="n">
@@ -4751,7 +4751,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>T8.5</t>
+          <t>T8.2</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -4761,26 +4761,26 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Fund prod treasury with ICP float (10–20 ICP) + …</t>
+          <t>Upload subjects/protocol/honeypots to staging</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>human</t>
+          <t>haiku-4.5</t>
         </is>
       </c>
       <c r="E87" s="3" t="n">
-        <v>46428</v>
+        <v>46409</v>
       </c>
       <c r="F87" s="3" t="n">
-        <v>46428</v>
+        <v>46409</v>
       </c>
       <c r="G87" t="n">
         <v>1</v>
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>T8.6</t>
+          <t>T8.14,T8.1,T7.6</t>
         </is>
       </c>
       <c r="I87" s="4" t="n">
@@ -4798,7 +4798,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>T8.3</t>
+          <t>T8.5</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -4808,7 +4808,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Closed beta (10-20 owners)</t>
+          <t>Fund prod treasury with ICP float (10–20 ICP) + …</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -4817,17 +4817,17 @@
         </is>
       </c>
       <c r="E88" s="3" t="n">
-        <v>46412</v>
+        <v>46428</v>
       </c>
       <c r="F88" s="3" t="n">
-        <v>46423</v>
+        <v>46428</v>
       </c>
       <c r="G88" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>T8.2,T6.10</t>
+          <t>T8.6</t>
         </is>
       </c>
       <c r="I88" s="4" t="n">
@@ -4845,7 +4845,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>T8.4</t>
+          <t>T8.3</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -4855,12 +4855,12 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Beta fixes &amp; tuning</t>
+          <t>Closed beta (10-20 owners)</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>sonnet-5</t>
+          <t>human</t>
         </is>
       </c>
       <c r="E89" s="3" t="n">
@@ -4892,7 +4892,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>T8.6</t>
+          <t>T8.4</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -4902,7 +4902,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Production deploy, II metadata, treasury watch l…</t>
+          <t>Beta fixes &amp; tuning</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -4911,17 +4911,17 @@
         </is>
       </c>
       <c r="E90" s="3" t="n">
-        <v>46426</v>
+        <v>46412</v>
       </c>
       <c r="F90" s="3" t="n">
-        <v>46427</v>
+        <v>46423</v>
       </c>
       <c r="G90" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>T8.3,T8.4,T8.13</t>
+          <t>T8.2,T6.10</t>
         </is>
       </c>
       <c r="I90" s="4" t="n">
@@ -4939,7 +4939,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>T8.7</t>
+          <t>T8.6</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -4949,26 +4949,26 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Public launch</t>
+          <t>Production deploy, II metadata, treasury watch l…</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>human</t>
+          <t>sonnet-5</t>
         </is>
       </c>
       <c r="E91" s="3" t="n">
-        <v>46429</v>
+        <v>46426</v>
       </c>
       <c r="F91" s="3" t="n">
-        <v>46429</v>
+        <v>46427</v>
       </c>
       <c r="G91" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>T8.6,T8.5,T9.5</t>
+          <t>T8.3,T8.4,T8.13</t>
         </is>
       </c>
       <c r="I91" s="4" t="n">
@@ -4986,36 +4986,36 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>T9.1</t>
+          <t>T8.7</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>P9</t>
+          <t>P8</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Import mockups (Claude Design), reconcile, desig…</t>
+          <t>Public launch</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>sonnet-5</t>
+          <t>human</t>
         </is>
       </c>
       <c r="E92" s="3" t="n">
-        <v>46409</v>
+        <v>46429</v>
       </c>
       <c r="F92" s="3" t="n">
-        <v>46414</v>
+        <v>46429</v>
       </c>
       <c r="G92" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>T6.10</t>
+          <t>T8.6,T8.5,T9.5</t>
         </is>
       </c>
       <c r="I92" s="4" t="n">
@@ -5033,7 +5033,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>T9.2</t>
+          <t>T9.1</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -5043,7 +5043,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Style public pages: landing, museum, discovery, …</t>
+          <t>Import mockups (Claude Design), reconcile, desig…</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -5052,17 +5052,17 @@
         </is>
       </c>
       <c r="E93" s="3" t="n">
-        <v>46415</v>
+        <v>46409</v>
       </c>
       <c r="F93" s="3" t="n">
-        <v>46420</v>
+        <v>46414</v>
       </c>
       <c r="G93" t="n">
         <v>4</v>
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>T9.1</t>
+          <t>T6.10</t>
         </is>
       </c>
       <c r="I93" s="4" t="n">
@@ -5080,7 +5080,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>T9.3</t>
+          <t>T9.2</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -5090,7 +5090,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Style owner flows: spawn, dashboard, connect age…</t>
+          <t>Style public pages: landing, museum, discovery, …</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -5127,7 +5127,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>T9.4</t>
+          <t>T9.3</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -5137,22 +5137,22 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Style admin console + about/legal/practice pages</t>
+          <t>Style owner flows: spawn, dashboard, connect age…</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>haiku-4.5</t>
+          <t>sonnet-5</t>
         </is>
       </c>
       <c r="E95" s="3" t="n">
-        <v>46421</v>
+        <v>46415</v>
       </c>
       <c r="F95" s="3" t="n">
-        <v>46422</v>
+        <v>46420</v>
       </c>
       <c r="G95" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H95" t="inlineStr">
         <is>
@@ -5174,7 +5174,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>T9.5</t>
+          <t>T9.4</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -5184,7 +5184,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Responsive/mobile pass, visual-regression baseli…</t>
+          <t>Style admin console + about/legal/practice pages</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -5193,17 +5193,17 @@
         </is>
       </c>
       <c r="E96" s="3" t="n">
-        <v>46423</v>
+        <v>46421</v>
       </c>
       <c r="F96" s="3" t="n">
-        <v>46426</v>
+        <v>46422</v>
       </c>
       <c r="G96" t="n">
         <v>2</v>
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>T9.2,T9.3,T9.4</t>
+          <t>T9.1</t>
         </is>
       </c>
       <c r="I96" s="4" t="n">
@@ -5221,36 +5221,36 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>T8.13</t>
+          <t>T9.5</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>P8</t>
+          <t>P9</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Custom domain + II alternative origins</t>
+          <t>Responsive/mobile pass, visual-regression baseli…</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>human</t>
+          <t>haiku-4.5</t>
         </is>
       </c>
       <c r="E97" s="3" t="n">
-        <v>46409</v>
+        <v>46423</v>
       </c>
       <c r="F97" s="3" t="n">
-        <v>46409</v>
+        <v>46426</v>
       </c>
       <c r="G97" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>T8.1</t>
+          <t>T9.2,T9.3,T9.4</t>
         </is>
       </c>
       <c r="I97" s="4" t="n">
@@ -5268,7 +5268,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>T8.12</t>
+          <t>T8.13</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -5278,7 +5278,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Firebase projects (staging/prod) + GA4 funnels &amp;…</t>
+          <t>Custom domain + II alternative origins</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -5287,17 +5287,17 @@
         </is>
       </c>
       <c r="E98" s="3" t="n">
-        <v>46296</v>
+        <v>46409</v>
       </c>
       <c r="F98" s="3" t="n">
-        <v>46296</v>
+        <v>46409</v>
       </c>
       <c r="G98" t="n">
         <v>1</v>
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>T0.4</t>
+          <t>T8.1</t>
         </is>
       </c>
       <c r="I98" s="4" t="n">
@@ -5315,7 +5315,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>T8.8</t>
+          <t>T8.12</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -5325,7 +5325,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Compliance check for card &amp; crypto fuel packs (r…</t>
+          <t>Firebase projects (staging/prod) + GA4 funnels &amp;…</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -5337,10 +5337,10 @@
         <v>46296</v>
       </c>
       <c r="F99" s="3" t="n">
-        <v>46302</v>
+        <v>46296</v>
       </c>
       <c r="G99" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H99" t="inlineStr">
         <is>
@@ -5362,7 +5362,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>T8.9</t>
+          <t>T8.8</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -5372,7 +5372,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Enable BTC/ETH on production (card stays off)</t>
+          <t>Compliance check for card &amp; crypto fuel packs (r…</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -5381,17 +5381,17 @@
         </is>
       </c>
       <c r="E100" s="3" t="n">
-        <v>46428</v>
+        <v>46296</v>
       </c>
       <c r="F100" s="3" t="n">
-        <v>46428</v>
+        <v>46302</v>
       </c>
       <c r="G100" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>T8.6,T8.8</t>
+          <t>T0.4</t>
         </is>
       </c>
       <c r="I100" s="4" t="n">
@@ -5406,8 +5406,55 @@
         <v/>
       </c>
     </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>T8.9</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>P8</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Enable BTC/ETH on production (card stays off)</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>human</t>
+        </is>
+      </c>
+      <c r="E101" s="3" t="n">
+        <v>46428</v>
+      </c>
+      <c r="F101" s="3" t="n">
+        <v>46428</v>
+      </c>
+      <c r="G101" t="n">
+        <v>1</v>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>T8.6,T8.8</t>
+        </is>
+      </c>
+      <c r="I101" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J101">
+        <f>IF(I101&gt;=1,"Done",IF(TODAY()&gt;F101,"Late",IF(I101&gt;0,"In progress","Not started")))</f>
+        <v/>
+      </c>
+      <c r="K101">
+        <f>G101*I101</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="L2:AF100">
+  <conditionalFormatting sqref="L2:AF101">
     <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="1">
       <formula>AND(L$1+6&gt;=$E2,L$1&lt;=$F2,L$1&lt;=$E2+($F2-$E2)*$I2)</formula>
     </cfRule>
@@ -5445,7 +5492,7 @@
       <formula>AND(TODAY()&gt;=L$1,TODAY()&lt;L$1+7)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J2:J100">
+  <conditionalFormatting sqref="J2:J101">
     <cfRule type="expression" priority="13" dxfId="12">
       <formula>LEFT(J2,4)="Late"</formula>
     </cfRule>
@@ -5976,7 +6023,7 @@
         <v/>
       </c>
       <c r="G12" s="17">
-        <f>IF(C12&gt;0,SUM(Gantt!K2:K100)/C12,0)</f>
+        <f>IF(C12&gt;0,SUM(Gantt!K2:K101)/C12,0)</f>
         <v/>
       </c>
       <c r="H12" s="18" t="n">

</xml_diff>

<commit_message>
plan: T6.1 reset to in_progress 30% after review (mock data, no auth/tests); T1.7 44%
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/space-compute-gantt-v3.xlsx
+++ b/docs/space-compute-gantt-v3.xlsx
@@ -1259,7 +1259,7 @@
         </is>
       </c>
       <c r="I12" s="4" t="n">
-        <v>0.35</v>
+        <v>0.45</v>
       </c>
       <c r="J12">
         <f>IF(I12&gt;=1,"Done",IF(TODAY()&gt;F12,"Late",IF(I12&gt;0,"In progress","Not started")))</f>
@@ -3656,7 +3656,7 @@
         </is>
       </c>
       <c r="I63" s="4" t="n">
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="J63">
         <f>IF(I63&gt;=1,"Done",IF(TODAY()&gt;F63,"Late",IF(I63&gt;0,"In progress","Not started")))</f>

</xml_diff>

<commit_message>
T8.15: owner review of the discovery + peer-review agent process
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/space-compute-gantt-v3.xlsx
+++ b/docs/space-compute-gantt-v3.xlsx
@@ -600,7 +600,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF102"/>
+  <dimension ref="A1:AF103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -5409,7 +5409,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>T8.8</t>
+          <t>T8.15</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -5419,7 +5419,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Compliance check for card &amp; crypto fuel packs (r…</t>
+          <t>Owner review: discovery + peer-review agent proc…</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -5431,10 +5431,10 @@
         <v>46296</v>
       </c>
       <c r="F101" s="3" t="n">
-        <v>46302</v>
+        <v>46296</v>
       </c>
       <c r="G101" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H101" t="inlineStr">
         <is>
@@ -5456,7 +5456,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>T8.9</t>
+          <t>T8.8</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -5466,7 +5466,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Enable BTC/ETH on production (card stays off)</t>
+          <t>Compliance check for card &amp; crypto fuel packs (r…</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -5475,17 +5475,17 @@
         </is>
       </c>
       <c r="E102" s="3" t="n">
-        <v>46429</v>
+        <v>46296</v>
       </c>
       <c r="F102" s="3" t="n">
-        <v>46429</v>
+        <v>46302</v>
       </c>
       <c r="G102" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>T8.6,T8.8</t>
+          <t>T0.4</t>
         </is>
       </c>
       <c r="I102" s="4" t="n">
@@ -5500,8 +5500,55 @@
         <v/>
       </c>
     </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>T8.9</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>P8</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Enable BTC/ETH on production (card stays off)</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>human</t>
+        </is>
+      </c>
+      <c r="E103" s="3" t="n">
+        <v>46429</v>
+      </c>
+      <c r="F103" s="3" t="n">
+        <v>46429</v>
+      </c>
+      <c r="G103" t="n">
+        <v>1</v>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>T8.6,T8.8</t>
+        </is>
+      </c>
+      <c r="I103" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J103">
+        <f>IF(I103&gt;=1,"Done",IF(TODAY()&gt;F103,"Late",IF(I103&gt;0,"In progress","Not started")))</f>
+        <v/>
+      </c>
+      <c r="K103">
+        <f>G103*I103</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="L2:AF102">
+  <conditionalFormatting sqref="L2:AF103">
     <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="1">
       <formula>AND(L$1+6&gt;=$E2,L$1&lt;=$F2,L$1&lt;=$E2+($F2-$E2)*$I2)</formula>
     </cfRule>
@@ -5539,7 +5586,7 @@
       <formula>AND(TODAY()&gt;=L$1,TODAY()&lt;L$1+7)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J2:J102">
+  <conditionalFormatting sqref="J2:J103">
     <cfRule type="expression" priority="13" dxfId="12">
       <formula>LEFT(J2,4)="Late"</formula>
     </cfRule>
@@ -6070,7 +6117,7 @@
         <v/>
       </c>
       <c r="G12" s="17">
-        <f>IF(C12&gt;0,SUM(Gantt!K2:K102)/C12,0)</f>
+        <f>IF(C12&gt;0,SUM(Gantt!K2:K103)/C12,0)</f>
         <v/>
       </c>
       <c r="H12" s="18" t="n">

</xml_diff>

<commit_message>
T1.7: 5,000 JWST dossiers rendered, hashed and QA'd (common-grid RGB)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/space-compute-gantt-v3.xlsx
+++ b/docs/space-compute-gantt-v3.xlsx
@@ -1259,7 +1259,7 @@
         </is>
       </c>
       <c r="I12" s="4" t="n">
-        <v>0.65</v>
+        <v>1</v>
       </c>
       <c r="J12">
         <f>IF(I12&gt;=1,"Done",IF(TODAY()&gt;F12,"Late",IF(I12&gt;0,"In progress","Not started")))</f>
@@ -1964,7 +1964,7 @@
         </is>
       </c>
       <c r="I27" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J27">
         <f>IF(I27&gt;=1,"Done",IF(TODAY()&gt;F27,"Late",IF(I27&gt;0,"In progress","Not started")))</f>

</xml_diff>

<commit_message>
T5.1: done; remove Stripe/card from payments and defer T5.12 (no Stripe until the app is ready)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/space-compute-gantt-v3.xlsx
+++ b/docs/space-compute-gantt-v3.xlsx
@@ -600,7 +600,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF103"/>
+  <dimension ref="A1:AF102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2904,7 +2904,7 @@
         </is>
       </c>
       <c r="I47" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J47">
         <f>IF(I47&gt;=1,"Done",IF(TODAY()&gt;F47,"Late",IF(I47&gt;0,"In progress","Not started")))</f>
@@ -3200,7 +3200,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>T5.12</t>
+          <t>T5.9</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -3210,22 +3210,22 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>stripe_credit endpoint (flag-gated, mock-relay t…</t>
+          <t>ckBTC fuel-pack deposits (address, update_balanc…</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>haiku-4.5</t>
+          <t>opus-5.5 (high)</t>
         </is>
       </c>
       <c r="E54" s="3" t="n">
         <v>46364</v>
       </c>
       <c r="F54" s="3" t="n">
-        <v>46365</v>
+        <v>46366</v>
       </c>
       <c r="G54" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H54" t="inlineStr">
         <is>
@@ -3247,7 +3247,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>T5.9</t>
+          <t>T5.10</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -3257,26 +3257,26 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>ckBTC fuel-pack deposits (address, update_balanc…</t>
+          <t>ckETH fuel-pack deposits</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>opus-5.5 (high)</t>
+          <t>sonnet-5</t>
         </is>
       </c>
       <c r="E55" s="3" t="n">
         <v>46364</v>
       </c>
       <c r="F55" s="3" t="n">
-        <v>46366</v>
+        <v>46365</v>
       </c>
       <c r="G55" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>T5.8</t>
+          <t>T5.8,SP-6</t>
         </is>
       </c>
       <c r="I55" s="4" t="n">
@@ -3294,7 +3294,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>T5.10</t>
+          <t>T5.13</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -3304,7 +3304,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>ckETH fuel-pack deposits</t>
+          <t>Non-ICP payment tests (04 §6.7)</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -3313,17 +3313,17 @@
         </is>
       </c>
       <c r="E56" s="3" t="n">
-        <v>46364</v>
+        <v>46367</v>
       </c>
       <c r="F56" s="3" t="n">
-        <v>46365</v>
+        <v>46370</v>
       </c>
       <c r="G56" t="n">
         <v>2</v>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>T5.8,SP-6</t>
+          <t>T5.9,T5.10</t>
         </is>
       </c>
       <c r="I56" s="4" t="n">
@@ -3341,36 +3341,36 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
+          <t>T5.15</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Payments admin APIs + audit log</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>haiku-4.5</t>
+        </is>
+      </c>
+      <c r="E57" s="3" t="n">
+        <v>46371</v>
+      </c>
+      <c r="F57" s="3" t="n">
+        <v>46371</v>
+      </c>
+      <c r="G57" t="n">
+        <v>1</v>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
           <t>T5.13</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>P5</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>Non-ICP payment tests (04 §6.7)</t>
-        </is>
-      </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>sonnet-5</t>
-        </is>
-      </c>
-      <c r="E57" s="3" t="n">
-        <v>46367</v>
-      </c>
-      <c r="F57" s="3" t="n">
-        <v>46370</v>
-      </c>
-      <c r="G57" t="n">
-        <v>2</v>
-      </c>
-      <c r="H57" t="inlineStr">
-        <is>
-          <t>T5.9,T5.10,T5.12</t>
         </is>
       </c>
       <c r="I57" s="4" t="n">
@@ -3388,7 +3388,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>T5.15</t>
+          <t>T5.16</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -3398,26 +3398,26 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Payments admin APIs + audit log</t>
+          <t>Feature flags + invite codes (sponsored spawn)</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>haiku-4.5</t>
+          <t>sonnet-5</t>
         </is>
       </c>
       <c r="E58" s="3" t="n">
-        <v>46371</v>
+        <v>46360</v>
       </c>
       <c r="F58" s="3" t="n">
-        <v>46371</v>
+        <v>46363</v>
       </c>
       <c r="G58" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>T5.13</t>
+          <t>T5.3</t>
         </is>
       </c>
       <c r="I58" s="4" t="n">
@@ -3435,7 +3435,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>T5.16</t>
+          <t>T5.17</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -3445,26 +3445,26 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Feature flags + invite codes (sponsored spawn)</t>
+          <t>treasury canister: owner-funded reserve, cycles …</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>sonnet-5</t>
+          <t>opus-5.5 (high)</t>
         </is>
       </c>
       <c r="E59" s="3" t="n">
+        <v>46364</v>
+      </c>
+      <c r="F59" s="3" t="n">
         <v>46366</v>
       </c>
-      <c r="F59" s="3" t="n">
-        <v>46367</v>
-      </c>
       <c r="G59" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>T5.3</t>
+          <t>T2.1,T1.4</t>
         </is>
       </c>
       <c r="I59" s="4" t="n">
@@ -3482,7 +3482,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>T5.17</t>
+          <t>T5.18</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -3492,26 +3492,26 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>treasury canister: owner-funded reserve, cycles …</t>
+          <t>treasury PocketIC tests (ICP ledger + CMC, no NN…</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>opus-5.5 (high)</t>
+          <t>sonnet-5</t>
         </is>
       </c>
       <c r="E60" s="3" t="n">
         <v>46367</v>
       </c>
       <c r="F60" s="3" t="n">
-        <v>46371</v>
+        <v>46367</v>
       </c>
       <c r="G60" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>T2.1,T1.4</t>
+          <t>T5.17</t>
         </is>
       </c>
       <c r="I60" s="4" t="n">
@@ -3529,7 +3529,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>T5.18</t>
+          <t>T5.7</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -3539,26 +3539,26 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>treasury PocketIC tests (ICP ledger + CMC, no NN…</t>
+          <t>Internal payments security review</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>sonnet-5</t>
+          <t>opus-5.5 (high)</t>
         </is>
       </c>
       <c r="E61" s="3" t="n">
-        <v>46372</v>
+        <v>46371</v>
       </c>
       <c r="F61" s="3" t="n">
         <v>46372</v>
       </c>
       <c r="G61" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>T5.17</t>
+          <t>T5.6,T5.13,T5.16</t>
         </is>
       </c>
       <c r="I61" s="4" t="n">
@@ -3576,40 +3576,40 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>T5.7</t>
+          <t>T6.1</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>P5</t>
+          <t>P6</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Internal payments security review</t>
+          <t>App scaffold: routing, bindgen, II auth, ic_env,…</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>opus-5.5 (high)</t>
+          <t>sonnet-5</t>
         </is>
       </c>
       <c r="E62" s="3" t="n">
+        <v>46367</v>
+      </c>
+      <c r="F62" s="3" t="n">
         <v>46371</v>
       </c>
-      <c r="F62" s="3" t="n">
-        <v>46372</v>
-      </c>
       <c r="G62" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>T5.6,T5.13,T5.16</t>
+          <t>T1.1</t>
         </is>
       </c>
       <c r="I62" s="4" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="J62">
         <f>IF(I62&gt;=1,"Done",IF(TODAY()&gt;F62,"Late",IF(I62&gt;0,"In progress","Not started")))</f>
@@ -3623,7 +3623,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>T6.1</t>
+          <t>T6.3</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -3633,7 +3633,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>App scaffold: routing, bindgen, II auth, ic_env,…</t>
+          <t>Landing, Discovery Museum feed, Discovery detail…</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -3645,18 +3645,18 @@
         <v>46372</v>
       </c>
       <c r="F63" s="3" t="n">
-        <v>46374</v>
+        <v>46378</v>
       </c>
       <c r="G63" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>T1.1</t>
+          <t>T6.1</t>
         </is>
       </c>
       <c r="I63" s="4" t="n">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="J63">
         <f>IF(I63&gt;=1,"Done",IF(TODAY()&gt;F63,"Late",IF(I63&gt;0,"In progress","Not started")))</f>
@@ -3670,7 +3670,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>T6.3</t>
+          <t>T6.4</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -3680,26 +3680,26 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Landing, Discovery Museum feed, Discovery detail…</t>
+          <t>AAA profile + Leaderboard</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>sonnet-5</t>
+          <t>haiku-4.5</t>
         </is>
       </c>
       <c r="E64" s="3" t="n">
-        <v>46377</v>
+        <v>46379</v>
       </c>
       <c r="F64" s="3" t="n">
         <v>46385</v>
       </c>
       <c r="G64" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>T6.1</t>
+          <t>T6.3</t>
         </is>
       </c>
       <c r="I64" s="4" t="n">
@@ -3717,7 +3717,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>T6.4</t>
+          <t>T6.5</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -3727,26 +3727,26 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>AAA profile + Leaderboard</t>
+          <t>Payment component (wallet + deposit)</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>haiku-4.5</t>
+          <t>sonnet-5</t>
         </is>
       </c>
       <c r="E65" s="3" t="n">
-        <v>46386</v>
+        <v>46372</v>
       </c>
       <c r="F65" s="3" t="n">
-        <v>46392</v>
+        <v>46377</v>
       </c>
       <c r="G65" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>T6.3</t>
+          <t>T6.1,SP-2,T5.4</t>
         </is>
       </c>
       <c r="I65" s="4" t="n">
@@ -3764,7 +3764,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>T6.5</t>
+          <t>T6.6</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -3774,26 +3774,26 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Payment component (wallet + deposit)</t>
+          <t>Spawn flow</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>sonnet-5</t>
+          <t>haiku-4.5</t>
         </is>
       </c>
       <c r="E66" s="3" t="n">
-        <v>46377</v>
+        <v>46378</v>
       </c>
       <c r="F66" s="3" t="n">
-        <v>46384</v>
+        <v>46379</v>
       </c>
       <c r="G66" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>T6.1,SP-2,T5.4</t>
+          <t>T6.5,T5.3</t>
         </is>
       </c>
       <c r="I66" s="4" t="n">
@@ -3811,7 +3811,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>T6.6</t>
+          <t>T6.7</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -3821,26 +3821,26 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Spawn flow</t>
+          <t>Owner dashboard</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>haiku-4.5</t>
+          <t>sonnet-5</t>
         </is>
       </c>
       <c r="E67" s="3" t="n">
+        <v>46378</v>
+      </c>
+      <c r="F67" s="3" t="n">
         <v>46385</v>
       </c>
-      <c r="F67" s="3" t="n">
-        <v>46386</v>
-      </c>
       <c r="G67" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>T6.5,T5.3</t>
+          <t>T6.1,T3.3,T4.6</t>
         </is>
       </c>
       <c r="I67" s="4" t="n">
@@ -3858,36 +3858,36 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
+          <t>T6.8</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>P6</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Connect your agent + Activity &amp; records</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>haiku-4.5</t>
+        </is>
+      </c>
+      <c r="E68" s="3" t="n">
+        <v>46386</v>
+      </c>
+      <c r="F68" s="3" t="n">
+        <v>46392</v>
+      </c>
+      <c r="G68" t="n">
+        <v>3</v>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
           <t>T6.7</t>
-        </is>
-      </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>P6</t>
-        </is>
-      </c>
-      <c r="C68" t="inlineStr">
-        <is>
-          <t>Owner dashboard</t>
-        </is>
-      </c>
-      <c r="D68" t="inlineStr">
-        <is>
-          <t>sonnet-5</t>
-        </is>
-      </c>
-      <c r="E68" s="3" t="n">
-        <v>46377</v>
-      </c>
-      <c r="F68" s="3" t="n">
-        <v>46384</v>
-      </c>
-      <c r="G68" t="n">
-        <v>4</v>
-      </c>
-      <c r="H68" t="inlineStr">
-        <is>
-          <t>T6.1,T3.3,T4.6</t>
         </is>
       </c>
       <c r="I68" s="4" t="n">
@@ -3905,7 +3905,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>T6.8</t>
+          <t>T6.9</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -3915,7 +3915,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Connect your agent + Activity &amp; records</t>
+          <t>Fuel &amp; billing + auto top-up</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -3924,17 +3924,17 @@
         </is>
       </c>
       <c r="E69" s="3" t="n">
-        <v>46385</v>
+        <v>46384</v>
       </c>
       <c r="F69" s="3" t="n">
-        <v>46391</v>
+        <v>46386</v>
       </c>
       <c r="G69" t="n">
         <v>3</v>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>T6.7</t>
+          <t>T6.5,T5.5</t>
         </is>
       </c>
       <c r="I69" s="4" t="n">
@@ -3952,7 +3952,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>T6.9</t>
+          <t>T6.11</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -3962,26 +3962,26 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Fuel &amp; billing + auto top-up</t>
+          <t>BTC &amp; ETH methods + feature-flag gating</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>haiku-4.5</t>
+          <t>sonnet-5</t>
         </is>
       </c>
       <c r="E70" s="3" t="n">
-        <v>46391</v>
+        <v>46386</v>
       </c>
       <c r="F70" s="3" t="n">
         <v>46393</v>
       </c>
       <c r="G70" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>T6.5,T5.5</t>
+          <t>T6.5,T5.9,T5.10</t>
         </is>
       </c>
       <c r="I70" s="4" t="n">
@@ -3999,7 +3999,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>T6.11</t>
+          <t>T6.12</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -4009,7 +4009,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>BTC &amp; ETH methods + feature-flag gating (card hi…</t>
+          <t>Admin console (8 screens)</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -4018,17 +4018,17 @@
         </is>
       </c>
       <c r="E71" s="3" t="n">
-        <v>46392</v>
+        <v>46391</v>
       </c>
       <c r="F71" s="3" t="n">
         <v>46395</v>
       </c>
       <c r="G71" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>T6.5,T5.9,T5.10</t>
+          <t>T6.1,T4.10,T5.15</t>
         </is>
       </c>
       <c r="I71" s="4" t="n">
@@ -4046,7 +4046,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>T6.12</t>
+          <t>T6.13</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -4056,26 +4056,26 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Admin console (8 screens)</t>
+          <t>Firebase analytics + consent + event taxonomy + …</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>sonnet-5</t>
+          <t>haiku-4.5</t>
         </is>
       </c>
       <c r="E72" s="3" t="n">
         <v>46393</v>
       </c>
       <c r="F72" s="3" t="n">
-        <v>46399</v>
+        <v>46394</v>
       </c>
       <c r="G72" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>T6.1,T4.10,T5.15</t>
+          <t>T6.1</t>
         </is>
       </c>
       <c r="I72" s="4" t="n">
@@ -4093,7 +4093,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>T6.13</t>
+          <t>T6.14</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -4103,7 +4103,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Firebase analytics + consent + event taxonomy + …</t>
+          <t>About/legal/practice pages, invite spawn UI, adm…</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -4112,17 +4112,17 @@
         </is>
       </c>
       <c r="E73" s="3" t="n">
-        <v>46394</v>
+        <v>46398</v>
       </c>
       <c r="F73" s="3" t="n">
-        <v>46395</v>
+        <v>46400</v>
       </c>
       <c r="G73" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>T6.1</t>
+          <t>T6.12,T5.16,T5.18</t>
         </is>
       </c>
       <c r="I73" s="4" t="n">
@@ -4140,7 +4140,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>T6.14</t>
+          <t>T6.10</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -4150,26 +4150,26 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>About/legal/practice pages, invite spawn UI, adm…</t>
+          <t>States, accessibility, Playwright smoke</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>haiku-4.5</t>
+          <t>sonnet-5</t>
         </is>
       </c>
       <c r="E74" s="3" t="n">
-        <v>46400</v>
+        <v>46401</v>
       </c>
       <c r="F74" s="3" t="n">
-        <v>46402</v>
+        <v>46405</v>
       </c>
       <c r="G74" t="n">
         <v>3</v>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>T6.12,T5.16,T5.18</t>
+          <t>T6.4,T6.6,T6.8,T6.9,T6.11,T6.12,T6.13,T6.14</t>
         </is>
       </c>
       <c r="I74" s="4" t="n">
@@ -4187,17 +4187,17 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>T6.10</t>
+          <t>T7.1</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>P6</t>
+          <t>P7</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>States, accessibility, Playwright smoke</t>
+          <t>Upgrade tests for all canisters</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -4206,17 +4206,17 @@
         </is>
       </c>
       <c r="E75" s="3" t="n">
-        <v>46405</v>
+        <v>46394</v>
       </c>
       <c r="F75" s="3" t="n">
-        <v>46407</v>
+        <v>46395</v>
       </c>
       <c r="G75" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>T6.4,T6.6,T6.8,T6.9,T6.11,T6.12,T6.13,T6.14</t>
+          <t>T4.8,T5.6</t>
         </is>
       </c>
       <c r="I75" s="4" t="n">
@@ -4234,7 +4234,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>T7.1</t>
+          <t>T7.2</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -4244,7 +4244,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Upgrade tests for all canisters</t>
+          <t>Load test: 200 AAAs × 100 tasks</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -4263,7 +4263,7 @@
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>T4.8,T5.6</t>
+          <t>T7.1</t>
         </is>
       </c>
       <c r="I76" s="4" t="n">
@@ -4281,7 +4281,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>T7.2</t>
+          <t>T7.3</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -4291,7 +4291,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Load test: 200 AAAs × 100 tasks</t>
+          <t>Cycle cost measurement &amp; fee retune</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -4310,7 +4310,7 @@
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>T7.1</t>
+          <t>T7.2</t>
         </is>
       </c>
       <c r="I77" s="4" t="n">
@@ -4328,7 +4328,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>T7.3</t>
+          <t>T7.4</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -4338,7 +4338,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Cycle cost measurement &amp; fee retune</t>
+          <t>Reproducible AAA build + manual upgrade docs</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -4347,17 +4347,17 @@
         </is>
       </c>
       <c r="E78" s="3" t="n">
-        <v>46402</v>
+        <v>46398</v>
       </c>
       <c r="F78" s="3" t="n">
-        <v>46405</v>
+        <v>46399</v>
       </c>
       <c r="G78" t="n">
         <v>2</v>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>T7.2</t>
+          <t>T3.6,T5.7</t>
         </is>
       </c>
       <c r="I78" s="4" t="n">
@@ -4375,7 +4375,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>T7.4</t>
+          <t>T7.7</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -4385,26 +4385,26 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Reproducible AAA build + manual upgrade docs</t>
+          <t>Prompt-injection test with reference agent</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>sonnet-5</t>
+          <t>opus-5.5 (high)</t>
         </is>
       </c>
       <c r="E79" s="3" t="n">
-        <v>46398</v>
+        <v>46400</v>
       </c>
       <c r="F79" s="3" t="n">
-        <v>46399</v>
+        <v>46400</v>
       </c>
       <c r="G79" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>T3.6,T5.7</t>
+          <t>T3.7,T4.7</t>
         </is>
       </c>
       <c r="I79" s="4" t="n">
@@ -4422,7 +4422,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>T7.7</t>
+          <t>T7.9</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -4432,26 +4432,26 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Prompt-injection test with reference agent</t>
+          <t>Traceability audit + coverage gates to thresholds</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>opus-5.5 (high)</t>
+          <t>haiku-4.5</t>
         </is>
       </c>
       <c r="E80" s="3" t="n">
-        <v>46400</v>
+        <v>46401</v>
       </c>
       <c r="F80" s="3" t="n">
-        <v>46400</v>
+        <v>46402</v>
       </c>
       <c r="G80" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>T3.7,T4.7</t>
+          <t>T7.1</t>
         </is>
       </c>
       <c r="I80" s="4" t="n">
@@ -4469,7 +4469,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>T7.9</t>
+          <t>T7.10</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -4479,7 +4479,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Traceability audit + coverage gates to thresholds</t>
+          <t>Practice set + open data release tooling</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -4488,17 +4488,17 @@
         </is>
       </c>
       <c r="E81" s="3" t="n">
-        <v>46401</v>
+        <v>46402</v>
       </c>
       <c r="F81" s="3" t="n">
-        <v>46402</v>
+        <v>46405</v>
       </c>
       <c r="G81" t="n">
         <v>2</v>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>T7.1</t>
+          <t>T1.7,T4.8</t>
         </is>
       </c>
       <c r="I81" s="4" t="n">
@@ -4516,7 +4516,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>T7.10</t>
+          <t>T7.5</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -4526,26 +4526,26 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Practice set + open data release tooling</t>
+          <t>External security review (payments + platform)</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>haiku-4.5</t>
+          <t>human</t>
         </is>
       </c>
       <c r="E82" s="3" t="n">
-        <v>46405</v>
+        <v>46373</v>
       </c>
       <c r="F82" s="3" t="n">
-        <v>46406</v>
+        <v>46379</v>
       </c>
       <c r="G82" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>T1.7,T4.8</t>
+          <t>T5.7,T4.8</t>
         </is>
       </c>
       <c r="I82" s="4" t="n">
@@ -4563,36 +4563,36 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
+          <t>T7.6</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Fix security findings</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>opus-5.5 (high)</t>
+        </is>
+      </c>
+      <c r="E83" s="3" t="n">
+        <v>46405</v>
+      </c>
+      <c r="F83" s="3" t="n">
+        <v>46407</v>
+      </c>
+      <c r="G83" t="n">
+        <v>3</v>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
           <t>T7.5</t>
-        </is>
-      </c>
-      <c r="B83" t="inlineStr">
-        <is>
-          <t>P7</t>
-        </is>
-      </c>
-      <c r="C83" t="inlineStr">
-        <is>
-          <t>External security review (payments + platform)</t>
-        </is>
-      </c>
-      <c r="D83" t="inlineStr">
-        <is>
-          <t>human</t>
-        </is>
-      </c>
-      <c r="E83" s="3" t="n">
-        <v>46373</v>
-      </c>
-      <c r="F83" s="3" t="n">
-        <v>46379</v>
-      </c>
-      <c r="G83" t="n">
-        <v>5</v>
-      </c>
-      <c r="H83" t="inlineStr">
-        <is>
-          <t>T5.7,T4.8</t>
         </is>
       </c>
       <c r="I83" s="4" t="n">
@@ -4610,7 +4610,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>T7.6</t>
+          <t>T7.11</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -4620,26 +4620,26 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Fix security findings</t>
+          <t>Continuous data refresh: 15-day scheduled job (n…</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>opus-5.5 (high)</t>
+          <t>sonnet-5</t>
         </is>
       </c>
       <c r="E84" s="3" t="n">
         <v>46406</v>
       </c>
       <c r="F84" s="3" t="n">
-        <v>46408</v>
+        <v>46407</v>
       </c>
       <c r="G84" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>T7.5</t>
+          <t>T1.7,T2.3</t>
         </is>
       </c>
       <c r="I84" s="4" t="n">
@@ -4657,36 +4657,36 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>T7.11</t>
+          <t>T8.14</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>P7</t>
+          <t>P8</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Continuous data refresh: 15-day scheduled job (n…</t>
+          <t>Create Cloudflare R2 bucket + API token + custom…</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>sonnet-5</t>
+          <t>human</t>
         </is>
       </c>
       <c r="E85" s="3" t="n">
-        <v>46407</v>
+        <v>46316</v>
       </c>
       <c r="F85" s="3" t="n">
-        <v>46408</v>
+        <v>46316</v>
       </c>
       <c r="G85" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>T1.7,T2.3</t>
+          <t>T1.7</t>
         </is>
       </c>
       <c r="I85" s="4" t="n">
@@ -4704,7 +4704,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>T8.14</t>
+          <t>T8.1</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -4714,26 +4714,26 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Create Cloudflare R2 bucket + API token + custom…</t>
+          <t>Staging deploy, deploy workflow, snapshots, cycl…</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>human</t>
+          <t>sonnet-5</t>
         </is>
       </c>
       <c r="E86" s="3" t="n">
-        <v>46316</v>
+        <v>46406</v>
       </c>
       <c r="F86" s="3" t="n">
-        <v>46316</v>
+        <v>46407</v>
       </c>
       <c r="G86" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>T1.7</t>
+          <t>T7.1</t>
         </is>
       </c>
       <c r="I86" s="4" t="n">
@@ -4751,7 +4751,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>T8.1</t>
+          <t>T8.2</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -4761,26 +4761,26 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Staging deploy, deploy workflow, snapshots, cycl…</t>
+          <t>Upload subjects/protocol/honeypots to staging</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>sonnet-5</t>
+          <t>haiku-4.5</t>
         </is>
       </c>
       <c r="E87" s="3" t="n">
         <v>46408</v>
       </c>
       <c r="F87" s="3" t="n">
-        <v>46409</v>
+        <v>46408</v>
       </c>
       <c r="G87" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>T7.1</t>
+          <t>T8.14,T8.1,T7.6</t>
         </is>
       </c>
       <c r="I87" s="4" t="n">
@@ -4798,7 +4798,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>T8.2</t>
+          <t>T8.5</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -4808,26 +4808,26 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Upload subjects/protocol/honeypots to staging</t>
+          <t>Fund prod treasury with ICP float (10–20 ICP) + …</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>haiku-4.5</t>
+          <t>human</t>
         </is>
       </c>
       <c r="E88" s="3" t="n">
-        <v>46412</v>
+        <v>46427</v>
       </c>
       <c r="F88" s="3" t="n">
-        <v>46412</v>
+        <v>46427</v>
       </c>
       <c r="G88" t="n">
         <v>1</v>
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>T8.14,T8.1,T7.6</t>
+          <t>T8.6</t>
         </is>
       </c>
       <c r="I88" s="4" t="n">
@@ -4845,7 +4845,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>T8.5</t>
+          <t>T8.3</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -4855,7 +4855,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Fund prod treasury with ICP float (10–20 ICP) + …</t>
+          <t>Closed beta (10-20 owners)</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -4864,17 +4864,17 @@
         </is>
       </c>
       <c r="E89" s="3" t="n">
-        <v>46429</v>
+        <v>46409</v>
       </c>
       <c r="F89" s="3" t="n">
-        <v>46429</v>
+        <v>46422</v>
       </c>
       <c r="G89" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>T8.6</t>
+          <t>T8.2,T6.10</t>
         </is>
       </c>
       <c r="I89" s="4" t="n">
@@ -4892,7 +4892,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>T8.3</t>
+          <t>T8.4</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -4902,19 +4902,19 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Closed beta (10-20 owners)</t>
+          <t>Beta fixes &amp; tuning</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>human</t>
+          <t>sonnet-5</t>
         </is>
       </c>
       <c r="E90" s="3" t="n">
-        <v>46413</v>
+        <v>46409</v>
       </c>
       <c r="F90" s="3" t="n">
-        <v>46426</v>
+        <v>46422</v>
       </c>
       <c r="G90" t="n">
         <v>10</v>
@@ -4939,7 +4939,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>T8.4</t>
+          <t>T8.6</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -4949,7 +4949,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Beta fixes &amp; tuning</t>
+          <t>Production deploy, II metadata, treasury watch l…</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -4958,17 +4958,17 @@
         </is>
       </c>
       <c r="E91" s="3" t="n">
-        <v>46413</v>
+        <v>46423</v>
       </c>
       <c r="F91" s="3" t="n">
         <v>46426</v>
       </c>
       <c r="G91" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>T8.2,T6.10</t>
+          <t>T8.3,T8.4,T8.13</t>
         </is>
       </c>
       <c r="I91" s="4" t="n">
@@ -4986,7 +4986,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>T8.6</t>
+          <t>T8.7</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -4996,26 +4996,26 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Production deploy, II metadata, treasury watch l…</t>
+          <t>Public launch</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>sonnet-5</t>
+          <t>human</t>
         </is>
       </c>
       <c r="E92" s="3" t="n">
-        <v>46427</v>
+        <v>46428</v>
       </c>
       <c r="F92" s="3" t="n">
         <v>46428</v>
       </c>
       <c r="G92" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>T8.3,T8.4,T8.13</t>
+          <t>T8.6,T8.5,T9.5</t>
         </is>
       </c>
       <c r="I92" s="4" t="n">
@@ -5033,36 +5033,36 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>T8.7</t>
+          <t>T9.1</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>P8</t>
+          <t>P9</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Public launch</t>
+          <t>Import mockups (Claude Design), reconcile, desig…</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>human</t>
+          <t>sonnet-5</t>
         </is>
       </c>
       <c r="E93" s="3" t="n">
-        <v>46430</v>
+        <v>46408</v>
       </c>
       <c r="F93" s="3" t="n">
-        <v>46430</v>
+        <v>46413</v>
       </c>
       <c r="G93" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>T8.6,T8.5,T9.5</t>
+          <t>T6.10</t>
         </is>
       </c>
       <c r="I93" s="4" t="n">
@@ -5080,7 +5080,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>T9.1</t>
+          <t>T9.2</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -5090,7 +5090,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Import mockups (Claude Design), reconcile, desig…</t>
+          <t>Style public pages: landing, museum, discovery, …</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -5099,17 +5099,17 @@
         </is>
       </c>
       <c r="E94" s="3" t="n">
-        <v>46409</v>
+        <v>46414</v>
       </c>
       <c r="F94" s="3" t="n">
-        <v>46414</v>
+        <v>46419</v>
       </c>
       <c r="G94" t="n">
         <v>4</v>
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>T6.10</t>
+          <t>T9.1</t>
         </is>
       </c>
       <c r="I94" s="4" t="n">
@@ -5127,7 +5127,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>T9.2</t>
+          <t>T9.3</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -5137,7 +5137,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Style public pages: landing, museum, discovery, …</t>
+          <t>Style owner flows: spawn, dashboard, connect age…</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -5146,10 +5146,10 @@
         </is>
       </c>
       <c r="E95" s="3" t="n">
-        <v>46415</v>
+        <v>46414</v>
       </c>
       <c r="F95" s="3" t="n">
-        <v>46420</v>
+        <v>46419</v>
       </c>
       <c r="G95" t="n">
         <v>4</v>
@@ -5174,7 +5174,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>T9.3</t>
+          <t>T9.4</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -5184,22 +5184,22 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Style owner flows: spawn, dashboard, connect age…</t>
+          <t>Style admin console + about/legal/practice pages</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>sonnet-5</t>
+          <t>haiku-4.5</t>
         </is>
       </c>
       <c r="E96" s="3" t="n">
-        <v>46415</v>
+        <v>46420</v>
       </c>
       <c r="F96" s="3" t="n">
-        <v>46420</v>
+        <v>46421</v>
       </c>
       <c r="G96" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H96" t="inlineStr">
         <is>
@@ -5221,7 +5221,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>T9.4</t>
+          <t>T9.5</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -5231,7 +5231,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Style admin console + about/legal/practice pages</t>
+          <t>Responsive/mobile pass, visual-regression baseli…</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -5240,17 +5240,17 @@
         </is>
       </c>
       <c r="E97" s="3" t="n">
-        <v>46421</v>
+        <v>46422</v>
       </c>
       <c r="F97" s="3" t="n">
-        <v>46422</v>
+        <v>46423</v>
       </c>
       <c r="G97" t="n">
         <v>2</v>
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>T9.1</t>
+          <t>T9.2,T9.3,T9.4</t>
         </is>
       </c>
       <c r="I97" s="4" t="n">
@@ -5268,36 +5268,36 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>T9.5</t>
+          <t>T8.13</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>P9</t>
+          <t>P8</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Responsive/mobile pass, visual-regression baseli…</t>
+          <t>Custom domain + II alternative origins</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>haiku-4.5</t>
+          <t>human</t>
         </is>
       </c>
       <c r="E98" s="3" t="n">
-        <v>46423</v>
+        <v>46408</v>
       </c>
       <c r="F98" s="3" t="n">
-        <v>46426</v>
+        <v>46408</v>
       </c>
       <c r="G98" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>T9.2,T9.3,T9.4</t>
+          <t>T8.1</t>
         </is>
       </c>
       <c r="I98" s="4" t="n">
@@ -5315,7 +5315,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>T8.13</t>
+          <t>T8.12</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -5325,7 +5325,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Custom domain + II alternative origins</t>
+          <t>Firebase projects (staging/prod) + GA4 funnels &amp;…</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -5334,17 +5334,17 @@
         </is>
       </c>
       <c r="E99" s="3" t="n">
-        <v>46412</v>
+        <v>46296</v>
       </c>
       <c r="F99" s="3" t="n">
-        <v>46412</v>
+        <v>46296</v>
       </c>
       <c r="G99" t="n">
         <v>1</v>
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>T8.1</t>
+          <t>T0.4</t>
         </is>
       </c>
       <c r="I99" s="4" t="n">
@@ -5362,7 +5362,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>T8.12</t>
+          <t>T8.15</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -5372,7 +5372,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Firebase projects (staging/prod) + GA4 funnels &amp;…</t>
+          <t>Owner review: discovery + peer-review agent proc…</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -5409,7 +5409,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>T8.15</t>
+          <t>T8.8</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -5419,7 +5419,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Owner review: discovery + peer-review agent proc…</t>
+          <t>Compliance check for crypto fuel packs (recommen…</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -5431,10 +5431,10 @@
         <v>46296</v>
       </c>
       <c r="F101" s="3" t="n">
-        <v>46296</v>
+        <v>46302</v>
       </c>
       <c r="G101" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H101" t="inlineStr">
         <is>
@@ -5456,7 +5456,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>T8.8</t>
+          <t>T8.9</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -5466,7 +5466,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Compliance check for card &amp; crypto fuel packs (r…</t>
+          <t>Enable BTC/ETH on production</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -5475,17 +5475,17 @@
         </is>
       </c>
       <c r="E102" s="3" t="n">
-        <v>46296</v>
+        <v>46427</v>
       </c>
       <c r="F102" s="3" t="n">
-        <v>46302</v>
+        <v>46427</v>
       </c>
       <c r="G102" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>T0.4</t>
+          <t>T8.6,T8.8</t>
         </is>
       </c>
       <c r="I102" s="4" t="n">
@@ -5500,55 +5500,8 @@
         <v/>
       </c>
     </row>
-    <row r="103">
-      <c r="A103" t="inlineStr">
-        <is>
-          <t>T8.9</t>
-        </is>
-      </c>
-      <c r="B103" t="inlineStr">
-        <is>
-          <t>P8</t>
-        </is>
-      </c>
-      <c r="C103" t="inlineStr">
-        <is>
-          <t>Enable BTC/ETH on production (card stays off)</t>
-        </is>
-      </c>
-      <c r="D103" t="inlineStr">
-        <is>
-          <t>human</t>
-        </is>
-      </c>
-      <c r="E103" s="3" t="n">
-        <v>46429</v>
-      </c>
-      <c r="F103" s="3" t="n">
-        <v>46429</v>
-      </c>
-      <c r="G103" t="n">
-        <v>1</v>
-      </c>
-      <c r="H103" t="inlineStr">
-        <is>
-          <t>T8.6,T8.8</t>
-        </is>
-      </c>
-      <c r="I103" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J103">
-        <f>IF(I103&gt;=1,"Done",IF(TODAY()&gt;F103,"Late",IF(I103&gt;0,"In progress","Not started")))</f>
-        <v/>
-      </c>
-      <c r="K103">
-        <f>G103*I103</f>
-        <v/>
-      </c>
-    </row>
   </sheetData>
-  <conditionalFormatting sqref="L2:AF103">
+  <conditionalFormatting sqref="L2:AF102">
     <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="1">
       <formula>AND(L$1+6&gt;=$E2,L$1&lt;=$F2,L$1&lt;=$E2+($F2-$E2)*$I2)</formula>
     </cfRule>
@@ -5586,7 +5539,7 @@
       <formula>AND(TODAY()&gt;=L$1,TODAY()&lt;L$1+7)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J2:J103">
+  <conditionalFormatting sqref="J2:J102">
     <cfRule type="expression" priority="13" dxfId="12">
       <formula>LEFT(J2,4)="Late"</formula>
     </cfRule>
@@ -5953,10 +5906,10 @@
         <v/>
       </c>
       <c r="H8" s="3" t="n">
-        <v>46372</v>
+        <v>46367</v>
       </c>
       <c r="I8" s="3" t="n">
-        <v>46407</v>
+        <v>46405</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
@@ -5998,7 +5951,7 @@
         <v>46373</v>
       </c>
       <c r="I9" s="3" t="n">
-        <v>46408</v>
+        <v>46407</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
@@ -6040,7 +5993,7 @@
         <v>46296</v>
       </c>
       <c r="I10" s="3" t="n">
-        <v>46430</v>
+        <v>46428</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
@@ -6079,10 +6032,10 @@
         <v/>
       </c>
       <c r="H11" s="3" t="n">
-        <v>46409</v>
+        <v>46408</v>
       </c>
       <c r="I11" s="3" t="n">
-        <v>46426</v>
+        <v>46423</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
@@ -6117,14 +6070,14 @@
         <v/>
       </c>
       <c r="G12" s="17">
-        <f>IF(C12&gt;0,SUM(Gantt!K2:K103)/C12,0)</f>
+        <f>IF(C12&gt;0,SUM(Gantt!K2:K102)/C12,0)</f>
         <v/>
       </c>
       <c r="H12" s="18" t="n">
         <v>46286</v>
       </c>
       <c r="I12" s="18" t="n">
-        <v>46430</v>
+        <v>46428</v>
       </c>
     </row>
     <row r="14">

</xml_diff>

<commit_message>
plan: add T8.16 (20k dataset before beta), fix stale card/audit wording, R2 dep for refresh; handoff prompt
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/space-compute-gantt-v3.xlsx
+++ b/docs/space-compute-gantt-v3.xlsx
@@ -600,7 +600,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF102"/>
+  <dimension ref="A1:AF103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2740,7 +2740,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Admin read APIs + audit log (platform)</t>
+          <t>Admin read APIs (platform; audit log exists sinc…</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -3351,7 +3351,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Payments admin APIs + audit log</t>
+          <t>Payments admin APIs (audit log exists since T5.1)</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -4639,7 +4639,7 @@
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>T1.7,T2.3</t>
+          <t>T1.7,T2.3,T8.14</t>
         </is>
       </c>
       <c r="I84" s="4" t="n">
@@ -4704,7 +4704,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>T8.1</t>
+          <t>T8.16</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -4714,26 +4714,26 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Staging deploy, deploy workflow, snapshots, cycl…</t>
+          <t>Scale dataset to 20,000 subjects (R-62) and publ…</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>sonnet-5</t>
+          <t>haiku-4.5</t>
         </is>
       </c>
       <c r="E86" s="3" t="n">
         <v>46406</v>
       </c>
       <c r="F86" s="3" t="n">
-        <v>46407</v>
+        <v>46406</v>
       </c>
       <c r="G86" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>T7.1</t>
+          <t>T8.14</t>
         </is>
       </c>
       <c r="I86" s="4" t="n">
@@ -4751,7 +4751,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>T8.2</t>
+          <t>T8.1</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -4761,26 +4761,26 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Upload subjects/protocol/honeypots to staging</t>
+          <t>Staging deploy, deploy workflow, snapshots, cycl…</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>haiku-4.5</t>
+          <t>sonnet-5</t>
         </is>
       </c>
       <c r="E87" s="3" t="n">
-        <v>46408</v>
+        <v>46407</v>
       </c>
       <c r="F87" s="3" t="n">
         <v>46408</v>
       </c>
       <c r="G87" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>T8.14,T8.1,T7.6</t>
+          <t>T7.1</t>
         </is>
       </c>
       <c r="I87" s="4" t="n">
@@ -4798,7 +4798,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>T8.5</t>
+          <t>T8.2</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -4808,26 +4808,26 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Fund prod treasury with ICP float (10–20 ICP) + …</t>
+          <t>Upload subjects/protocol/honeypots to staging</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>human</t>
+          <t>haiku-4.5</t>
         </is>
       </c>
       <c r="E88" s="3" t="n">
-        <v>46427</v>
+        <v>46409</v>
       </c>
       <c r="F88" s="3" t="n">
-        <v>46427</v>
+        <v>46409</v>
       </c>
       <c r="G88" t="n">
         <v>1</v>
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>T8.6</t>
+          <t>T8.16,T8.1,T7.6</t>
         </is>
       </c>
       <c r="I88" s="4" t="n">
@@ -4845,7 +4845,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>T8.3</t>
+          <t>T8.5</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -4855,7 +4855,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Closed beta (10-20 owners)</t>
+          <t>Fund prod treasury with ICP float (10–20 ICP) + …</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -4864,17 +4864,17 @@
         </is>
       </c>
       <c r="E89" s="3" t="n">
-        <v>46409</v>
+        <v>46428</v>
       </c>
       <c r="F89" s="3" t="n">
-        <v>46422</v>
+        <v>46428</v>
       </c>
       <c r="G89" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>T8.2,T6.10</t>
+          <t>T8.6</t>
         </is>
       </c>
       <c r="I89" s="4" t="n">
@@ -4892,7 +4892,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>T8.4</t>
+          <t>T8.3</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -4902,19 +4902,19 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Beta fixes &amp; tuning</t>
+          <t>Closed beta (10-20 owners)</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>sonnet-5</t>
+          <t>human</t>
         </is>
       </c>
       <c r="E90" s="3" t="n">
-        <v>46409</v>
+        <v>46412</v>
       </c>
       <c r="F90" s="3" t="n">
-        <v>46422</v>
+        <v>46423</v>
       </c>
       <c r="G90" t="n">
         <v>10</v>
@@ -4939,7 +4939,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>T8.6</t>
+          <t>T8.4</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -4949,7 +4949,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Production deploy, II metadata, treasury watch l…</t>
+          <t>Beta fixes &amp; tuning</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -4958,17 +4958,17 @@
         </is>
       </c>
       <c r="E91" s="3" t="n">
+        <v>46412</v>
+      </c>
+      <c r="F91" s="3" t="n">
         <v>46423</v>
       </c>
-      <c r="F91" s="3" t="n">
-        <v>46426</v>
-      </c>
       <c r="G91" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>T8.3,T8.4,T8.13</t>
+          <t>T8.2,T6.10</t>
         </is>
       </c>
       <c r="I91" s="4" t="n">
@@ -4986,7 +4986,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>T8.7</t>
+          <t>T8.6</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -4996,26 +4996,26 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Public launch</t>
+          <t>Production deploy, II metadata, treasury watch l…</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>human</t>
+          <t>sonnet-5</t>
         </is>
       </c>
       <c r="E92" s="3" t="n">
-        <v>46428</v>
+        <v>46426</v>
       </c>
       <c r="F92" s="3" t="n">
-        <v>46428</v>
+        <v>46427</v>
       </c>
       <c r="G92" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>T8.6,T8.5,T9.5</t>
+          <t>T8.3,T8.4,T8.13</t>
         </is>
       </c>
       <c r="I92" s="4" t="n">
@@ -5033,36 +5033,36 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>T9.1</t>
+          <t>T8.7</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>P9</t>
+          <t>P8</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Import mockups (Claude Design), reconcile, desig…</t>
+          <t>Public launch</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>sonnet-5</t>
+          <t>human</t>
         </is>
       </c>
       <c r="E93" s="3" t="n">
-        <v>46408</v>
+        <v>46429</v>
       </c>
       <c r="F93" s="3" t="n">
-        <v>46413</v>
+        <v>46429</v>
       </c>
       <c r="G93" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>T6.10</t>
+          <t>T8.6,T8.5,T9.5</t>
         </is>
       </c>
       <c r="I93" s="4" t="n">
@@ -5080,7 +5080,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>T9.2</t>
+          <t>T9.1</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -5090,7 +5090,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Style public pages: landing, museum, discovery, …</t>
+          <t>Import mockups (Claude Design), reconcile, desig…</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -5099,17 +5099,17 @@
         </is>
       </c>
       <c r="E94" s="3" t="n">
-        <v>46414</v>
+        <v>46408</v>
       </c>
       <c r="F94" s="3" t="n">
-        <v>46419</v>
+        <v>46413</v>
       </c>
       <c r="G94" t="n">
         <v>4</v>
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>T9.1</t>
+          <t>T6.10</t>
         </is>
       </c>
       <c r="I94" s="4" t="n">
@@ -5127,7 +5127,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>T9.3</t>
+          <t>T9.2</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -5137,7 +5137,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Style owner flows: spawn, dashboard, connect age…</t>
+          <t>Style public pages: landing, museum, discovery, …</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -5174,7 +5174,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>T9.4</t>
+          <t>T9.3</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -5184,22 +5184,22 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Style admin console + about/legal/practice pages</t>
+          <t>Style owner flows: spawn, dashboard, connect age…</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>haiku-4.5</t>
+          <t>sonnet-5</t>
         </is>
       </c>
       <c r="E96" s="3" t="n">
-        <v>46420</v>
+        <v>46414</v>
       </c>
       <c r="F96" s="3" t="n">
-        <v>46421</v>
+        <v>46419</v>
       </c>
       <c r="G96" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H96" t="inlineStr">
         <is>
@@ -5221,7 +5221,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>T9.5</t>
+          <t>T9.4</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -5231,7 +5231,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Responsive/mobile pass, visual-regression baseli…</t>
+          <t>Style admin console + about/legal/practice pages</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -5240,17 +5240,17 @@
         </is>
       </c>
       <c r="E97" s="3" t="n">
-        <v>46422</v>
+        <v>46420</v>
       </c>
       <c r="F97" s="3" t="n">
-        <v>46423</v>
+        <v>46421</v>
       </c>
       <c r="G97" t="n">
         <v>2</v>
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>T9.2,T9.3,T9.4</t>
+          <t>T9.1</t>
         </is>
       </c>
       <c r="I97" s="4" t="n">
@@ -5268,36 +5268,36 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>T8.13</t>
+          <t>T9.5</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>P8</t>
+          <t>P9</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Custom domain + II alternative origins</t>
+          <t>Responsive/mobile pass, visual-regression baseli…</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>human</t>
+          <t>haiku-4.5</t>
         </is>
       </c>
       <c r="E98" s="3" t="n">
-        <v>46408</v>
+        <v>46422</v>
       </c>
       <c r="F98" s="3" t="n">
-        <v>46408</v>
+        <v>46423</v>
       </c>
       <c r="G98" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>T8.1</t>
+          <t>T9.2,T9.3,T9.4</t>
         </is>
       </c>
       <c r="I98" s="4" t="n">
@@ -5315,7 +5315,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>T8.12</t>
+          <t>T8.13</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -5325,7 +5325,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Firebase projects (staging/prod) + GA4 funnels &amp;…</t>
+          <t>Custom domain + II alternative origins</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -5334,17 +5334,17 @@
         </is>
       </c>
       <c r="E99" s="3" t="n">
-        <v>46296</v>
+        <v>46409</v>
       </c>
       <c r="F99" s="3" t="n">
-        <v>46296</v>
+        <v>46409</v>
       </c>
       <c r="G99" t="n">
         <v>1</v>
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>T0.4</t>
+          <t>T8.1</t>
         </is>
       </c>
       <c r="I99" s="4" t="n">
@@ -5362,7 +5362,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>T8.15</t>
+          <t>T8.12</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -5372,7 +5372,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Owner review: discovery + peer-review agent proc…</t>
+          <t>Firebase projects (staging/prod) + GA4 funnels &amp;…</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -5409,7 +5409,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>T8.8</t>
+          <t>T8.15</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -5419,7 +5419,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Compliance check for crypto fuel packs (recommen…</t>
+          <t>Owner review: discovery + peer-review agent proc…</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -5431,10 +5431,10 @@
         <v>46296</v>
       </c>
       <c r="F101" s="3" t="n">
-        <v>46302</v>
+        <v>46296</v>
       </c>
       <c r="G101" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H101" t="inlineStr">
         <is>
@@ -5456,7 +5456,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>T8.9</t>
+          <t>T8.8</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -5466,7 +5466,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Enable BTC/ETH on production</t>
+          <t>Compliance check for crypto fuel packs (recommen…</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -5475,17 +5475,17 @@
         </is>
       </c>
       <c r="E102" s="3" t="n">
-        <v>46427</v>
+        <v>46296</v>
       </c>
       <c r="F102" s="3" t="n">
-        <v>46427</v>
+        <v>46302</v>
       </c>
       <c r="G102" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>T8.6,T8.8</t>
+          <t>T0.4</t>
         </is>
       </c>
       <c r="I102" s="4" t="n">
@@ -5500,8 +5500,55 @@
         <v/>
       </c>
     </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>T8.9</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>P8</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Enable BTC/ETH on production</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>human</t>
+        </is>
+      </c>
+      <c r="E103" s="3" t="n">
+        <v>46428</v>
+      </c>
+      <c r="F103" s="3" t="n">
+        <v>46428</v>
+      </c>
+      <c r="G103" t="n">
+        <v>1</v>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>T8.6,T8.8</t>
+        </is>
+      </c>
+      <c r="I103" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J103">
+        <f>IF(I103&gt;=1,"Done",IF(TODAY()&gt;F103,"Late",IF(I103&gt;0,"In progress","Not started")))</f>
+        <v/>
+      </c>
+      <c r="K103">
+        <f>G103*I103</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="L2:AF102">
+  <conditionalFormatting sqref="L2:AF103">
     <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="1">
       <formula>AND(L$1+6&gt;=$E2,L$1&lt;=$F2,L$1&lt;=$E2+($F2-$E2)*$I2)</formula>
     </cfRule>
@@ -5539,7 +5586,7 @@
       <formula>AND(TODAY()&gt;=L$1,TODAY()&lt;L$1+7)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J2:J102">
+  <conditionalFormatting sqref="J2:J103">
     <cfRule type="expression" priority="13" dxfId="12">
       <formula>LEFT(J2,4)="Late"</formula>
     </cfRule>
@@ -5993,7 +6040,7 @@
         <v>46296</v>
       </c>
       <c r="I10" s="3" t="n">
-        <v>46428</v>
+        <v>46429</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
@@ -6070,14 +6117,14 @@
         <v/>
       </c>
       <c r="G12" s="17">
-        <f>IF(C12&gt;0,SUM(Gantt!K2:K102)/C12,0)</f>
+        <f>IF(C12&gt;0,SUM(Gantt!K2:K103)/C12,0)</f>
         <v/>
       </c>
       <c r="H12" s="18" t="n">
         <v>46286</v>
       </c>
       <c r="I12" s="18" t="n">
-        <v>46428</v>
+        <v>46429</v>
       </c>
     </row>
     <row r="14">

</xml_diff>

<commit_message>
T5.17: treasury keeper — owner-funded reserve, 6 h cycles top-ups via CMC, health/status/history, two-admin proposals
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/space-compute-gantt-v3.xlsx
+++ b/docs/space-compute-gantt-v3.xlsx
@@ -600,7 +600,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF103"/>
+  <dimension ref="A1:AF104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1931,40 +1931,40 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>T3.1</t>
+          <t>T2.9</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>AAA skeleton: roles, operators, config, inspect_…</t>
+          <t>Lead-review fixes for P2 (gold leak, verify auth…</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>sonnet-5</t>
+          <t>opus-5.5 (high)</t>
         </is>
       </c>
       <c r="E27" s="3" t="n">
-        <v>46318</v>
+        <v>46322</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>46321</v>
+        <v>46323</v>
       </c>
       <c r="G27" t="n">
         <v>2</v>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>T1.2</t>
+          <t>T2.7,T2.8</t>
         </is>
       </c>
       <c r="I27" s="4" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="J27">
         <f>IF(I27&gt;=1,"Done",IF(TODAY()&gt;F27,"Late",IF(I27&gt;0,"In progress","Not started")))</f>
@@ -1978,7 +1978,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>T3.2</t>
+          <t>T3.1</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1988,26 +1988,26 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>AAA forwarding w/ fees, retries, idempotency, lo…</t>
+          <t>AAA skeleton: roles, operators, config, inspect_…</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>opus-5.5 (high)</t>
+          <t>sonnet-5</t>
         </is>
       </c>
       <c r="E28" s="3" t="n">
-        <v>46322</v>
+        <v>46318</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>46324</v>
+        <v>46321</v>
       </c>
       <c r="G28" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>T3.1,T2.4</t>
+          <t>T1.2</t>
         </is>
       </c>
       <c r="I28" s="4" t="n">
@@ -2025,7 +2025,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>T3.3</t>
+          <t>T3.2</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -2035,26 +2035,26 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>AAA repository records + queries + credits copy</t>
+          <t>AAA forwarding w/ fees, retries, idempotency, lo…</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>haiku-4.5</t>
+          <t>opus-5.5 (high)</t>
         </is>
       </c>
       <c r="E29" s="3" t="n">
-        <v>46325</v>
+        <v>46322</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>46328</v>
+        <v>46324</v>
       </c>
       <c r="G29" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>T3.2</t>
+          <t>T3.1,T2.4</t>
         </is>
       </c>
       <c r="I29" s="4" t="n">
@@ -2072,7 +2072,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>T3.4</t>
+          <t>T3.3</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -2082,30 +2082,30 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>AAA timers: burn EMA, heartbeat, credits sync, a…</t>
+          <t>AAA repository records + queries + credits copy</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>sonnet-5</t>
+          <t>haiku-4.5</t>
         </is>
       </c>
       <c r="E30" s="3" t="n">
-        <v>46329</v>
+        <v>46325</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>46330</v>
+        <v>46328</v>
       </c>
       <c r="G30" t="n">
         <v>2</v>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>T3.3</t>
+          <t>T3.2</t>
         </is>
       </c>
       <c r="I30" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J30">
         <f>IF(I30&gt;=1,"Done",IF(TODAY()&gt;F30,"Late",IF(I30&gt;0,"In progress","Not started")))</f>
@@ -2119,7 +2119,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>T3.5</t>
+          <t>T3.4</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2129,30 +2129,30 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>get_api_doc + wasm size budget ≤1.5 MiB gz</t>
+          <t>AAA timers: burn EMA, heartbeat, credits sync, a…</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>haiku-4.5</t>
+          <t>sonnet-5</t>
         </is>
       </c>
       <c r="E31" s="3" t="n">
-        <v>46325</v>
+        <v>46329</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>46325</v>
+        <v>46330</v>
       </c>
       <c r="G31" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>T3.2</t>
+          <t>T3.3</t>
         </is>
       </c>
       <c r="I31" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J31">
         <f>IF(I31&gt;=1,"Done",IF(TODAY()&gt;F31,"Late",IF(I31&gt;0,"In progress","Not started")))</f>
@@ -2166,7 +2166,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>T3.6</t>
+          <t>T3.5</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2176,30 +2176,30 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>AAA PocketIC tests (03 §8)</t>
+          <t>get_api_doc + wasm size budget ≤1.5 MiB gz</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>sonnet-5</t>
+          <t>haiku-4.5</t>
         </is>
       </c>
       <c r="E32" s="3" t="n">
-        <v>46331</v>
+        <v>46325</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>46332</v>
+        <v>46325</v>
       </c>
       <c r="G32" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>T3.4</t>
+          <t>T3.2</t>
         </is>
       </c>
       <c r="I32" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J32">
         <f>IF(I32&gt;=1,"Done",IF(TODAY()&gt;F32,"Late",IF(I32&gt;0,"In progress","Not started")))</f>
@@ -2213,7 +2213,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>T3.8</t>
+          <t>T3.6</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2223,26 +2223,26 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Local seed script + dev loop (tools/seed-local)</t>
+          <t>AAA PocketIC tests (03 §8)</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>haiku-4.5</t>
+          <t>sonnet-5</t>
         </is>
       </c>
       <c r="E33" s="3" t="n">
-        <v>46325</v>
+        <v>46331</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>46325</v>
+        <v>46332</v>
       </c>
       <c r="G33" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>T2.2,T3.2,T1.7,T1.8</t>
+          <t>T3.4</t>
         </is>
       </c>
       <c r="I33" s="4" t="n">
@@ -2260,7 +2260,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>T3.7</t>
+          <t>T3.8</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2270,26 +2270,26 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Operator skill + JWST protocol primer + analyze.…</t>
+          <t>Local seed script + dev loop (tools/seed-local)</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>opus-5.5 (high)</t>
+          <t>haiku-4.5</t>
         </is>
       </c>
       <c r="E34" s="3" t="n">
-        <v>46328</v>
+        <v>46325</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>46331</v>
+        <v>46325</v>
       </c>
       <c r="G34" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>T3.5,T1.7</t>
+          <t>T2.2,T3.2,T1.7,T1.8</t>
         </is>
       </c>
       <c r="I34" s="4" t="n">
@@ -2307,7 +2307,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>T3.9</t>
+          <t>T3.7</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2317,26 +2317,26 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Headless runner recipe + practice.py self-eval</t>
+          <t>Operator skill + JWST protocol primer + analyze.…</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>haiku-4.5</t>
+          <t>opus-5.5 (high)</t>
         </is>
       </c>
       <c r="E35" s="3" t="n">
-        <v>46332</v>
+        <v>46328</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>46332</v>
+        <v>46331</v>
       </c>
       <c r="G35" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>T3.7</t>
+          <t>T3.5,T1.7</t>
         </is>
       </c>
       <c r="I35" s="4" t="n">
@@ -2354,36 +2354,36 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>T4.3</t>
+          <t>T3.9</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>P4</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Progression: XP, reputation, tiers, badges, lead…</t>
+          <t>Headless runner recipe + practice.py self-eval</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>sonnet-5</t>
+          <t>haiku-4.5</t>
         </is>
       </c>
       <c r="E36" s="3" t="n">
-        <v>46328</v>
+        <v>46332</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>46331</v>
+        <v>46332</v>
       </c>
       <c r="G36" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>T2.5,T2.7</t>
+          <t>T3.7</t>
         </is>
       </c>
       <c r="I36" s="4" t="n">
@@ -2401,7 +2401,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>T4.1</t>
+          <t>T4.3</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -2411,7 +2411,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Discoveries: flagging, rate limit, public IDs</t>
+          <t>Progression: XP, reputation, tiers, badges, lead…</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -2420,17 +2420,17 @@
         </is>
       </c>
       <c r="E37" s="3" t="n">
-        <v>46332</v>
+        <v>46328</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>46335</v>
+        <v>46331</v>
       </c>
       <c r="G37" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>T2.4</t>
+          <t>T2.5,T2.7</t>
         </is>
       </c>
       <c r="I37" s="4" t="n">
@@ -2448,7 +2448,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>T4.9</t>
+          <t>T4.1</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -2458,26 +2458,26 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>First-claim rule: sky claim index + corroboratio…</t>
+          <t>Discoveries: flagging, rate limit, public IDs</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>opus-5.5 (high)</t>
+          <t>sonnet-5</t>
         </is>
       </c>
       <c r="E38" s="3" t="n">
-        <v>46336</v>
+        <v>46332</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>46337</v>
+        <v>46335</v>
       </c>
       <c r="G38" t="n">
         <v>2</v>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>T4.1</t>
+          <t>T2.4</t>
         </is>
       </c>
       <c r="I38" s="4" t="n">
@@ -2495,7 +2495,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>T4.2</t>
+          <t>T4.9</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -2505,7 +2505,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Review assignment: eligibility, blind, leases, h…</t>
+          <t>First-claim rule: sky claim index + corroboratio…</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -2517,14 +2517,14 @@
         <v>46336</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>46338</v>
+        <v>46337</v>
       </c>
       <c r="G39" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>T4.1,T4.3</t>
+          <t>T4.1</t>
         </is>
       </c>
       <c r="I39" s="4" t="n">
@@ -2542,7 +2542,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>T4.4</t>
+          <t>T4.2</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2552,7 +2552,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>evaluate(), atomic resolution, starvation rule</t>
+          <t>Review assignment: eligibility, blind, leases, h…</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -2561,17 +2561,17 @@
         </is>
       </c>
       <c r="E40" s="3" t="n">
-        <v>46339</v>
+        <v>46336</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>46343</v>
+        <v>46338</v>
       </c>
       <c r="G40" t="n">
         <v>3</v>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>T4.2</t>
+          <t>T4.1,T4.3</t>
         </is>
       </c>
       <c r="I40" s="4" t="n">
@@ -2589,7 +2589,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>T4.5</t>
+          <t>T4.4</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2599,7 +2599,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Citations + certification tree + get_citation</t>
+          <t>evaluate(), atomic resolution, starvation rule</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -2608,17 +2608,17 @@
         </is>
       </c>
       <c r="E41" s="3" t="n">
-        <v>46344</v>
+        <v>46339</v>
       </c>
       <c r="F41" s="3" t="n">
-        <v>46346</v>
+        <v>46343</v>
       </c>
       <c r="G41" t="n">
         <v>3</v>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>T4.4</t>
+          <t>T4.2</t>
         </is>
       </c>
       <c r="I41" s="4" t="n">
@@ -2636,7 +2636,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>T4.6</t>
+          <t>T4.5</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2646,26 +2646,26 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Visibility rules &amp; public discovery queries</t>
+          <t>Citations + certification tree + get_citation</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>sonnet-5</t>
+          <t>opus-5.5 (high)</t>
         </is>
       </c>
       <c r="E42" s="3" t="n">
-        <v>46349</v>
+        <v>46344</v>
       </c>
       <c r="F42" s="3" t="n">
-        <v>46350</v>
+        <v>46346</v>
       </c>
       <c r="G42" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>T4.5</t>
+          <t>T4.4</t>
         </is>
       </c>
       <c r="I42" s="4" t="n">
@@ -2683,7 +2683,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>T4.7</t>
+          <t>T4.6</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2693,26 +2693,26 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Honeypot seeding (120 specs)</t>
+          <t>Visibility rules &amp; public discovery queries</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>haiku-4.5</t>
+          <t>sonnet-5</t>
         </is>
       </c>
       <c r="E43" s="3" t="n">
-        <v>46339</v>
+        <v>46349</v>
       </c>
       <c r="F43" s="3" t="n">
-        <v>46339</v>
+        <v>46350</v>
       </c>
       <c r="G43" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>T4.2,T1.7</t>
+          <t>T4.5</t>
         </is>
       </c>
       <c r="I43" s="4" t="n">
@@ -2730,7 +2730,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>T4.10</t>
+          <t>T4.7</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2740,7 +2740,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Admin read APIs (platform; audit log exists sinc…</t>
+          <t>Honeypot seeding (120 specs)</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -2749,17 +2749,17 @@
         </is>
       </c>
       <c r="E44" s="3" t="n">
-        <v>46351</v>
+        <v>46339</v>
       </c>
       <c r="F44" s="3" t="n">
-        <v>46356</v>
+        <v>46339</v>
       </c>
       <c r="G44" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>T4.6</t>
+          <t>T4.2,T1.7</t>
         </is>
       </c>
       <c r="I44" s="4" t="n">
@@ -2777,7 +2777,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>T4.11</t>
+          <t>T4.10</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Name blocklist, admin_rename_aaa, house AAAs</t>
+          <t>Admin read APIs (platform; audit log exists sinc…</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -2796,17 +2796,17 @@
         </is>
       </c>
       <c r="E45" s="3" t="n">
-        <v>46357</v>
+        <v>46351</v>
       </c>
       <c r="F45" s="3" t="n">
-        <v>46357</v>
+        <v>46356</v>
       </c>
       <c r="G45" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>T4.10</t>
+          <t>T4.6</t>
         </is>
       </c>
       <c r="I45" s="4" t="n">
@@ -2824,7 +2824,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>T4.8</t>
+          <t>T4.11</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2834,26 +2834,26 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Review/credits tests + proptests (02 §11 #4-9)</t>
+          <t>Name blocklist, admin_rename_aaa, house AAAs</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>sonnet-5</t>
+          <t>haiku-4.5</t>
         </is>
       </c>
       <c r="E46" s="3" t="n">
-        <v>46351</v>
+        <v>46357</v>
       </c>
       <c r="F46" s="3" t="n">
         <v>46357</v>
       </c>
       <c r="G46" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>T4.6,T4.9</t>
+          <t>T4.10</t>
         </is>
       </c>
       <c r="I46" s="4" t="n">
@@ -2871,17 +2871,17 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>T5.1</t>
+          <t>T4.8</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>P5</t>
+          <t>P4</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>payments skeleton: config, journal, guards, admin</t>
+          <t>Review/credits tests + proptests (02 §11 #4-9)</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -2890,21 +2890,21 @@
         </is>
       </c>
       <c r="E47" s="3" t="n">
-        <v>46336</v>
+        <v>46351</v>
       </c>
       <c r="F47" s="3" t="n">
-        <v>46337</v>
+        <v>46357</v>
       </c>
       <c r="G47" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>T1.2,SP-1</t>
+          <t>T4.6,T4.9</t>
         </is>
       </c>
       <c r="I47" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J47">
         <f>IF(I47&gt;=1,"Done",IF(TODAY()&gt;F47,"Late",IF(I47&gt;0,"In progress","Not started")))</f>
@@ -2918,7 +2918,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>T5.2</t>
+          <t>T5.1</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2928,7 +2928,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>CMC integration, XDR cache, quotes, deposit acco…</t>
+          <t>payments skeleton: config, journal, guards, admin</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -2937,21 +2937,21 @@
         </is>
       </c>
       <c r="E48" s="3" t="n">
-        <v>46338</v>
+        <v>46336</v>
       </c>
       <c r="F48" s="3" t="n">
-        <v>46339</v>
+        <v>46337</v>
       </c>
       <c r="G48" t="n">
         <v>2</v>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>T5.1</t>
+          <t>T1.2,SP-1</t>
         </is>
       </c>
       <c r="I48" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J48">
         <f>IF(I48&gt;=1,"Done",IF(TODAY()&gt;F48,"Late",IF(I48&gt;0,"In progress","Not started")))</f>
@@ -2965,7 +2965,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>T5.3</t>
+          <t>T5.2</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2975,26 +2975,26 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Spawn saga (wallet + deposit) + resume timer</t>
+          <t>CMC integration, XDR cache, quotes, deposit acco…</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>opus-5.5 (high)</t>
+          <t>sonnet-5</t>
         </is>
       </c>
       <c r="E49" s="3" t="n">
-        <v>46342</v>
+        <v>46338</v>
       </c>
       <c r="F49" s="3" t="n">
-        <v>46345</v>
+        <v>46339</v>
       </c>
       <c r="G49" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>T5.2,T2.2</t>
+          <t>T5.1</t>
         </is>
       </c>
       <c r="I49" s="4" t="n">
@@ -3012,7 +3012,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>T5.4</t>
+          <t>T5.3</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -3022,26 +3022,26 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>One-time top-up (wallet + deposit sweep)</t>
+          <t>Spawn saga (wallet + deposit) + resume timer</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>sonnet-5</t>
+          <t>opus-5.5 (high)</t>
         </is>
       </c>
       <c r="E50" s="3" t="n">
-        <v>46346</v>
+        <v>46342</v>
       </c>
       <c r="F50" s="3" t="n">
-        <v>46349</v>
+        <v>46345</v>
       </c>
       <c r="G50" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>T5.2</t>
+          <t>T5.2,T2.2</t>
         </is>
       </c>
       <c r="I50" s="4" t="n">
@@ -3059,7 +3059,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>T5.5</t>
+          <t>T5.4</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -3069,7 +3069,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Auto top-up mandates, rolling 30-day cap</t>
+          <t>One-time top-up (wallet + deposit sweep)</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -3078,17 +3078,17 @@
         </is>
       </c>
       <c r="E51" s="3" t="n">
-        <v>46350</v>
+        <v>46346</v>
       </c>
       <c r="F51" s="3" t="n">
-        <v>46356</v>
+        <v>46349</v>
       </c>
       <c r="G51" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>T5.4,T3.4</t>
+          <t>T5.2</t>
         </is>
       </c>
       <c r="I51" s="4" t="n">
@@ -3106,7 +3106,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>T5.6</t>
+          <t>T5.5</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -3116,7 +3116,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Payments PocketIC tests — ICP paths (04 §5)</t>
+          <t>Auto top-up mandates, rolling 30-day cap</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -3125,17 +3125,17 @@
         </is>
       </c>
       <c r="E52" s="3" t="n">
-        <v>46357</v>
+        <v>46350</v>
       </c>
       <c r="F52" s="3" t="n">
-        <v>46359</v>
+        <v>46356</v>
       </c>
       <c r="G52" t="n">
         <v>3</v>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>T5.3,T5.5</t>
+          <t>T5.4,T3.4</t>
         </is>
       </c>
       <c r="I52" s="4" t="n">
@@ -3153,7 +3153,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>T5.8</t>
+          <t>T5.6</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -3163,26 +3163,26 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>XRC rates, fuel treasury guard rails + auto inta…</t>
+          <t>Payments PocketIC tests — ICP paths (04 §5)</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>opus-5.5 (high)</t>
+          <t>sonnet-5</t>
         </is>
       </c>
       <c r="E53" s="3" t="n">
-        <v>46358</v>
+        <v>46357</v>
       </c>
       <c r="F53" s="3" t="n">
-        <v>46363</v>
+        <v>46359</v>
       </c>
       <c r="G53" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>T5.2</t>
+          <t>T5.3,T5.5</t>
         </is>
       </c>
       <c r="I53" s="4" t="n">
@@ -3200,7 +3200,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>T5.9</t>
+          <t>T5.8</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -3210,7 +3210,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>ckBTC fuel-pack deposits (address, update_balanc…</t>
+          <t>XRC rates, fuel treasury guard rails + auto inta…</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -3219,17 +3219,17 @@
         </is>
       </c>
       <c r="E54" s="3" t="n">
-        <v>46364</v>
+        <v>46358</v>
       </c>
       <c r="F54" s="3" t="n">
-        <v>46366</v>
+        <v>46363</v>
       </c>
       <c r="G54" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>T5.8</t>
+          <t>T5.2</t>
         </is>
       </c>
       <c r="I54" s="4" t="n">
@@ -3247,7 +3247,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>T5.10</t>
+          <t>T5.9</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -3257,26 +3257,26 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>ckETH fuel-pack deposits</t>
+          <t>ckBTC fuel-pack deposits (address, update_balanc…</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>sonnet-5</t>
+          <t>opus-5.5 (high)</t>
         </is>
       </c>
       <c r="E55" s="3" t="n">
         <v>46364</v>
       </c>
       <c r="F55" s="3" t="n">
-        <v>46365</v>
+        <v>46366</v>
       </c>
       <c r="G55" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>T5.8,SP-6</t>
+          <t>T5.8</t>
         </is>
       </c>
       <c r="I55" s="4" t="n">
@@ -3294,7 +3294,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>T5.13</t>
+          <t>T5.10</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -3304,7 +3304,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Non-ICP payment tests (04 §6.7)</t>
+          <t>ckETH fuel-pack deposits</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -3313,17 +3313,17 @@
         </is>
       </c>
       <c r="E56" s="3" t="n">
-        <v>46367</v>
+        <v>46364</v>
       </c>
       <c r="F56" s="3" t="n">
-        <v>46370</v>
+        <v>46365</v>
       </c>
       <c r="G56" t="n">
         <v>2</v>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>T5.9,T5.10</t>
+          <t>T5.8,SP-6</t>
         </is>
       </c>
       <c r="I56" s="4" t="n">
@@ -3341,7 +3341,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>T5.15</t>
+          <t>T5.13</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -3351,26 +3351,26 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Payments admin APIs (audit log exists since T5.1)</t>
+          <t>Non-ICP payment tests (04 §6.7)</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>haiku-4.5</t>
+          <t>sonnet-5</t>
         </is>
       </c>
       <c r="E57" s="3" t="n">
-        <v>46371</v>
+        <v>46367</v>
       </c>
       <c r="F57" s="3" t="n">
-        <v>46371</v>
+        <v>46370</v>
       </c>
       <c r="G57" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>T5.13</t>
+          <t>T5.9,T5.10</t>
         </is>
       </c>
       <c r="I57" s="4" t="n">
@@ -3388,7 +3388,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>T5.16</t>
+          <t>T5.15</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -3398,26 +3398,26 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Feature flags + invite codes (sponsored spawn)</t>
+          <t>Payments admin APIs (audit log exists since T5.1)</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>sonnet-5</t>
+          <t>haiku-4.5</t>
         </is>
       </c>
       <c r="E58" s="3" t="n">
-        <v>46360</v>
+        <v>46371</v>
       </c>
       <c r="F58" s="3" t="n">
-        <v>46363</v>
+        <v>46371</v>
       </c>
       <c r="G58" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>T5.3</t>
+          <t>T5.13</t>
         </is>
       </c>
       <c r="I58" s="4" t="n">
@@ -3435,7 +3435,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>T5.17</t>
+          <t>T5.16</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -3445,26 +3445,26 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>treasury canister: owner-funded reserve, cycles …</t>
+          <t>Feature flags + invite codes (sponsored spawn)</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>opus-5.5 (high)</t>
+          <t>sonnet-5</t>
         </is>
       </c>
       <c r="E59" s="3" t="n">
-        <v>46364</v>
+        <v>46360</v>
       </c>
       <c r="F59" s="3" t="n">
-        <v>46366</v>
+        <v>46363</v>
       </c>
       <c r="G59" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>T2.1,T1.4</t>
+          <t>T5.3</t>
         </is>
       </c>
       <c r="I59" s="4" t="n">
@@ -3482,7 +3482,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>T5.18</t>
+          <t>T5.17</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -3492,30 +3492,30 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>treasury PocketIC tests (ICP ledger + CMC, no NN…</t>
+          <t>treasury canister: owner-funded reserve, cycles …</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>sonnet-5</t>
+          <t>opus-5.5 (high)</t>
         </is>
       </c>
       <c r="E60" s="3" t="n">
-        <v>46367</v>
+        <v>46364</v>
       </c>
       <c r="F60" s="3" t="n">
-        <v>46367</v>
+        <v>46366</v>
       </c>
       <c r="G60" t="n">
+        <v>3</v>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>T2.1,T1.4</t>
+        </is>
+      </c>
+      <c r="I60" s="4" t="n">
         <v>1</v>
-      </c>
-      <c r="H60" t="inlineStr">
-        <is>
-          <t>T5.17</t>
-        </is>
-      </c>
-      <c r="I60" s="4" t="n">
-        <v>0</v>
       </c>
       <c r="J60">
         <f>IF(I60&gt;=1,"Done",IF(TODAY()&gt;F60,"Late",IF(I60&gt;0,"In progress","Not started")))</f>
@@ -3529,7 +3529,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>T5.7</t>
+          <t>T5.18</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -3539,26 +3539,26 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Internal payments security review</t>
+          <t>treasury PocketIC tests (ICP ledger + CMC, no NN…</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>opus-5.5 (high)</t>
+          <t>sonnet-5</t>
         </is>
       </c>
       <c r="E61" s="3" t="n">
-        <v>46371</v>
+        <v>46367</v>
       </c>
       <c r="F61" s="3" t="n">
-        <v>46372</v>
+        <v>46367</v>
       </c>
       <c r="G61" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>T5.6,T5.13,T5.16</t>
+          <t>T5.17</t>
         </is>
       </c>
       <c r="I61" s="4" t="n">
@@ -3576,40 +3576,40 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>T6.1</t>
+          <t>T5.7</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>P6</t>
+          <t>P5</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>App scaffold: routing, bindgen, II auth, ic_env,…</t>
+          <t>Internal payments security review</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>sonnet-5</t>
+          <t>opus-5.5 (high)</t>
         </is>
       </c>
       <c r="E62" s="3" t="n">
-        <v>46367</v>
+        <v>46371</v>
       </c>
       <c r="F62" s="3" t="n">
-        <v>46371</v>
+        <v>46372</v>
       </c>
       <c r="G62" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>T1.1</t>
+          <t>T5.6,T5.13,T5.16</t>
         </is>
       </c>
       <c r="I62" s="4" t="n">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="J62">
         <f>IF(I62&gt;=1,"Done",IF(TODAY()&gt;F62,"Late",IF(I62&gt;0,"In progress","Not started")))</f>
@@ -3623,7 +3623,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>T6.3</t>
+          <t>T6.1</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -3633,7 +3633,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Landing, Discovery Museum feed, Discovery detail…</t>
+          <t>App scaffold: routing, bindgen, II auth, ic_env,…</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -3642,21 +3642,21 @@
         </is>
       </c>
       <c r="E63" s="3" t="n">
-        <v>46372</v>
+        <v>46367</v>
       </c>
       <c r="F63" s="3" t="n">
-        <v>46378</v>
+        <v>46371</v>
       </c>
       <c r="G63" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>T6.1</t>
+          <t>T1.1</t>
         </is>
       </c>
       <c r="I63" s="4" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="J63">
         <f>IF(I63&gt;=1,"Done",IF(TODAY()&gt;F63,"Late",IF(I63&gt;0,"In progress","Not started")))</f>
@@ -3670,7 +3670,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>T6.4</t>
+          <t>T6.3</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -3680,26 +3680,26 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>AAA profile + Leaderboard</t>
+          <t>Landing, Discovery Museum feed, Discovery detail…</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>haiku-4.5</t>
+          <t>sonnet-5</t>
         </is>
       </c>
       <c r="E64" s="3" t="n">
-        <v>46379</v>
+        <v>46372</v>
       </c>
       <c r="F64" s="3" t="n">
-        <v>46385</v>
+        <v>46378</v>
       </c>
       <c r="G64" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>T6.3</t>
+          <t>T6.1</t>
         </is>
       </c>
       <c r="I64" s="4" t="n">
@@ -3717,7 +3717,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>T6.5</t>
+          <t>T6.4</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -3727,26 +3727,26 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Payment component (wallet + deposit)</t>
+          <t>AAA profile + Leaderboard</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>sonnet-5</t>
+          <t>haiku-4.5</t>
         </is>
       </c>
       <c r="E65" s="3" t="n">
-        <v>46372</v>
+        <v>46379</v>
       </c>
       <c r="F65" s="3" t="n">
-        <v>46377</v>
+        <v>46385</v>
       </c>
       <c r="G65" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>T6.1,SP-2,T5.4</t>
+          <t>T6.3</t>
         </is>
       </c>
       <c r="I65" s="4" t="n">
@@ -3764,7 +3764,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>T6.6</t>
+          <t>T6.5</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -3774,26 +3774,26 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Spawn flow</t>
+          <t>Payment component (wallet + deposit)</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>haiku-4.5</t>
+          <t>sonnet-5</t>
         </is>
       </c>
       <c r="E66" s="3" t="n">
-        <v>46378</v>
+        <v>46372</v>
       </c>
       <c r="F66" s="3" t="n">
-        <v>46379</v>
+        <v>46377</v>
       </c>
       <c r="G66" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>T6.5,T5.3</t>
+          <t>T6.1,SP-2,T5.4</t>
         </is>
       </c>
       <c r="I66" s="4" t="n">
@@ -3811,7 +3811,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>T6.7</t>
+          <t>T6.6</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -3821,26 +3821,26 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Owner dashboard</t>
+          <t>Spawn flow</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>sonnet-5</t>
+          <t>haiku-4.5</t>
         </is>
       </c>
       <c r="E67" s="3" t="n">
         <v>46378</v>
       </c>
       <c r="F67" s="3" t="n">
-        <v>46385</v>
+        <v>46379</v>
       </c>
       <c r="G67" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>T6.1,T3.3,T4.6</t>
+          <t>T6.5,T5.3</t>
         </is>
       </c>
       <c r="I67" s="4" t="n">
@@ -3858,7 +3858,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>T6.8</t>
+          <t>T6.7</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -3868,26 +3868,26 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Connect your agent + Activity &amp; records</t>
+          <t>Owner dashboard</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>haiku-4.5</t>
+          <t>sonnet-5</t>
         </is>
       </c>
       <c r="E68" s="3" t="n">
-        <v>46386</v>
+        <v>46378</v>
       </c>
       <c r="F68" s="3" t="n">
-        <v>46392</v>
+        <v>46385</v>
       </c>
       <c r="G68" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>T6.7</t>
+          <t>T6.1,T3.3,T4.6</t>
         </is>
       </c>
       <c r="I68" s="4" t="n">
@@ -3905,7 +3905,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>T6.9</t>
+          <t>T6.8</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -3915,7 +3915,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Fuel &amp; billing + auto top-up</t>
+          <t>Connect your agent + Activity &amp; records</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -3924,17 +3924,17 @@
         </is>
       </c>
       <c r="E69" s="3" t="n">
-        <v>46384</v>
+        <v>46386</v>
       </c>
       <c r="F69" s="3" t="n">
-        <v>46386</v>
+        <v>46392</v>
       </c>
       <c r="G69" t="n">
         <v>3</v>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>T6.5,T5.5</t>
+          <t>T6.7</t>
         </is>
       </c>
       <c r="I69" s="4" t="n">
@@ -3952,7 +3952,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>T6.11</t>
+          <t>T6.9</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -3962,26 +3962,26 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>BTC &amp; ETH methods + feature-flag gating</t>
+          <t>Fuel &amp; billing + auto top-up</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>sonnet-5</t>
+          <t>haiku-4.5</t>
         </is>
       </c>
       <c r="E70" s="3" t="n">
+        <v>46384</v>
+      </c>
+      <c r="F70" s="3" t="n">
         <v>46386</v>
       </c>
-      <c r="F70" s="3" t="n">
-        <v>46393</v>
-      </c>
       <c r="G70" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>T6.5,T5.9,T5.10</t>
+          <t>T6.5,T5.5</t>
         </is>
       </c>
       <c r="I70" s="4" t="n">
@@ -3999,7 +3999,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>T6.12</t>
+          <t>T6.11</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -4009,7 +4009,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Admin console (8 screens)</t>
+          <t>BTC &amp; ETH methods + feature-flag gating</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -4018,17 +4018,17 @@
         </is>
       </c>
       <c r="E71" s="3" t="n">
-        <v>46391</v>
+        <v>46386</v>
       </c>
       <c r="F71" s="3" t="n">
-        <v>46395</v>
+        <v>46393</v>
       </c>
       <c r="G71" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>T6.1,T4.10,T5.15</t>
+          <t>T6.5,T5.9,T5.10</t>
         </is>
       </c>
       <c r="I71" s="4" t="n">
@@ -4046,7 +4046,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>T6.13</t>
+          <t>T6.12</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -4056,26 +4056,26 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Firebase analytics + consent + event taxonomy + …</t>
+          <t>Admin console (8 screens)</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>haiku-4.5</t>
+          <t>sonnet-5</t>
         </is>
       </c>
       <c r="E72" s="3" t="n">
-        <v>46393</v>
+        <v>46391</v>
       </c>
       <c r="F72" s="3" t="n">
-        <v>46394</v>
+        <v>46395</v>
       </c>
       <c r="G72" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>T6.1</t>
+          <t>T6.1,T4.10,T5.15</t>
         </is>
       </c>
       <c r="I72" s="4" t="n">
@@ -4093,7 +4093,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>T6.14</t>
+          <t>T6.13</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -4103,7 +4103,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>About/legal/practice pages, invite spawn UI, adm…</t>
+          <t>Firebase analytics + consent + event taxonomy + …</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -4112,17 +4112,17 @@
         </is>
       </c>
       <c r="E73" s="3" t="n">
-        <v>46398</v>
+        <v>46393</v>
       </c>
       <c r="F73" s="3" t="n">
-        <v>46400</v>
+        <v>46394</v>
       </c>
       <c r="G73" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>T6.12,T5.16,T5.18</t>
+          <t>T6.1</t>
         </is>
       </c>
       <c r="I73" s="4" t="n">
@@ -4140,7 +4140,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>T6.10</t>
+          <t>T6.14</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -4150,26 +4150,26 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>States, accessibility, Playwright smoke</t>
+          <t>About/legal/practice pages, invite spawn UI, adm…</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>sonnet-5</t>
+          <t>haiku-4.5</t>
         </is>
       </c>
       <c r="E74" s="3" t="n">
-        <v>46401</v>
+        <v>46398</v>
       </c>
       <c r="F74" s="3" t="n">
-        <v>46405</v>
+        <v>46400</v>
       </c>
       <c r="G74" t="n">
         <v>3</v>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>T6.4,T6.6,T6.8,T6.9,T6.11,T6.12,T6.13,T6.14</t>
+          <t>T6.12,T5.16,T5.18</t>
         </is>
       </c>
       <c r="I74" s="4" t="n">
@@ -4187,17 +4187,17 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>T7.1</t>
+          <t>T6.10</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>P7</t>
+          <t>P6</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Upgrade tests for all canisters</t>
+          <t>States, accessibility, Playwright smoke</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -4206,17 +4206,17 @@
         </is>
       </c>
       <c r="E75" s="3" t="n">
-        <v>46394</v>
+        <v>46401</v>
       </c>
       <c r="F75" s="3" t="n">
-        <v>46395</v>
+        <v>46405</v>
       </c>
       <c r="G75" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>T4.8,T5.6</t>
+          <t>T6.4,T6.6,T6.8,T6.9,T6.11,T6.12,T6.13,T6.14</t>
         </is>
       </c>
       <c r="I75" s="4" t="n">
@@ -4234,7 +4234,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>T7.2</t>
+          <t>T7.1</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -4244,7 +4244,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Load test: 200 AAAs × 100 tasks</t>
+          <t>Upgrade tests for all canisters</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -4253,17 +4253,17 @@
         </is>
       </c>
       <c r="E76" s="3" t="n">
-        <v>46398</v>
+        <v>46394</v>
       </c>
       <c r="F76" s="3" t="n">
-        <v>46399</v>
+        <v>46395</v>
       </c>
       <c r="G76" t="n">
         <v>2</v>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>T7.1</t>
+          <t>T4.8,T5.6</t>
         </is>
       </c>
       <c r="I76" s="4" t="n">
@@ -4281,7 +4281,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>T7.3</t>
+          <t>T7.2</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -4291,7 +4291,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Cycle cost measurement &amp; fee retune</t>
+          <t>Load test: 200 AAAs × 100 tasks</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -4300,17 +4300,17 @@
         </is>
       </c>
       <c r="E77" s="3" t="n">
-        <v>46400</v>
+        <v>46398</v>
       </c>
       <c r="F77" s="3" t="n">
-        <v>46401</v>
+        <v>46399</v>
       </c>
       <c r="G77" t="n">
         <v>2</v>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>T7.2</t>
+          <t>T7.1</t>
         </is>
       </c>
       <c r="I77" s="4" t="n">
@@ -4328,7 +4328,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>T7.4</t>
+          <t>T7.3</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -4338,7 +4338,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Reproducible AAA build + manual upgrade docs</t>
+          <t>Cycle cost measurement &amp; fee retune</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -4347,17 +4347,17 @@
         </is>
       </c>
       <c r="E78" s="3" t="n">
-        <v>46398</v>
+        <v>46400</v>
       </c>
       <c r="F78" s="3" t="n">
-        <v>46399</v>
+        <v>46401</v>
       </c>
       <c r="G78" t="n">
         <v>2</v>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>T3.6,T5.7</t>
+          <t>T7.2</t>
         </is>
       </c>
       <c r="I78" s="4" t="n">
@@ -4375,7 +4375,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>T7.7</t>
+          <t>T7.4</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -4385,26 +4385,26 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Prompt-injection test with reference agent</t>
+          <t>Reproducible AAA build + manual upgrade docs</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>opus-5.5 (high)</t>
+          <t>sonnet-5</t>
         </is>
       </c>
       <c r="E79" s="3" t="n">
-        <v>46400</v>
+        <v>46398</v>
       </c>
       <c r="F79" s="3" t="n">
-        <v>46400</v>
+        <v>46399</v>
       </c>
       <c r="G79" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>T3.7,T4.7</t>
+          <t>T3.6,T5.7</t>
         </is>
       </c>
       <c r="I79" s="4" t="n">
@@ -4422,7 +4422,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>T7.9</t>
+          <t>T7.7</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -4432,26 +4432,26 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Traceability audit + coverage gates to thresholds</t>
+          <t>Prompt-injection test with reference agent</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>haiku-4.5</t>
+          <t>opus-5.5 (high)</t>
         </is>
       </c>
       <c r="E80" s="3" t="n">
-        <v>46401</v>
+        <v>46400</v>
       </c>
       <c r="F80" s="3" t="n">
-        <v>46402</v>
+        <v>46400</v>
       </c>
       <c r="G80" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>T7.1</t>
+          <t>T3.7,T4.7</t>
         </is>
       </c>
       <c r="I80" s="4" t="n">
@@ -4469,7 +4469,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>T7.10</t>
+          <t>T7.9</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -4479,7 +4479,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Practice set + open data release tooling</t>
+          <t>Traceability audit + coverage gates to thresholds</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -4488,17 +4488,17 @@
         </is>
       </c>
       <c r="E81" s="3" t="n">
+        <v>46401</v>
+      </c>
+      <c r="F81" s="3" t="n">
         <v>46402</v>
-      </c>
-      <c r="F81" s="3" t="n">
-        <v>46405</v>
       </c>
       <c r="G81" t="n">
         <v>2</v>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>T1.7,T4.8</t>
+          <t>T7.1</t>
         </is>
       </c>
       <c r="I81" s="4" t="n">
@@ -4516,7 +4516,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>T7.5</t>
+          <t>T7.10</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -4526,26 +4526,26 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>External security review (payments + platform)</t>
+          <t>Practice set + open data release tooling</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>human</t>
+          <t>haiku-4.5</t>
         </is>
       </c>
       <c r="E82" s="3" t="n">
-        <v>46373</v>
+        <v>46402</v>
       </c>
       <c r="F82" s="3" t="n">
-        <v>46379</v>
+        <v>46405</v>
       </c>
       <c r="G82" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>T5.7,T4.8</t>
+          <t>T1.7,T4.8</t>
         </is>
       </c>
       <c r="I82" s="4" t="n">
@@ -4563,7 +4563,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>T7.6</t>
+          <t>T7.5</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -4573,26 +4573,26 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Fix security findings</t>
+          <t>External security review (payments + platform)</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>opus-5.5 (high)</t>
+          <t>human</t>
         </is>
       </c>
       <c r="E83" s="3" t="n">
-        <v>46405</v>
+        <v>46373</v>
       </c>
       <c r="F83" s="3" t="n">
-        <v>46407</v>
+        <v>46379</v>
       </c>
       <c r="G83" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>T7.5</t>
+          <t>T5.7,T4.8</t>
         </is>
       </c>
       <c r="I83" s="4" t="n">
@@ -4610,7 +4610,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>T7.11</t>
+          <t>T7.6</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -4620,26 +4620,26 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Continuous data refresh: 15-day scheduled job (n…</t>
+          <t>Fix security findings</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>sonnet-5</t>
+          <t>opus-5.5 (high)</t>
         </is>
       </c>
       <c r="E84" s="3" t="n">
-        <v>46406</v>
+        <v>46405</v>
       </c>
       <c r="F84" s="3" t="n">
         <v>46407</v>
       </c>
       <c r="G84" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>T1.7,T2.3,T8.14</t>
+          <t>T7.5</t>
         </is>
       </c>
       <c r="I84" s="4" t="n">
@@ -4657,36 +4657,36 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>T8.14</t>
+          <t>T7.11</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>P8</t>
+          <t>P7</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Create Cloudflare R2 bucket + API token + custom…</t>
+          <t>Continuous data refresh: 15-day scheduled job (n…</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>human</t>
+          <t>sonnet-5</t>
         </is>
       </c>
       <c r="E85" s="3" t="n">
-        <v>46316</v>
+        <v>46406</v>
       </c>
       <c r="F85" s="3" t="n">
-        <v>46316</v>
+        <v>46407</v>
       </c>
       <c r="G85" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>T1.7</t>
+          <t>T1.7,T2.3,T8.14</t>
         </is>
       </c>
       <c r="I85" s="4" t="n">
@@ -4704,7 +4704,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>T8.16</t>
+          <t>T8.14</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -4714,26 +4714,26 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Scale dataset to 20,000 subjects (R-62) and publ…</t>
+          <t>Create Cloudflare R2 bucket + API token + custom…</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>haiku-4.5</t>
+          <t>human</t>
         </is>
       </c>
       <c r="E86" s="3" t="n">
-        <v>46406</v>
+        <v>46316</v>
       </c>
       <c r="F86" s="3" t="n">
-        <v>46406</v>
+        <v>46316</v>
       </c>
       <c r="G86" t="n">
         <v>1</v>
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>T8.14</t>
+          <t>T1.7</t>
         </is>
       </c>
       <c r="I86" s="4" t="n">
@@ -4751,7 +4751,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>T8.1</t>
+          <t>T8.16</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -4761,26 +4761,26 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Staging deploy, deploy workflow, snapshots, cycl…</t>
+          <t>Scale dataset to 20,000 subjects (R-62) and publ…</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>sonnet-5</t>
+          <t>haiku-4.5</t>
         </is>
       </c>
       <c r="E87" s="3" t="n">
-        <v>46407</v>
+        <v>46406</v>
       </c>
       <c r="F87" s="3" t="n">
-        <v>46408</v>
+        <v>46406</v>
       </c>
       <c r="G87" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>T7.1</t>
+          <t>T8.14</t>
         </is>
       </c>
       <c r="I87" s="4" t="n">
@@ -4798,7 +4798,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>T8.2</t>
+          <t>T8.1</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -4808,26 +4808,26 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Upload subjects/protocol/honeypots to staging</t>
+          <t>Staging deploy, deploy workflow, snapshots, cycl…</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>haiku-4.5</t>
+          <t>sonnet-5</t>
         </is>
       </c>
       <c r="E88" s="3" t="n">
-        <v>46409</v>
+        <v>46407</v>
       </c>
       <c r="F88" s="3" t="n">
-        <v>46409</v>
+        <v>46408</v>
       </c>
       <c r="G88" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>T8.16,T8.1,T7.6</t>
+          <t>T7.1</t>
         </is>
       </c>
       <c r="I88" s="4" t="n">
@@ -4845,7 +4845,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>T8.5</t>
+          <t>T8.2</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -4855,26 +4855,26 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Fund prod treasury with ICP float (10–20 ICP) + …</t>
+          <t>Upload subjects/protocol/honeypots to staging</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>human</t>
+          <t>haiku-4.5</t>
         </is>
       </c>
       <c r="E89" s="3" t="n">
-        <v>46428</v>
+        <v>46409</v>
       </c>
       <c r="F89" s="3" t="n">
-        <v>46428</v>
+        <v>46409</v>
       </c>
       <c r="G89" t="n">
         <v>1</v>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>T8.6</t>
+          <t>T8.16,T8.1,T7.6</t>
         </is>
       </c>
       <c r="I89" s="4" t="n">
@@ -4892,7 +4892,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>T8.3</t>
+          <t>T8.5</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -4902,7 +4902,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Closed beta (10-20 owners)</t>
+          <t>Fund prod treasury with ICP float (10–20 ICP) + …</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -4911,17 +4911,17 @@
         </is>
       </c>
       <c r="E90" s="3" t="n">
-        <v>46412</v>
+        <v>46428</v>
       </c>
       <c r="F90" s="3" t="n">
-        <v>46423</v>
+        <v>46428</v>
       </c>
       <c r="G90" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>T8.2,T6.10</t>
+          <t>T8.6</t>
         </is>
       </c>
       <c r="I90" s="4" t="n">
@@ -4939,7 +4939,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>T8.4</t>
+          <t>T8.3</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -4949,12 +4949,12 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Beta fixes &amp; tuning</t>
+          <t>Closed beta (10-20 owners)</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>sonnet-5</t>
+          <t>human</t>
         </is>
       </c>
       <c r="E91" s="3" t="n">
@@ -4986,7 +4986,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>T8.6</t>
+          <t>T8.4</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -4996,7 +4996,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Production deploy, II metadata, treasury watch l…</t>
+          <t>Beta fixes &amp; tuning</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -5005,17 +5005,17 @@
         </is>
       </c>
       <c r="E92" s="3" t="n">
-        <v>46426</v>
+        <v>46412</v>
       </c>
       <c r="F92" s="3" t="n">
-        <v>46427</v>
+        <v>46423</v>
       </c>
       <c r="G92" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>T8.3,T8.4,T8.13</t>
+          <t>T8.2,T6.10</t>
         </is>
       </c>
       <c r="I92" s="4" t="n">
@@ -5033,7 +5033,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>T8.7</t>
+          <t>T8.6</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -5043,26 +5043,26 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Public launch</t>
+          <t>Production deploy, II metadata, treasury watch l…</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>human</t>
+          <t>sonnet-5</t>
         </is>
       </c>
       <c r="E93" s="3" t="n">
-        <v>46429</v>
+        <v>46426</v>
       </c>
       <c r="F93" s="3" t="n">
-        <v>46429</v>
+        <v>46427</v>
       </c>
       <c r="G93" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>T8.6,T8.5,T9.5</t>
+          <t>T8.3,T8.4,T8.13</t>
         </is>
       </c>
       <c r="I93" s="4" t="n">
@@ -5080,36 +5080,36 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>T9.1</t>
+          <t>T8.7</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>P9</t>
+          <t>P8</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Import mockups (Claude Design), reconcile, desig…</t>
+          <t>Public launch</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>sonnet-5</t>
+          <t>human</t>
         </is>
       </c>
       <c r="E94" s="3" t="n">
-        <v>46408</v>
+        <v>46429</v>
       </c>
       <c r="F94" s="3" t="n">
-        <v>46413</v>
+        <v>46429</v>
       </c>
       <c r="G94" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>T6.10</t>
+          <t>T8.6,T8.5,T9.5</t>
         </is>
       </c>
       <c r="I94" s="4" t="n">
@@ -5127,7 +5127,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>T9.2</t>
+          <t>T9.1</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -5137,7 +5137,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Style public pages: landing, museum, discovery, …</t>
+          <t>Import mockups (Claude Design), reconcile, desig…</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -5146,17 +5146,17 @@
         </is>
       </c>
       <c r="E95" s="3" t="n">
-        <v>46414</v>
+        <v>46408</v>
       </c>
       <c r="F95" s="3" t="n">
-        <v>46419</v>
+        <v>46413</v>
       </c>
       <c r="G95" t="n">
         <v>4</v>
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>T9.1</t>
+          <t>T6.10</t>
         </is>
       </c>
       <c r="I95" s="4" t="n">
@@ -5174,7 +5174,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>T9.3</t>
+          <t>T9.2</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -5184,7 +5184,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Style owner flows: spawn, dashboard, connect age…</t>
+          <t>Style public pages: landing, museum, discovery, …</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -5221,7 +5221,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>T9.4</t>
+          <t>T9.3</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -5231,22 +5231,22 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Style admin console + about/legal/practice pages</t>
+          <t>Style owner flows: spawn, dashboard, connect age…</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>haiku-4.5</t>
+          <t>sonnet-5</t>
         </is>
       </c>
       <c r="E97" s="3" t="n">
-        <v>46420</v>
+        <v>46414</v>
       </c>
       <c r="F97" s="3" t="n">
-        <v>46421</v>
+        <v>46419</v>
       </c>
       <c r="G97" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H97" t="inlineStr">
         <is>
@@ -5268,7 +5268,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>T9.5</t>
+          <t>T9.4</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -5278,7 +5278,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Responsive/mobile pass, visual-regression baseli…</t>
+          <t>Style admin console + about/legal/practice pages</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -5287,17 +5287,17 @@
         </is>
       </c>
       <c r="E98" s="3" t="n">
-        <v>46422</v>
+        <v>46420</v>
       </c>
       <c r="F98" s="3" t="n">
-        <v>46423</v>
+        <v>46421</v>
       </c>
       <c r="G98" t="n">
         <v>2</v>
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>T9.2,T9.3,T9.4</t>
+          <t>T9.1</t>
         </is>
       </c>
       <c r="I98" s="4" t="n">
@@ -5315,36 +5315,36 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>T8.13</t>
+          <t>T9.5</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>P8</t>
+          <t>P9</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Custom domain + II alternative origins</t>
+          <t>Responsive/mobile pass, visual-regression baseli…</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>human</t>
+          <t>haiku-4.5</t>
         </is>
       </c>
       <c r="E99" s="3" t="n">
-        <v>46409</v>
+        <v>46422</v>
       </c>
       <c r="F99" s="3" t="n">
-        <v>46409</v>
+        <v>46423</v>
       </c>
       <c r="G99" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>T8.1</t>
+          <t>T9.2,T9.3,T9.4</t>
         </is>
       </c>
       <c r="I99" s="4" t="n">
@@ -5362,7 +5362,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>T8.12</t>
+          <t>T8.13</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -5372,7 +5372,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Firebase projects (staging/prod) + GA4 funnels &amp;…</t>
+          <t>Custom domain + II alternative origins</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -5381,17 +5381,17 @@
         </is>
       </c>
       <c r="E100" s="3" t="n">
-        <v>46296</v>
+        <v>46409</v>
       </c>
       <c r="F100" s="3" t="n">
-        <v>46296</v>
+        <v>46409</v>
       </c>
       <c r="G100" t="n">
         <v>1</v>
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>T0.4</t>
+          <t>T8.1</t>
         </is>
       </c>
       <c r="I100" s="4" t="n">
@@ -5409,7 +5409,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>T8.15</t>
+          <t>T8.12</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -5419,7 +5419,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Owner review: discovery + peer-review agent proc…</t>
+          <t>Firebase projects (staging/prod) + GA4 funnels &amp;…</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -5456,7 +5456,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>T8.8</t>
+          <t>T8.15</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -5466,7 +5466,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Compliance check for crypto fuel packs (recommen…</t>
+          <t>Owner review: discovery + peer-review agent proc…</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -5478,10 +5478,10 @@
         <v>46296</v>
       </c>
       <c r="F102" s="3" t="n">
-        <v>46302</v>
+        <v>46296</v>
       </c>
       <c r="G102" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H102" t="inlineStr">
         <is>
@@ -5503,7 +5503,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>T8.9</t>
+          <t>T8.8</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -5513,7 +5513,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Enable BTC/ETH on production</t>
+          <t>Compliance check for crypto fuel packs (recommen…</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -5522,17 +5522,17 @@
         </is>
       </c>
       <c r="E103" s="3" t="n">
-        <v>46428</v>
+        <v>46296</v>
       </c>
       <c r="F103" s="3" t="n">
-        <v>46428</v>
+        <v>46302</v>
       </c>
       <c r="G103" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>T8.6,T8.8</t>
+          <t>T0.4</t>
         </is>
       </c>
       <c r="I103" s="4" t="n">
@@ -5547,8 +5547,55 @@
         <v/>
       </c>
     </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>T8.9</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>P8</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Enable BTC/ETH on production</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>human</t>
+        </is>
+      </c>
+      <c r="E104" s="3" t="n">
+        <v>46428</v>
+      </c>
+      <c r="F104" s="3" t="n">
+        <v>46428</v>
+      </c>
+      <c r="G104" t="n">
+        <v>1</v>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>T8.6,T8.8</t>
+        </is>
+      </c>
+      <c r="I104" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J104">
+        <f>IF(I104&gt;=1,"Done",IF(TODAY()&gt;F104,"Late",IF(I104&gt;0,"In progress","Not started")))</f>
+        <v/>
+      </c>
+      <c r="K104">
+        <f>G104*I104</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="L2:AF103">
+  <conditionalFormatting sqref="L2:AF104">
     <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="1">
       <formula>AND(L$1+6&gt;=$E2,L$1&lt;=$F2,L$1&lt;=$E2+($F2-$E2)*$I2)</formula>
     </cfRule>
@@ -5586,7 +5633,7 @@
       <formula>AND(TODAY()&gt;=L$1,TODAY()&lt;L$1+7)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J2:J103">
+  <conditionalFormatting sqref="J2:J104">
     <cfRule type="expression" priority="13" dxfId="12">
       <formula>LEFT(J2,4)="Late"</formula>
     </cfRule>
@@ -5788,7 +5835,7 @@
         <v>46304</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>46321</v>
+        <v>46323</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
@@ -6117,7 +6164,7 @@
         <v/>
       </c>
       <c r="G12" s="17">
-        <f>IF(C12&gt;0,SUM(Gantt!K2:K103)/C12,0)</f>
+        <f>IF(C12&gt;0,SUM(Gantt!K2:K104)/C12,0)</f>
         <v/>
       </c>
       <c r="H12" s="18" t="n">

</xml_diff>

<commit_message>
T3.8: one-command local seed (protocol v1, 500 subjects, AAA wasm, local image server); admin bootstrap on upgrade; immutable wasm versions
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/space-compute-gantt-v3.xlsx
+++ b/docs/space-compute-gantt-v3.xlsx
@@ -1964,7 +1964,7 @@
         </is>
       </c>
       <c r="I27" s="4" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="J27">
         <f>IF(I27&gt;=1,"Done",IF(TODAY()&gt;F27,"Late",IF(I27&gt;0,"In progress","Not started")))</f>
@@ -2152,7 +2152,7 @@
         </is>
       </c>
       <c r="I31" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J31">
         <f>IF(I31&gt;=1,"Done",IF(TODAY()&gt;F31,"Late",IF(I31&gt;0,"In progress","Not started")))</f>
@@ -2293,7 +2293,7 @@
         </is>
       </c>
       <c r="I34" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J34">
         <f>IF(I34&gt;=1,"Done",IF(TODAY()&gt;F34,"Late",IF(I34&gt;0,"In progress","Not started")))</f>
@@ -2998,7 +2998,7 @@
         </is>
       </c>
       <c r="I49" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J49">
         <f>IF(I49&gt;=1,"Done",IF(TODAY()&gt;F49,"Late",IF(I49&gt;0,"In progress","Not started")))</f>

</xml_diff>

<commit_message>
plan: remove Firebase/GA4 analytics (T6.13, T8.12) - not needed for MVP
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/space-compute-gantt-v3.xlsx
+++ b/docs/space-compute-gantt-v3.xlsx
@@ -600,7 +600,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF104"/>
+  <dimension ref="A1:AF102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -4093,7 +4093,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>T6.13</t>
+          <t>T6.14</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -4103,7 +4103,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Firebase analytics + consent + event taxonomy + …</t>
+          <t>About/legal/practice pages, invite spawn UI, adm…</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -4112,17 +4112,17 @@
         </is>
       </c>
       <c r="E73" s="3" t="n">
-        <v>46393</v>
+        <v>46398</v>
       </c>
       <c r="F73" s="3" t="n">
-        <v>46394</v>
+        <v>46400</v>
       </c>
       <c r="G73" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>T6.1</t>
+          <t>T6.12,T5.16,T5.18</t>
         </is>
       </c>
       <c r="I73" s="4" t="n">
@@ -4140,7 +4140,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>T6.14</t>
+          <t>T6.10</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -4150,26 +4150,26 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>About/legal/practice pages, invite spawn UI, adm…</t>
+          <t>States, accessibility, Playwright smoke</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>haiku-4.5</t>
+          <t>sonnet-5</t>
         </is>
       </c>
       <c r="E74" s="3" t="n">
-        <v>46398</v>
+        <v>46401</v>
       </c>
       <c r="F74" s="3" t="n">
-        <v>46400</v>
+        <v>46405</v>
       </c>
       <c r="G74" t="n">
         <v>3</v>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>T6.12,T5.16,T5.18</t>
+          <t>T6.4,T6.6,T6.8,T6.9,T6.11,T6.12,T6.14</t>
         </is>
       </c>
       <c r="I74" s="4" t="n">
@@ -4187,17 +4187,17 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>T6.10</t>
+          <t>T7.1</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>P6</t>
+          <t>P7</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>States, accessibility, Playwright smoke</t>
+          <t>Upgrade tests for all canisters</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -4206,17 +4206,17 @@
         </is>
       </c>
       <c r="E75" s="3" t="n">
-        <v>46401</v>
+        <v>46394</v>
       </c>
       <c r="F75" s="3" t="n">
-        <v>46405</v>
+        <v>46395</v>
       </c>
       <c r="G75" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>T6.4,T6.6,T6.8,T6.9,T6.11,T6.12,T6.13,T6.14</t>
+          <t>T4.8,T5.6</t>
         </is>
       </c>
       <c r="I75" s="4" t="n">
@@ -4234,7 +4234,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>T7.1</t>
+          <t>T7.2</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -4244,7 +4244,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Upgrade tests for all canisters</t>
+          <t>Load test: 200 AAAs × 100 tasks</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -4253,17 +4253,17 @@
         </is>
       </c>
       <c r="E76" s="3" t="n">
-        <v>46394</v>
+        <v>46398</v>
       </c>
       <c r="F76" s="3" t="n">
-        <v>46395</v>
+        <v>46399</v>
       </c>
       <c r="G76" t="n">
         <v>2</v>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>T4.8,T5.6</t>
+          <t>T7.1</t>
         </is>
       </c>
       <c r="I76" s="4" t="n">
@@ -4281,7 +4281,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>T7.2</t>
+          <t>T7.3</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -4291,7 +4291,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Load test: 200 AAAs × 100 tasks</t>
+          <t>Cycle cost measurement &amp; fee retune</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -4300,17 +4300,17 @@
         </is>
       </c>
       <c r="E77" s="3" t="n">
-        <v>46398</v>
+        <v>46400</v>
       </c>
       <c r="F77" s="3" t="n">
-        <v>46399</v>
+        <v>46401</v>
       </c>
       <c r="G77" t="n">
         <v>2</v>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>T7.1</t>
+          <t>T7.2</t>
         </is>
       </c>
       <c r="I77" s="4" t="n">
@@ -4328,7 +4328,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>T7.3</t>
+          <t>T7.4</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -4338,7 +4338,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Cycle cost measurement &amp; fee retune</t>
+          <t>Reproducible AAA build + manual upgrade docs</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -4347,17 +4347,17 @@
         </is>
       </c>
       <c r="E78" s="3" t="n">
-        <v>46400</v>
+        <v>46398</v>
       </c>
       <c r="F78" s="3" t="n">
-        <v>46401</v>
+        <v>46399</v>
       </c>
       <c r="G78" t="n">
         <v>2</v>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>T7.2</t>
+          <t>T3.6,T5.7</t>
         </is>
       </c>
       <c r="I78" s="4" t="n">
@@ -4375,7 +4375,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>T7.4</t>
+          <t>T7.7</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -4385,26 +4385,26 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Reproducible AAA build + manual upgrade docs</t>
+          <t>Prompt-injection test with reference agent</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>sonnet-5</t>
+          <t>opus-5.5 (high)</t>
         </is>
       </c>
       <c r="E79" s="3" t="n">
-        <v>46398</v>
+        <v>46400</v>
       </c>
       <c r="F79" s="3" t="n">
-        <v>46399</v>
+        <v>46400</v>
       </c>
       <c r="G79" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>T3.6,T5.7</t>
+          <t>T3.7,T4.7</t>
         </is>
       </c>
       <c r="I79" s="4" t="n">
@@ -4422,7 +4422,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>T7.7</t>
+          <t>T7.9</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -4432,26 +4432,26 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Prompt-injection test with reference agent</t>
+          <t>Traceability audit + coverage gates to thresholds</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>opus-5.5 (high)</t>
+          <t>haiku-4.5</t>
         </is>
       </c>
       <c r="E80" s="3" t="n">
-        <v>46400</v>
+        <v>46401</v>
       </c>
       <c r="F80" s="3" t="n">
-        <v>46400</v>
+        <v>46402</v>
       </c>
       <c r="G80" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>T3.7,T4.7</t>
+          <t>T7.1</t>
         </is>
       </c>
       <c r="I80" s="4" t="n">
@@ -4469,7 +4469,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>T7.9</t>
+          <t>T7.10</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -4479,7 +4479,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Traceability audit + coverage gates to thresholds</t>
+          <t>Practice set + open data release tooling</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -4488,17 +4488,17 @@
         </is>
       </c>
       <c r="E81" s="3" t="n">
-        <v>46401</v>
+        <v>46402</v>
       </c>
       <c r="F81" s="3" t="n">
-        <v>46402</v>
+        <v>46405</v>
       </c>
       <c r="G81" t="n">
         <v>2</v>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>T7.1</t>
+          <t>T1.7,T4.8</t>
         </is>
       </c>
       <c r="I81" s="4" t="n">
@@ -4516,7 +4516,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>T7.10</t>
+          <t>T7.5</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -4526,26 +4526,26 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Practice set + open data release tooling</t>
+          <t>External security review (payments + platform)</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>haiku-4.5</t>
+          <t>human</t>
         </is>
       </c>
       <c r="E82" s="3" t="n">
-        <v>46402</v>
+        <v>46373</v>
       </c>
       <c r="F82" s="3" t="n">
-        <v>46405</v>
+        <v>46379</v>
       </c>
       <c r="G82" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>T1.7,T4.8</t>
+          <t>T5.7,T4.8</t>
         </is>
       </c>
       <c r="I82" s="4" t="n">
@@ -4563,36 +4563,36 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
+          <t>T7.6</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Fix security findings</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>opus-5.5 (high)</t>
+        </is>
+      </c>
+      <c r="E83" s="3" t="n">
+        <v>46405</v>
+      </c>
+      <c r="F83" s="3" t="n">
+        <v>46407</v>
+      </c>
+      <c r="G83" t="n">
+        <v>3</v>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
           <t>T7.5</t>
-        </is>
-      </c>
-      <c r="B83" t="inlineStr">
-        <is>
-          <t>P7</t>
-        </is>
-      </c>
-      <c r="C83" t="inlineStr">
-        <is>
-          <t>External security review (payments + platform)</t>
-        </is>
-      </c>
-      <c r="D83" t="inlineStr">
-        <is>
-          <t>human</t>
-        </is>
-      </c>
-      <c r="E83" s="3" t="n">
-        <v>46373</v>
-      </c>
-      <c r="F83" s="3" t="n">
-        <v>46379</v>
-      </c>
-      <c r="G83" t="n">
-        <v>5</v>
-      </c>
-      <c r="H83" t="inlineStr">
-        <is>
-          <t>T5.7,T4.8</t>
         </is>
       </c>
       <c r="I83" s="4" t="n">
@@ -4610,7 +4610,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>T7.6</t>
+          <t>T7.11</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -4620,26 +4620,26 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Fix security findings</t>
+          <t>Continuous data refresh: 15-day scheduled job (n…</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>opus-5.5 (high)</t>
+          <t>sonnet-5</t>
         </is>
       </c>
       <c r="E84" s="3" t="n">
-        <v>46405</v>
+        <v>46406</v>
       </c>
       <c r="F84" s="3" t="n">
         <v>46407</v>
       </c>
       <c r="G84" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>T7.5</t>
+          <t>T1.7,T2.3,T8.14</t>
         </is>
       </c>
       <c r="I84" s="4" t="n">
@@ -4657,36 +4657,36 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>T7.11</t>
+          <t>T8.14</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>P7</t>
+          <t>P8</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Continuous data refresh: 15-day scheduled job (n…</t>
+          <t>Create Cloudflare R2 bucket + API token + custom…</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>sonnet-5</t>
+          <t>human</t>
         </is>
       </c>
       <c r="E85" s="3" t="n">
-        <v>46406</v>
+        <v>46316</v>
       </c>
       <c r="F85" s="3" t="n">
-        <v>46407</v>
+        <v>46316</v>
       </c>
       <c r="G85" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>T1.7,T2.3,T8.14</t>
+          <t>T1.7</t>
         </is>
       </c>
       <c r="I85" s="4" t="n">
@@ -4704,36 +4704,36 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
+          <t>T8.16</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>P8</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Scale dataset to 20,000 subjects (R-62) and publ…</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>haiku-4.5</t>
+        </is>
+      </c>
+      <c r="E86" s="3" t="n">
+        <v>46406</v>
+      </c>
+      <c r="F86" s="3" t="n">
+        <v>46406</v>
+      </c>
+      <c r="G86" t="n">
+        <v>1</v>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
           <t>T8.14</t>
-        </is>
-      </c>
-      <c r="B86" t="inlineStr">
-        <is>
-          <t>P8</t>
-        </is>
-      </c>
-      <c r="C86" t="inlineStr">
-        <is>
-          <t>Create Cloudflare R2 bucket + API token + custom…</t>
-        </is>
-      </c>
-      <c r="D86" t="inlineStr">
-        <is>
-          <t>human</t>
-        </is>
-      </c>
-      <c r="E86" s="3" t="n">
-        <v>46316</v>
-      </c>
-      <c r="F86" s="3" t="n">
-        <v>46316</v>
-      </c>
-      <c r="G86" t="n">
-        <v>1</v>
-      </c>
-      <c r="H86" t="inlineStr">
-        <is>
-          <t>T1.7</t>
         </is>
       </c>
       <c r="I86" s="4" t="n">
@@ -4751,7 +4751,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>T8.16</t>
+          <t>T8.1</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -4761,26 +4761,26 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Scale dataset to 20,000 subjects (R-62) and publ…</t>
+          <t>Staging deploy, deploy workflow, snapshots, cycl…</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>haiku-4.5</t>
+          <t>sonnet-5</t>
         </is>
       </c>
       <c r="E87" s="3" t="n">
-        <v>46406</v>
+        <v>46407</v>
       </c>
       <c r="F87" s="3" t="n">
-        <v>46406</v>
+        <v>46408</v>
       </c>
       <c r="G87" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>T8.14</t>
+          <t>T7.1</t>
         </is>
       </c>
       <c r="I87" s="4" t="n">
@@ -4798,7 +4798,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>T8.1</t>
+          <t>T8.2</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -4808,26 +4808,26 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Staging deploy, deploy workflow, snapshots, cycl…</t>
+          <t>Upload subjects/protocol/honeypots to staging</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>sonnet-5</t>
+          <t>haiku-4.5</t>
         </is>
       </c>
       <c r="E88" s="3" t="n">
-        <v>46407</v>
+        <v>46409</v>
       </c>
       <c r="F88" s="3" t="n">
-        <v>46408</v>
+        <v>46409</v>
       </c>
       <c r="G88" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>T7.1</t>
+          <t>T8.16,T8.1,T7.6</t>
         </is>
       </c>
       <c r="I88" s="4" t="n">
@@ -4845,7 +4845,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>T8.2</t>
+          <t>T8.5</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -4855,26 +4855,26 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Upload subjects/protocol/honeypots to staging</t>
+          <t>Fund prod treasury with ICP float (10–20 ICP) + …</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>haiku-4.5</t>
+          <t>human</t>
         </is>
       </c>
       <c r="E89" s="3" t="n">
-        <v>46409</v>
+        <v>46428</v>
       </c>
       <c r="F89" s="3" t="n">
-        <v>46409</v>
+        <v>46428</v>
       </c>
       <c r="G89" t="n">
         <v>1</v>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>T8.16,T8.1,T7.6</t>
+          <t>T8.6</t>
         </is>
       </c>
       <c r="I89" s="4" t="n">
@@ -4892,7 +4892,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>T8.5</t>
+          <t>T8.3</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -4902,7 +4902,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Fund prod treasury with ICP float (10–20 ICP) + …</t>
+          <t>Closed beta (10-20 owners)</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -4911,17 +4911,17 @@
         </is>
       </c>
       <c r="E90" s="3" t="n">
-        <v>46428</v>
+        <v>46412</v>
       </c>
       <c r="F90" s="3" t="n">
-        <v>46428</v>
+        <v>46423</v>
       </c>
       <c r="G90" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>T8.6</t>
+          <t>T8.2,T6.10</t>
         </is>
       </c>
       <c r="I90" s="4" t="n">
@@ -4939,7 +4939,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>T8.3</t>
+          <t>T8.4</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -4949,12 +4949,12 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Closed beta (10-20 owners)</t>
+          <t>Beta fixes &amp; tuning</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>human</t>
+          <t>sonnet-5</t>
         </is>
       </c>
       <c r="E91" s="3" t="n">
@@ -4986,7 +4986,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>T8.4</t>
+          <t>T8.6</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -4996,7 +4996,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Beta fixes &amp; tuning</t>
+          <t>Production deploy, II metadata, treasury watch l…</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -5005,17 +5005,17 @@
         </is>
       </c>
       <c r="E92" s="3" t="n">
-        <v>46412</v>
+        <v>46426</v>
       </c>
       <c r="F92" s="3" t="n">
-        <v>46423</v>
+        <v>46427</v>
       </c>
       <c r="G92" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>T8.2,T6.10</t>
+          <t>T8.3,T8.4,T8.13</t>
         </is>
       </c>
       <c r="I92" s="4" t="n">
@@ -5033,7 +5033,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>T8.6</t>
+          <t>T8.7</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -5043,26 +5043,26 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Production deploy, II metadata, treasury watch l…</t>
+          <t>Public launch</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>sonnet-5</t>
+          <t>human</t>
         </is>
       </c>
       <c r="E93" s="3" t="n">
-        <v>46426</v>
+        <v>46429</v>
       </c>
       <c r="F93" s="3" t="n">
-        <v>46427</v>
+        <v>46429</v>
       </c>
       <c r="G93" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>T8.3,T8.4,T8.13</t>
+          <t>T8.6,T8.5,T9.5</t>
         </is>
       </c>
       <c r="I93" s="4" t="n">
@@ -5080,36 +5080,36 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>T8.7</t>
+          <t>T9.1</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>P8</t>
+          <t>P9</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Public launch</t>
+          <t>Import mockups (Claude Design), reconcile, desig…</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>human</t>
+          <t>sonnet-5</t>
         </is>
       </c>
       <c r="E94" s="3" t="n">
-        <v>46429</v>
+        <v>46408</v>
       </c>
       <c r="F94" s="3" t="n">
-        <v>46429</v>
+        <v>46413</v>
       </c>
       <c r="G94" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>T8.6,T8.5,T9.5</t>
+          <t>T6.10</t>
         </is>
       </c>
       <c r="I94" s="4" t="n">
@@ -5127,7 +5127,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>T9.1</t>
+          <t>T9.2</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -5137,7 +5137,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Import mockups (Claude Design), reconcile, desig…</t>
+          <t>Style public pages: landing, museum, discovery, …</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -5146,17 +5146,17 @@
         </is>
       </c>
       <c r="E95" s="3" t="n">
-        <v>46408</v>
+        <v>46414</v>
       </c>
       <c r="F95" s="3" t="n">
-        <v>46413</v>
+        <v>46419</v>
       </c>
       <c r="G95" t="n">
         <v>4</v>
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>T6.10</t>
+          <t>T9.1</t>
         </is>
       </c>
       <c r="I95" s="4" t="n">
@@ -5174,7 +5174,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>T9.2</t>
+          <t>T9.3</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -5184,7 +5184,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Style public pages: landing, museum, discovery, …</t>
+          <t>Style owner flows: spawn, dashboard, connect age…</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -5221,7 +5221,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>T9.3</t>
+          <t>T9.4</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -5231,22 +5231,22 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Style owner flows: spawn, dashboard, connect age…</t>
+          <t>Style admin console + about/legal/practice pages</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>sonnet-5</t>
+          <t>haiku-4.5</t>
         </is>
       </c>
       <c r="E97" s="3" t="n">
-        <v>46414</v>
+        <v>46420</v>
       </c>
       <c r="F97" s="3" t="n">
-        <v>46419</v>
+        <v>46421</v>
       </c>
       <c r="G97" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H97" t="inlineStr">
         <is>
@@ -5268,7 +5268,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>T9.4</t>
+          <t>T9.5</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -5278,7 +5278,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Style admin console + about/legal/practice pages</t>
+          <t>Responsive/mobile pass, visual-regression baseli…</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -5287,17 +5287,17 @@
         </is>
       </c>
       <c r="E98" s="3" t="n">
-        <v>46420</v>
+        <v>46422</v>
       </c>
       <c r="F98" s="3" t="n">
-        <v>46421</v>
+        <v>46423</v>
       </c>
       <c r="G98" t="n">
         <v>2</v>
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>T9.1</t>
+          <t>T9.2,T9.3,T9.4</t>
         </is>
       </c>
       <c r="I98" s="4" t="n">
@@ -5315,36 +5315,36 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>T9.5</t>
+          <t>T8.13</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>P9</t>
+          <t>P8</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Responsive/mobile pass, visual-regression baseli…</t>
+          <t>Custom domain + II alternative origins</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>haiku-4.5</t>
+          <t>human</t>
         </is>
       </c>
       <c r="E99" s="3" t="n">
-        <v>46422</v>
+        <v>46409</v>
       </c>
       <c r="F99" s="3" t="n">
-        <v>46423</v>
+        <v>46409</v>
       </c>
       <c r="G99" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>T9.2,T9.3,T9.4</t>
+          <t>T8.1</t>
         </is>
       </c>
       <c r="I99" s="4" t="n">
@@ -5362,7 +5362,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>T8.13</t>
+          <t>T8.15</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -5372,7 +5372,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Custom domain + II alternative origins</t>
+          <t>Owner review: discovery + peer-review agent proc…</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -5381,17 +5381,17 @@
         </is>
       </c>
       <c r="E100" s="3" t="n">
-        <v>46409</v>
+        <v>46296</v>
       </c>
       <c r="F100" s="3" t="n">
-        <v>46409</v>
+        <v>46296</v>
       </c>
       <c r="G100" t="n">
         <v>1</v>
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>T8.1</t>
+          <t>T0.4</t>
         </is>
       </c>
       <c r="I100" s="4" t="n">
@@ -5409,7 +5409,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>T8.12</t>
+          <t>T8.8</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -5419,7 +5419,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Firebase projects (staging/prod) + GA4 funnels &amp;…</t>
+          <t>Compliance check for crypto fuel packs (recommen…</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -5431,10 +5431,10 @@
         <v>46296</v>
       </c>
       <c r="F101" s="3" t="n">
-        <v>46296</v>
+        <v>46302</v>
       </c>
       <c r="G101" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H101" t="inlineStr">
         <is>
@@ -5456,7 +5456,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>T8.15</t>
+          <t>T8.9</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -5466,7 +5466,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Owner review: discovery + peer-review agent proc…</t>
+          <t>Enable BTC/ETH on production</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -5475,17 +5475,17 @@
         </is>
       </c>
       <c r="E102" s="3" t="n">
-        <v>46296</v>
+        <v>46428</v>
       </c>
       <c r="F102" s="3" t="n">
-        <v>46296</v>
+        <v>46428</v>
       </c>
       <c r="G102" t="n">
         <v>1</v>
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>T0.4</t>
+          <t>T8.6,T8.8</t>
         </is>
       </c>
       <c r="I102" s="4" t="n">
@@ -5500,102 +5500,8 @@
         <v/>
       </c>
     </row>
-    <row r="103">
-      <c r="A103" t="inlineStr">
-        <is>
-          <t>T8.8</t>
-        </is>
-      </c>
-      <c r="B103" t="inlineStr">
-        <is>
-          <t>P8</t>
-        </is>
-      </c>
-      <c r="C103" t="inlineStr">
-        <is>
-          <t>Compliance check for crypto fuel packs (recommen…</t>
-        </is>
-      </c>
-      <c r="D103" t="inlineStr">
-        <is>
-          <t>human</t>
-        </is>
-      </c>
-      <c r="E103" s="3" t="n">
-        <v>46296</v>
-      </c>
-      <c r="F103" s="3" t="n">
-        <v>46302</v>
-      </c>
-      <c r="G103" t="n">
-        <v>5</v>
-      </c>
-      <c r="H103" t="inlineStr">
-        <is>
-          <t>T0.4</t>
-        </is>
-      </c>
-      <c r="I103" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J103">
-        <f>IF(I103&gt;=1,"Done",IF(TODAY()&gt;F103,"Late",IF(I103&gt;0,"In progress","Not started")))</f>
-        <v/>
-      </c>
-      <c r="K103">
-        <f>G103*I103</f>
-        <v/>
-      </c>
-    </row>
-    <row r="104">
-      <c r="A104" t="inlineStr">
-        <is>
-          <t>T8.9</t>
-        </is>
-      </c>
-      <c r="B104" t="inlineStr">
-        <is>
-          <t>P8</t>
-        </is>
-      </c>
-      <c r="C104" t="inlineStr">
-        <is>
-          <t>Enable BTC/ETH on production</t>
-        </is>
-      </c>
-      <c r="D104" t="inlineStr">
-        <is>
-          <t>human</t>
-        </is>
-      </c>
-      <c r="E104" s="3" t="n">
-        <v>46428</v>
-      </c>
-      <c r="F104" s="3" t="n">
-        <v>46428</v>
-      </c>
-      <c r="G104" t="n">
-        <v>1</v>
-      </c>
-      <c r="H104" t="inlineStr">
-        <is>
-          <t>T8.6,T8.8</t>
-        </is>
-      </c>
-      <c r="I104" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J104">
-        <f>IF(I104&gt;=1,"Done",IF(TODAY()&gt;F104,"Late",IF(I104&gt;0,"In progress","Not started")))</f>
-        <v/>
-      </c>
-      <c r="K104">
-        <f>G104*I104</f>
-        <v/>
-      </c>
-    </row>
   </sheetData>
-  <conditionalFormatting sqref="L2:AF104">
+  <conditionalFormatting sqref="L2:AF102">
     <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="1">
       <formula>AND(L$1+6&gt;=$E2,L$1&lt;=$F2,L$1&lt;=$E2+($F2-$E2)*$I2)</formula>
     </cfRule>
@@ -5633,7 +5539,7 @@
       <formula>AND(TODAY()&gt;=L$1,TODAY()&lt;L$1+7)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J2:J104">
+  <conditionalFormatting sqref="J2:J102">
     <cfRule type="expression" priority="13" dxfId="12">
       <formula>LEFT(J2,4)="Late"</formula>
     </cfRule>
@@ -6164,7 +6070,7 @@
         <v/>
       </c>
       <c r="G12" s="17">
-        <f>IF(C12&gt;0,SUM(Gantt!K2:K104)/C12,0)</f>
+        <f>IF(C12&gt;0,SUM(Gantt!K2:K102)/C12,0)</f>
         <v/>
       </c>
       <c r="H12" s="18" t="n">

</xml_diff>

<commit_message>
plan: ICP-only payments for MVP - defer ckBTC/ckETH (T5.8-T5.10,T5.13,T6.11,T8.8-T8.9 -> D6-D12)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/space-compute-gantt-v3.xlsx
+++ b/docs/space-compute-gantt-v3.xlsx
@@ -600,7 +600,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF102"/>
+  <dimension ref="A1:AE95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -634,7 +634,6 @@
     <col width="3.2" customWidth="1" min="29" max="29"/>
     <col width="3.2" customWidth="1" min="30" max="30"/>
     <col width="3.2" customWidth="1" min="31" max="31"/>
-    <col width="3.2" customWidth="1" min="32" max="32"/>
   </cols>
   <sheetData>
     <row r="1" ht="48" customHeight="1">
@@ -753,9 +752,6 @@
       <c r="AE1" s="2" t="n">
         <v>46419</v>
       </c>
-      <c r="AF1" s="2" t="n">
-        <v>46426</v>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3200,7 +3196,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>T5.8</t>
+          <t>T5.15</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -3210,26 +3206,26 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>XRC rates, fuel treasury guard rails + auto inta…</t>
+          <t>Payments admin APIs (audit log exists since T5.1)</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>opus-5.5 (high)</t>
+          <t>haiku-4.5</t>
         </is>
       </c>
       <c r="E54" s="3" t="n">
         <v>46358</v>
       </c>
       <c r="F54" s="3" t="n">
-        <v>46363</v>
+        <v>46358</v>
       </c>
       <c r="G54" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>T5.2</t>
+          <t>T5.1</t>
         </is>
       </c>
       <c r="I54" s="4" t="n">
@@ -3247,7 +3243,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>T5.9</t>
+          <t>T5.16</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -3257,26 +3253,26 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>ckBTC fuel-pack deposits (address, update_balanc…</t>
+          <t>Feature flags + invite codes (sponsored spawn)</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>opus-5.5 (high)</t>
+          <t>sonnet-5</t>
         </is>
       </c>
       <c r="E55" s="3" t="n">
-        <v>46364</v>
+        <v>46358</v>
       </c>
       <c r="F55" s="3" t="n">
-        <v>46366</v>
+        <v>46359</v>
       </c>
       <c r="G55" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>T5.8</t>
+          <t>T5.3</t>
         </is>
       </c>
       <c r="I55" s="4" t="n">
@@ -3294,7 +3290,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>T5.10</t>
+          <t>T5.17</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -3304,30 +3300,30 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>ckETH fuel-pack deposits</t>
+          <t>treasury canister: owner-funded reserve, cycles …</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>sonnet-5</t>
+          <t>opus-5.5 (high)</t>
         </is>
       </c>
       <c r="E56" s="3" t="n">
-        <v>46364</v>
+        <v>46359</v>
       </c>
       <c r="F56" s="3" t="n">
-        <v>46365</v>
+        <v>46363</v>
       </c>
       <c r="G56" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>T5.8,SP-6</t>
+          <t>T2.1,T1.4</t>
         </is>
       </c>
       <c r="I56" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J56">
         <f>IF(I56&gt;=1,"Done",IF(TODAY()&gt;F56,"Late",IF(I56&gt;0,"In progress","Not started")))</f>
@@ -3341,7 +3337,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>T5.13</t>
+          <t>T5.18</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -3351,7 +3347,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Non-ICP payment tests (04 §6.7)</t>
+          <t>treasury PocketIC tests (ICP ledger + CMC, no NN…</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -3360,21 +3356,21 @@
         </is>
       </c>
       <c r="E57" s="3" t="n">
-        <v>46367</v>
+        <v>46364</v>
       </c>
       <c r="F57" s="3" t="n">
-        <v>46370</v>
+        <v>46364</v>
       </c>
       <c r="G57" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>T5.9,T5.10</t>
+          <t>T5.17</t>
         </is>
       </c>
       <c r="I57" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J57">
         <f>IF(I57&gt;=1,"Done",IF(TODAY()&gt;F57,"Late",IF(I57&gt;0,"In progress","Not started")))</f>
@@ -3388,7 +3384,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>T5.15</t>
+          <t>T5.7</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -3398,26 +3394,26 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Payments admin APIs (audit log exists since T5.1)</t>
+          <t>Internal payments security review</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>haiku-4.5</t>
+          <t>opus-5.5 (high)</t>
         </is>
       </c>
       <c r="E58" s="3" t="n">
-        <v>46371</v>
+        <v>46360</v>
       </c>
       <c r="F58" s="3" t="n">
-        <v>46371</v>
+        <v>46363</v>
       </c>
       <c r="G58" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>T5.13</t>
+          <t>T5.6,T5.16</t>
         </is>
       </c>
       <c r="I58" s="4" t="n">
@@ -3435,17 +3431,17 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>T5.16</t>
+          <t>T6.1</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>P5</t>
+          <t>P6</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Feature flags + invite codes (sponsored spawn)</t>
+          <t>App scaffold: routing, bindgen, II auth, ic_env,…</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -3457,18 +3453,18 @@
         <v>46360</v>
       </c>
       <c r="F59" s="3" t="n">
-        <v>46363</v>
+        <v>46364</v>
       </c>
       <c r="G59" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>T5.3</t>
+          <t>T1.1</t>
         </is>
       </c>
       <c r="I59" s="4" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="J59">
         <f>IF(I59&gt;=1,"Done",IF(TODAY()&gt;F59,"Late",IF(I59&gt;0,"In progress","Not started")))</f>
@@ -3482,40 +3478,40 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>T5.17</t>
+          <t>T6.3</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>P5</t>
+          <t>P6</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>treasury canister: owner-funded reserve, cycles …</t>
+          <t>Landing, Discovery Museum feed, Discovery detail…</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>opus-5.5 (high)</t>
+          <t>sonnet-5</t>
         </is>
       </c>
       <c r="E60" s="3" t="n">
-        <v>46364</v>
+        <v>46365</v>
       </c>
       <c r="F60" s="3" t="n">
-        <v>46366</v>
+        <v>46371</v>
       </c>
       <c r="G60" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>T2.1,T1.4</t>
+          <t>T6.1</t>
         </is>
       </c>
       <c r="I60" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J60">
         <f>IF(I60&gt;=1,"Done",IF(TODAY()&gt;F60,"Late",IF(I60&gt;0,"In progress","Not started")))</f>
@@ -3529,40 +3525,40 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>T5.18</t>
+          <t>T6.4</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>P5</t>
+          <t>P6</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>treasury PocketIC tests (ICP ledger + CMC, no NN…</t>
+          <t>AAA profile + Leaderboard</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>sonnet-5</t>
+          <t>haiku-4.5</t>
         </is>
       </c>
       <c r="E61" s="3" t="n">
-        <v>46367</v>
+        <v>46372</v>
       </c>
       <c r="F61" s="3" t="n">
-        <v>46367</v>
+        <v>46374</v>
       </c>
       <c r="G61" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>T5.17</t>
+          <t>T6.3</t>
         </is>
       </c>
       <c r="I61" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J61">
         <f>IF(I61&gt;=1,"Done",IF(TODAY()&gt;F61,"Late",IF(I61&gt;0,"In progress","Not started")))</f>
@@ -3576,36 +3572,36 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>T5.7</t>
+          <t>T6.5</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>P5</t>
+          <t>P6</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Internal payments security review</t>
+          <t>Payment component (wallet + deposit)</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>opus-5.5 (high)</t>
+          <t>sonnet-5</t>
         </is>
       </c>
       <c r="E62" s="3" t="n">
-        <v>46371</v>
+        <v>46365</v>
       </c>
       <c r="F62" s="3" t="n">
-        <v>46372</v>
+        <v>46370</v>
       </c>
       <c r="G62" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>T5.6,T5.13,T5.16</t>
+          <t>T6.1,SP-2,T5.4</t>
         </is>
       </c>
       <c r="I62" s="4" t="n">
@@ -3623,7 +3619,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>T6.1</t>
+          <t>T6.6</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -3633,30 +3629,30 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>App scaffold: routing, bindgen, II auth, ic_env,…</t>
+          <t>Spawn flow</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>sonnet-5</t>
+          <t>haiku-4.5</t>
         </is>
       </c>
       <c r="E63" s="3" t="n">
-        <v>46367</v>
+        <v>46371</v>
       </c>
       <c r="F63" s="3" t="n">
-        <v>46371</v>
+        <v>46372</v>
       </c>
       <c r="G63" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>T1.1</t>
+          <t>T6.5,T5.3</t>
         </is>
       </c>
       <c r="I63" s="4" t="n">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="J63">
         <f>IF(I63&gt;=1,"Done",IF(TODAY()&gt;F63,"Late",IF(I63&gt;0,"In progress","Not started")))</f>
@@ -3670,7 +3666,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>T6.3</t>
+          <t>T6.7</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -3680,7 +3676,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Landing, Discovery Museum feed, Discovery detail…</t>
+          <t>Owner dashboard</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -3689,17 +3685,17 @@
         </is>
       </c>
       <c r="E64" s="3" t="n">
-        <v>46372</v>
+        <v>46365</v>
       </c>
       <c r="F64" s="3" t="n">
-        <v>46378</v>
+        <v>46370</v>
       </c>
       <c r="G64" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>T6.1</t>
+          <t>T6.1,T3.3,T4.6</t>
         </is>
       </c>
       <c r="I64" s="4" t="n">
@@ -3717,7 +3713,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>T6.4</t>
+          <t>T6.8</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -3727,7 +3723,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>AAA profile + Leaderboard</t>
+          <t>Connect your agent + Activity &amp; records</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -3736,17 +3732,17 @@
         </is>
       </c>
       <c r="E65" s="3" t="n">
-        <v>46379</v>
+        <v>46371</v>
       </c>
       <c r="F65" s="3" t="n">
-        <v>46385</v>
+        <v>46373</v>
       </c>
       <c r="G65" t="n">
         <v>3</v>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>T6.3</t>
+          <t>T6.7</t>
         </is>
       </c>
       <c r="I65" s="4" t="n">
@@ -3764,7 +3760,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>T6.5</t>
+          <t>T6.9</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -3774,26 +3770,26 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Payment component (wallet + deposit)</t>
+          <t>Fuel &amp; billing + auto top-up</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>sonnet-5</t>
+          <t>haiku-4.5</t>
         </is>
       </c>
       <c r="E66" s="3" t="n">
-        <v>46372</v>
+        <v>46373</v>
       </c>
       <c r="F66" s="3" t="n">
         <v>46377</v>
       </c>
       <c r="G66" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>T6.1,SP-2,T5.4</t>
+          <t>T6.5,T5.5</t>
         </is>
       </c>
       <c r="I66" s="4" t="n">
@@ -3811,7 +3807,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>T6.6</t>
+          <t>T6.12</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -3821,26 +3817,26 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Spawn flow</t>
+          <t>Admin console (8 screens)</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>haiku-4.5</t>
+          <t>sonnet-5</t>
         </is>
       </c>
       <c r="E67" s="3" t="n">
-        <v>46378</v>
+        <v>46374</v>
       </c>
       <c r="F67" s="3" t="n">
-        <v>46379</v>
+        <v>46384</v>
       </c>
       <c r="G67" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>T6.5,T5.3</t>
+          <t>T6.1,T4.10,T5.15</t>
         </is>
       </c>
       <c r="I67" s="4" t="n">
@@ -3858,7 +3854,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>T6.7</t>
+          <t>T6.14</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -3868,26 +3864,26 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Owner dashboard</t>
+          <t>About/legal/practice pages, invite spawn UI, adm…</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>sonnet-5</t>
+          <t>haiku-4.5</t>
         </is>
       </c>
       <c r="E68" s="3" t="n">
-        <v>46378</v>
+        <v>46385</v>
       </c>
       <c r="F68" s="3" t="n">
-        <v>46385</v>
+        <v>46391</v>
       </c>
       <c r="G68" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>T6.1,T3.3,T4.6</t>
+          <t>T6.12,T5.16,T5.18</t>
         </is>
       </c>
       <c r="I68" s="4" t="n">
@@ -3905,7 +3901,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>T6.8</t>
+          <t>T6.10</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -3915,26 +3911,26 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Connect your agent + Activity &amp; records</t>
+          <t>States, accessibility, Playwright smoke</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>haiku-4.5</t>
+          <t>sonnet-5</t>
         </is>
       </c>
       <c r="E69" s="3" t="n">
-        <v>46386</v>
+        <v>46392</v>
       </c>
       <c r="F69" s="3" t="n">
-        <v>46392</v>
+        <v>46394</v>
       </c>
       <c r="G69" t="n">
         <v>3</v>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>T6.7</t>
+          <t>T6.4,T6.6,T6.8,T6.9,T6.12,T6.14</t>
         </is>
       </c>
       <c r="I69" s="4" t="n">
@@ -3952,36 +3948,36 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>T6.9</t>
+          <t>T7.1</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>P6</t>
+          <t>P7</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Fuel &amp; billing + auto top-up</t>
+          <t>Upgrade tests for all canisters</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>haiku-4.5</t>
+          <t>sonnet-5</t>
         </is>
       </c>
       <c r="E70" s="3" t="n">
-        <v>46384</v>
+        <v>46378</v>
       </c>
       <c r="F70" s="3" t="n">
-        <v>46386</v>
+        <v>46379</v>
       </c>
       <c r="G70" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>T6.5,T5.5</t>
+          <t>T4.8,T5.6</t>
         </is>
       </c>
       <c r="I70" s="4" t="n">
@@ -3999,17 +3995,17 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>T6.11</t>
+          <t>T7.2</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>P6</t>
+          <t>P7</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>BTC &amp; ETH methods + feature-flag gating</t>
+          <t>Load test: 200 AAAs × 100 tasks</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -4018,17 +4014,17 @@
         </is>
       </c>
       <c r="E71" s="3" t="n">
-        <v>46386</v>
+        <v>46384</v>
       </c>
       <c r="F71" s="3" t="n">
-        <v>46393</v>
+        <v>46385</v>
       </c>
       <c r="G71" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>T6.5,T5.9,T5.10</t>
+          <t>T7.1</t>
         </is>
       </c>
       <c r="I71" s="4" t="n">
@@ -4046,17 +4042,17 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>T6.12</t>
+          <t>T7.3</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>P6</t>
+          <t>P7</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Admin console (8 screens)</t>
+          <t>Cycle cost measurement &amp; fee retune</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -4065,17 +4061,17 @@
         </is>
       </c>
       <c r="E72" s="3" t="n">
+        <v>46386</v>
+      </c>
+      <c r="F72" s="3" t="n">
         <v>46391</v>
       </c>
-      <c r="F72" s="3" t="n">
-        <v>46395</v>
-      </c>
       <c r="G72" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>T6.1,T4.10,T5.15</t>
+          <t>T7.2</t>
         </is>
       </c>
       <c r="I72" s="4" t="n">
@@ -4093,36 +4089,36 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>T6.14</t>
+          <t>T7.4</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>P6</t>
+          <t>P7</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>About/legal/practice pages, invite spawn UI, adm…</t>
+          <t>Reproducible AAA build + manual upgrade docs</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>haiku-4.5</t>
+          <t>sonnet-5</t>
         </is>
       </c>
       <c r="E73" s="3" t="n">
-        <v>46398</v>
+        <v>46385</v>
       </c>
       <c r="F73" s="3" t="n">
-        <v>46400</v>
+        <v>46386</v>
       </c>
       <c r="G73" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>T6.12,T5.16,T5.18</t>
+          <t>T3.6,T5.7</t>
         </is>
       </c>
       <c r="I73" s="4" t="n">
@@ -4140,36 +4136,36 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>T6.10</t>
+          <t>T7.7</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>P6</t>
+          <t>P7</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>States, accessibility, Playwright smoke</t>
+          <t>Prompt-injection test with reference agent</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>sonnet-5</t>
+          <t>opus-5.5 (high)</t>
         </is>
       </c>
       <c r="E74" s="3" t="n">
-        <v>46401</v>
+        <v>46391</v>
       </c>
       <c r="F74" s="3" t="n">
-        <v>46405</v>
+        <v>46391</v>
       </c>
       <c r="G74" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>T6.4,T6.6,T6.8,T6.9,T6.11,T6.12,T6.14</t>
+          <t>T3.7,T4.7</t>
         </is>
       </c>
       <c r="I74" s="4" t="n">
@@ -4187,7 +4183,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>T7.1</t>
+          <t>T7.9</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -4197,26 +4193,26 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Upgrade tests for all canisters</t>
+          <t>Traceability audit + coverage gates to thresholds</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>sonnet-5</t>
+          <t>haiku-4.5</t>
         </is>
       </c>
       <c r="E75" s="3" t="n">
-        <v>46394</v>
+        <v>46392</v>
       </c>
       <c r="F75" s="3" t="n">
-        <v>46395</v>
+        <v>46393</v>
       </c>
       <c r="G75" t="n">
         <v>2</v>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>T4.8,T5.6</t>
+          <t>T7.1</t>
         </is>
       </c>
       <c r="I75" s="4" t="n">
@@ -4234,7 +4230,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>T7.2</t>
+          <t>T7.10</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -4244,26 +4240,26 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Load test: 200 AAAs × 100 tasks</t>
+          <t>Practice set + open data release tooling</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>sonnet-5</t>
+          <t>haiku-4.5</t>
         </is>
       </c>
       <c r="E76" s="3" t="n">
-        <v>46398</v>
+        <v>46392</v>
       </c>
       <c r="F76" s="3" t="n">
-        <v>46399</v>
+        <v>46393</v>
       </c>
       <c r="G76" t="n">
         <v>2</v>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>T7.1</t>
+          <t>T1.7,T4.8</t>
         </is>
       </c>
       <c r="I76" s="4" t="n">
@@ -4281,7 +4277,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>T7.3</t>
+          <t>T7.5</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -4291,26 +4287,26 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Cycle cost measurement &amp; fee retune</t>
+          <t>External security review (payments + platform)</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>sonnet-5</t>
+          <t>human</t>
         </is>
       </c>
       <c r="E77" s="3" t="n">
-        <v>46400</v>
+        <v>46364</v>
       </c>
       <c r="F77" s="3" t="n">
-        <v>46401</v>
+        <v>46370</v>
       </c>
       <c r="G77" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>T7.2</t>
+          <t>T5.7,T4.8</t>
         </is>
       </c>
       <c r="I77" s="4" t="n">
@@ -4328,7 +4324,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>T7.4</t>
+          <t>T7.6</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -4338,26 +4334,26 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Reproducible AAA build + manual upgrade docs</t>
+          <t>Fix security findings</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>sonnet-5</t>
+          <t>opus-5.5 (high)</t>
         </is>
       </c>
       <c r="E78" s="3" t="n">
+        <v>46394</v>
+      </c>
+      <c r="F78" s="3" t="n">
         <v>46398</v>
       </c>
-      <c r="F78" s="3" t="n">
-        <v>46399</v>
-      </c>
       <c r="G78" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>T3.6,T5.7</t>
+          <t>T7.5</t>
         </is>
       </c>
       <c r="I78" s="4" t="n">
@@ -4375,7 +4371,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>T7.7</t>
+          <t>T7.11</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -4385,26 +4381,26 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Prompt-injection test with reference agent</t>
+          <t>Continuous data refresh: 15-day scheduled job (n…</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>opus-5.5 (high)</t>
+          <t>sonnet-5</t>
         </is>
       </c>
       <c r="E79" s="3" t="n">
-        <v>46400</v>
+        <v>46394</v>
       </c>
       <c r="F79" s="3" t="n">
-        <v>46400</v>
+        <v>46395</v>
       </c>
       <c r="G79" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>T3.7,T4.7</t>
+          <t>T1.7,T2.3,T8.14</t>
         </is>
       </c>
       <c r="I79" s="4" t="n">
@@ -4422,36 +4418,36 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>T7.9</t>
+          <t>T8.14</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>P7</t>
+          <t>P8</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Traceability audit + coverage gates to thresholds</t>
+          <t>Create Cloudflare R2 bucket + API token + custom…</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>haiku-4.5</t>
+          <t>human</t>
         </is>
       </c>
       <c r="E80" s="3" t="n">
-        <v>46401</v>
+        <v>46316</v>
       </c>
       <c r="F80" s="3" t="n">
-        <v>46402</v>
+        <v>46316</v>
       </c>
       <c r="G80" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>T7.1</t>
+          <t>T1.7</t>
         </is>
       </c>
       <c r="I80" s="4" t="n">
@@ -4469,17 +4465,17 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>T7.10</t>
+          <t>T8.16</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>P7</t>
+          <t>P8</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Practice set + open data release tooling</t>
+          <t>Scale dataset to 20,000 subjects (R-62) and publ…</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -4488,17 +4484,17 @@
         </is>
       </c>
       <c r="E81" s="3" t="n">
-        <v>46402</v>
+        <v>46395</v>
       </c>
       <c r="F81" s="3" t="n">
-        <v>46405</v>
+        <v>46395</v>
       </c>
       <c r="G81" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>T1.7,T4.8</t>
+          <t>T8.14</t>
         </is>
       </c>
       <c r="I81" s="4" t="n">
@@ -4516,36 +4512,36 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>T7.5</t>
+          <t>T8.1</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>P7</t>
+          <t>P8</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>External security review (payments + platform)</t>
+          <t>Staging deploy, deploy workflow, snapshots, cycl…</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>human</t>
+          <t>sonnet-5</t>
         </is>
       </c>
       <c r="E82" s="3" t="n">
-        <v>46373</v>
+        <v>46398</v>
       </c>
       <c r="F82" s="3" t="n">
-        <v>46379</v>
+        <v>46399</v>
       </c>
       <c r="G82" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>T5.7,T4.8</t>
+          <t>T7.1</t>
         </is>
       </c>
       <c r="I82" s="4" t="n">
@@ -4563,36 +4559,36 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>T7.6</t>
+          <t>T8.2</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>P7</t>
+          <t>P8</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Fix security findings</t>
+          <t>Upload subjects/protocol/honeypots to staging</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>opus-5.5 (high)</t>
+          <t>haiku-4.5</t>
         </is>
       </c>
       <c r="E83" s="3" t="n">
-        <v>46405</v>
+        <v>46400</v>
       </c>
       <c r="F83" s="3" t="n">
-        <v>46407</v>
+        <v>46400</v>
       </c>
       <c r="G83" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>T7.5</t>
+          <t>T8.16,T8.1,T7.6</t>
         </is>
       </c>
       <c r="I83" s="4" t="n">
@@ -4610,36 +4606,36 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>T7.11</t>
+          <t>T8.5</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>P7</t>
+          <t>P8</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Continuous data refresh: 15-day scheduled job (n…</t>
+          <t>Fund prod treasury with ICP float (10–20 ICP) + …</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>sonnet-5</t>
+          <t>human</t>
         </is>
       </c>
       <c r="E84" s="3" t="n">
-        <v>46406</v>
+        <v>46419</v>
       </c>
       <c r="F84" s="3" t="n">
-        <v>46407</v>
+        <v>46419</v>
       </c>
       <c r="G84" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>T1.7,T2.3,T8.14</t>
+          <t>T8.6</t>
         </is>
       </c>
       <c r="I84" s="4" t="n">
@@ -4657,7 +4653,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>T8.14</t>
+          <t>T8.3</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -4667,7 +4663,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Create Cloudflare R2 bucket + API token + custom…</t>
+          <t>Closed beta (10-20 owners)</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -4676,17 +4672,17 @@
         </is>
       </c>
       <c r="E85" s="3" t="n">
-        <v>46316</v>
+        <v>46401</v>
       </c>
       <c r="F85" s="3" t="n">
-        <v>46316</v>
+        <v>46414</v>
       </c>
       <c r="G85" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>T1.7</t>
+          <t>T8.2,T6.10</t>
         </is>
       </c>
       <c r="I85" s="4" t="n">
@@ -4704,7 +4700,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>T8.16</t>
+          <t>T8.4</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -4714,26 +4710,26 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Scale dataset to 20,000 subjects (R-62) and publ…</t>
+          <t>Beta fixes &amp; tuning</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>haiku-4.5</t>
+          <t>sonnet-5</t>
         </is>
       </c>
       <c r="E86" s="3" t="n">
-        <v>46406</v>
+        <v>46401</v>
       </c>
       <c r="F86" s="3" t="n">
-        <v>46406</v>
+        <v>46414</v>
       </c>
       <c r="G86" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>T8.14</t>
+          <t>T8.2,T6.10</t>
         </is>
       </c>
       <c r="I86" s="4" t="n">
@@ -4751,7 +4747,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>T8.1</t>
+          <t>T8.6</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -4761,7 +4757,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Staging deploy, deploy workflow, snapshots, cycl…</t>
+          <t>Production deploy, II metadata, treasury watch l…</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -4770,17 +4766,17 @@
         </is>
       </c>
       <c r="E87" s="3" t="n">
-        <v>46407</v>
+        <v>46415</v>
       </c>
       <c r="F87" s="3" t="n">
-        <v>46408</v>
+        <v>46416</v>
       </c>
       <c r="G87" t="n">
         <v>2</v>
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>T7.1</t>
+          <t>T8.3,T8.4,T8.13</t>
         </is>
       </c>
       <c r="I87" s="4" t="n">
@@ -4798,7 +4794,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>T8.2</t>
+          <t>T8.7</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -4808,26 +4804,26 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Upload subjects/protocol/honeypots to staging</t>
+          <t>Public launch</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>haiku-4.5</t>
+          <t>human</t>
         </is>
       </c>
       <c r="E88" s="3" t="n">
-        <v>46409</v>
+        <v>46420</v>
       </c>
       <c r="F88" s="3" t="n">
-        <v>46409</v>
+        <v>46420</v>
       </c>
       <c r="G88" t="n">
         <v>1</v>
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>T8.16,T8.1,T7.6</t>
+          <t>T8.6,T8.5,T9.5</t>
         </is>
       </c>
       <c r="I88" s="4" t="n">
@@ -4845,36 +4841,36 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>T8.5</t>
+          <t>T9.1</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>P8</t>
+          <t>P9</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Fund prod treasury with ICP float (10–20 ICP) + …</t>
+          <t>Import mockups (Claude Design), reconcile, desig…</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>human</t>
+          <t>sonnet-5</t>
         </is>
       </c>
       <c r="E89" s="3" t="n">
-        <v>46428</v>
+        <v>46398</v>
       </c>
       <c r="F89" s="3" t="n">
-        <v>46428</v>
+        <v>46401</v>
       </c>
       <c r="G89" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>T8.6</t>
+          <t>T6.10</t>
         </is>
       </c>
       <c r="I89" s="4" t="n">
@@ -4892,36 +4888,36 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>T8.3</t>
+          <t>T9.2</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>P8</t>
+          <t>P9</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Closed beta (10-20 owners)</t>
+          <t>Style public pages: landing, museum, discovery, …</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>human</t>
+          <t>sonnet-5</t>
         </is>
       </c>
       <c r="E90" s="3" t="n">
-        <v>46412</v>
+        <v>46402</v>
       </c>
       <c r="F90" s="3" t="n">
-        <v>46423</v>
+        <v>46407</v>
       </c>
       <c r="G90" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>T8.2,T6.10</t>
+          <t>T9.1</t>
         </is>
       </c>
       <c r="I90" s="4" t="n">
@@ -4939,17 +4935,17 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>T8.4</t>
+          <t>T9.3</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>P8</t>
+          <t>P9</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Beta fixes &amp; tuning</t>
+          <t>Style owner flows: spawn, dashboard, connect age…</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -4958,17 +4954,17 @@
         </is>
       </c>
       <c r="E91" s="3" t="n">
-        <v>46412</v>
+        <v>46402</v>
       </c>
       <c r="F91" s="3" t="n">
-        <v>46423</v>
+        <v>46407</v>
       </c>
       <c r="G91" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>T8.2,T6.10</t>
+          <t>T9.1</t>
         </is>
       </c>
       <c r="I91" s="4" t="n">
@@ -4986,36 +4982,36 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>T8.6</t>
+          <t>T9.4</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>P8</t>
+          <t>P9</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Production deploy, II metadata, treasury watch l…</t>
+          <t>Style admin console + about/legal/practice pages</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>sonnet-5</t>
+          <t>haiku-4.5</t>
         </is>
       </c>
       <c r="E92" s="3" t="n">
-        <v>46426</v>
+        <v>46408</v>
       </c>
       <c r="F92" s="3" t="n">
-        <v>46427</v>
+        <v>46409</v>
       </c>
       <c r="G92" t="n">
         <v>2</v>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>T8.3,T8.4,T8.13</t>
+          <t>T9.1</t>
         </is>
       </c>
       <c r="I92" s="4" t="n">
@@ -5033,36 +5029,36 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>T8.7</t>
+          <t>T9.5</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>P8</t>
+          <t>P9</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Public launch</t>
+          <t>Responsive/mobile pass, visual-regression baseli…</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>human</t>
+          <t>haiku-4.5</t>
         </is>
       </c>
       <c r="E93" s="3" t="n">
-        <v>46429</v>
+        <v>46412</v>
       </c>
       <c r="F93" s="3" t="n">
-        <v>46429</v>
+        <v>46413</v>
       </c>
       <c r="G93" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>T8.6,T8.5,T9.5</t>
+          <t>T9.2,T9.3,T9.4</t>
         </is>
       </c>
       <c r="I93" s="4" t="n">
@@ -5080,36 +5076,36 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>T9.1</t>
+          <t>T8.13</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>P9</t>
+          <t>P8</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Import mockups (Claude Design), reconcile, desig…</t>
+          <t>Custom domain + II alternative origins</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>sonnet-5</t>
+          <t>human</t>
         </is>
       </c>
       <c r="E94" s="3" t="n">
-        <v>46408</v>
+        <v>46400</v>
       </c>
       <c r="F94" s="3" t="n">
-        <v>46413</v>
+        <v>46400</v>
       </c>
       <c r="G94" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>T6.10</t>
+          <t>T8.1</t>
         </is>
       </c>
       <c r="I94" s="4" t="n">
@@ -5127,36 +5123,36 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>T9.2</t>
+          <t>T8.15</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>P9</t>
+          <t>P8</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Style public pages: landing, museum, discovery, …</t>
+          <t>Owner review: discovery + peer-review agent proc…</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>sonnet-5</t>
+          <t>human</t>
         </is>
       </c>
       <c r="E95" s="3" t="n">
-        <v>46414</v>
+        <v>46296</v>
       </c>
       <c r="F95" s="3" t="n">
-        <v>46419</v>
+        <v>46296</v>
       </c>
       <c r="G95" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>T9.1</t>
+          <t>T0.4</t>
         </is>
       </c>
       <c r="I95" s="4" t="n">
@@ -5171,337 +5167,8 @@
         <v/>
       </c>
     </row>
-    <row r="96">
-      <c r="A96" t="inlineStr">
-        <is>
-          <t>T9.3</t>
-        </is>
-      </c>
-      <c r="B96" t="inlineStr">
-        <is>
-          <t>P9</t>
-        </is>
-      </c>
-      <c r="C96" t="inlineStr">
-        <is>
-          <t>Style owner flows: spawn, dashboard, connect age…</t>
-        </is>
-      </c>
-      <c r="D96" t="inlineStr">
-        <is>
-          <t>sonnet-5</t>
-        </is>
-      </c>
-      <c r="E96" s="3" t="n">
-        <v>46414</v>
-      </c>
-      <c r="F96" s="3" t="n">
-        <v>46419</v>
-      </c>
-      <c r="G96" t="n">
-        <v>4</v>
-      </c>
-      <c r="H96" t="inlineStr">
-        <is>
-          <t>T9.1</t>
-        </is>
-      </c>
-      <c r="I96" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J96">
-        <f>IF(I96&gt;=1,"Done",IF(TODAY()&gt;F96,"Late",IF(I96&gt;0,"In progress","Not started")))</f>
-        <v/>
-      </c>
-      <c r="K96">
-        <f>G96*I96</f>
-        <v/>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" t="inlineStr">
-        <is>
-          <t>T9.4</t>
-        </is>
-      </c>
-      <c r="B97" t="inlineStr">
-        <is>
-          <t>P9</t>
-        </is>
-      </c>
-      <c r="C97" t="inlineStr">
-        <is>
-          <t>Style admin console + about/legal/practice pages</t>
-        </is>
-      </c>
-      <c r="D97" t="inlineStr">
-        <is>
-          <t>haiku-4.5</t>
-        </is>
-      </c>
-      <c r="E97" s="3" t="n">
-        <v>46420</v>
-      </c>
-      <c r="F97" s="3" t="n">
-        <v>46421</v>
-      </c>
-      <c r="G97" t="n">
-        <v>2</v>
-      </c>
-      <c r="H97" t="inlineStr">
-        <is>
-          <t>T9.1</t>
-        </is>
-      </c>
-      <c r="I97" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J97">
-        <f>IF(I97&gt;=1,"Done",IF(TODAY()&gt;F97,"Late",IF(I97&gt;0,"In progress","Not started")))</f>
-        <v/>
-      </c>
-      <c r="K97">
-        <f>G97*I97</f>
-        <v/>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" t="inlineStr">
-        <is>
-          <t>T9.5</t>
-        </is>
-      </c>
-      <c r="B98" t="inlineStr">
-        <is>
-          <t>P9</t>
-        </is>
-      </c>
-      <c r="C98" t="inlineStr">
-        <is>
-          <t>Responsive/mobile pass, visual-regression baseli…</t>
-        </is>
-      </c>
-      <c r="D98" t="inlineStr">
-        <is>
-          <t>haiku-4.5</t>
-        </is>
-      </c>
-      <c r="E98" s="3" t="n">
-        <v>46422</v>
-      </c>
-      <c r="F98" s="3" t="n">
-        <v>46423</v>
-      </c>
-      <c r="G98" t="n">
-        <v>2</v>
-      </c>
-      <c r="H98" t="inlineStr">
-        <is>
-          <t>T9.2,T9.3,T9.4</t>
-        </is>
-      </c>
-      <c r="I98" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J98">
-        <f>IF(I98&gt;=1,"Done",IF(TODAY()&gt;F98,"Late",IF(I98&gt;0,"In progress","Not started")))</f>
-        <v/>
-      </c>
-      <c r="K98">
-        <f>G98*I98</f>
-        <v/>
-      </c>
-    </row>
-    <row r="99">
-      <c r="A99" t="inlineStr">
-        <is>
-          <t>T8.13</t>
-        </is>
-      </c>
-      <c r="B99" t="inlineStr">
-        <is>
-          <t>P8</t>
-        </is>
-      </c>
-      <c r="C99" t="inlineStr">
-        <is>
-          <t>Custom domain + II alternative origins</t>
-        </is>
-      </c>
-      <c r="D99" t="inlineStr">
-        <is>
-          <t>human</t>
-        </is>
-      </c>
-      <c r="E99" s="3" t="n">
-        <v>46409</v>
-      </c>
-      <c r="F99" s="3" t="n">
-        <v>46409</v>
-      </c>
-      <c r="G99" t="n">
-        <v>1</v>
-      </c>
-      <c r="H99" t="inlineStr">
-        <is>
-          <t>T8.1</t>
-        </is>
-      </c>
-      <c r="I99" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J99">
-        <f>IF(I99&gt;=1,"Done",IF(TODAY()&gt;F99,"Late",IF(I99&gt;0,"In progress","Not started")))</f>
-        <v/>
-      </c>
-      <c r="K99">
-        <f>G99*I99</f>
-        <v/>
-      </c>
-    </row>
-    <row r="100">
-      <c r="A100" t="inlineStr">
-        <is>
-          <t>T8.15</t>
-        </is>
-      </c>
-      <c r="B100" t="inlineStr">
-        <is>
-          <t>P8</t>
-        </is>
-      </c>
-      <c r="C100" t="inlineStr">
-        <is>
-          <t>Owner review: discovery + peer-review agent proc…</t>
-        </is>
-      </c>
-      <c r="D100" t="inlineStr">
-        <is>
-          <t>human</t>
-        </is>
-      </c>
-      <c r="E100" s="3" t="n">
-        <v>46296</v>
-      </c>
-      <c r="F100" s="3" t="n">
-        <v>46296</v>
-      </c>
-      <c r="G100" t="n">
-        <v>1</v>
-      </c>
-      <c r="H100" t="inlineStr">
-        <is>
-          <t>T0.4</t>
-        </is>
-      </c>
-      <c r="I100" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J100">
-        <f>IF(I100&gt;=1,"Done",IF(TODAY()&gt;F100,"Late",IF(I100&gt;0,"In progress","Not started")))</f>
-        <v/>
-      </c>
-      <c r="K100">
-        <f>G100*I100</f>
-        <v/>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" t="inlineStr">
-        <is>
-          <t>T8.8</t>
-        </is>
-      </c>
-      <c r="B101" t="inlineStr">
-        <is>
-          <t>P8</t>
-        </is>
-      </c>
-      <c r="C101" t="inlineStr">
-        <is>
-          <t>Compliance check for crypto fuel packs (recommen…</t>
-        </is>
-      </c>
-      <c r="D101" t="inlineStr">
-        <is>
-          <t>human</t>
-        </is>
-      </c>
-      <c r="E101" s="3" t="n">
-        <v>46296</v>
-      </c>
-      <c r="F101" s="3" t="n">
-        <v>46302</v>
-      </c>
-      <c r="G101" t="n">
-        <v>5</v>
-      </c>
-      <c r="H101" t="inlineStr">
-        <is>
-          <t>T0.4</t>
-        </is>
-      </c>
-      <c r="I101" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J101">
-        <f>IF(I101&gt;=1,"Done",IF(TODAY()&gt;F101,"Late",IF(I101&gt;0,"In progress","Not started")))</f>
-        <v/>
-      </c>
-      <c r="K101">
-        <f>G101*I101</f>
-        <v/>
-      </c>
-    </row>
-    <row r="102">
-      <c r="A102" t="inlineStr">
-        <is>
-          <t>T8.9</t>
-        </is>
-      </c>
-      <c r="B102" t="inlineStr">
-        <is>
-          <t>P8</t>
-        </is>
-      </c>
-      <c r="C102" t="inlineStr">
-        <is>
-          <t>Enable BTC/ETH on production</t>
-        </is>
-      </c>
-      <c r="D102" t="inlineStr">
-        <is>
-          <t>human</t>
-        </is>
-      </c>
-      <c r="E102" s="3" t="n">
-        <v>46428</v>
-      </c>
-      <c r="F102" s="3" t="n">
-        <v>46428</v>
-      </c>
-      <c r="G102" t="n">
-        <v>1</v>
-      </c>
-      <c r="H102" t="inlineStr">
-        <is>
-          <t>T8.6,T8.8</t>
-        </is>
-      </c>
-      <c r="I102" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J102">
-        <f>IF(I102&gt;=1,"Done",IF(TODAY()&gt;F102,"Late",IF(I102&gt;0,"In progress","Not started")))</f>
-        <v/>
-      </c>
-      <c r="K102">
-        <f>G102*I102</f>
-        <v/>
-      </c>
-    </row>
   </sheetData>
-  <conditionalFormatting sqref="L2:AF102">
+  <conditionalFormatting sqref="L2:AE95">
     <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="1">
       <formula>AND(L$1+6&gt;=$E2,L$1&lt;=$F2,L$1&lt;=$E2+($F2-$E2)*$I2)</formula>
     </cfRule>
@@ -5539,7 +5206,7 @@
       <formula>AND(TODAY()&gt;=L$1,TODAY()&lt;L$1+7)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J2:J102">
+  <conditionalFormatting sqref="J2:J95">
     <cfRule type="expression" priority="13" dxfId="12">
       <formula>LEFT(J2,4)="Late"</formula>
     </cfRule>
@@ -5867,7 +5534,7 @@
         <v>46336</v>
       </c>
       <c r="I7" s="3" t="n">
-        <v>46372</v>
+        <v>46364</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
@@ -5906,10 +5573,10 @@
         <v/>
       </c>
       <c r="H8" s="3" t="n">
-        <v>46367</v>
+        <v>46360</v>
       </c>
       <c r="I8" s="3" t="n">
-        <v>46405</v>
+        <v>46394</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
@@ -5948,10 +5615,10 @@
         <v/>
       </c>
       <c r="H9" s="3" t="n">
-        <v>46373</v>
+        <v>46364</v>
       </c>
       <c r="I9" s="3" t="n">
-        <v>46407</v>
+        <v>46398</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
@@ -5993,7 +5660,7 @@
         <v>46296</v>
       </c>
       <c r="I10" s="3" t="n">
-        <v>46429</v>
+        <v>46420</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
@@ -6032,10 +5699,10 @@
         <v/>
       </c>
       <c r="H11" s="3" t="n">
-        <v>46408</v>
+        <v>46398</v>
       </c>
       <c r="I11" s="3" t="n">
-        <v>46423</v>
+        <v>46413</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
@@ -6070,14 +5737,14 @@
         <v/>
       </c>
       <c r="G12" s="17">
-        <f>IF(C12&gt;0,SUM(Gantt!K2:K102)/C12,0)</f>
+        <f>IF(C12&gt;0,SUM(Gantt!K2:K95)/C12,0)</f>
         <v/>
       </c>
       <c r="H12" s="18" t="n">
         <v>46286</v>
       </c>
       <c r="I12" s="18" t="n">
-        <v>46429</v>
+        <v>46420</v>
       </c>
     </row>
     <row r="14">

</xml_diff>

<commit_message>
deploy-local: wire platform<->payments ids; add T9.6 screenshot grid task; fix T3.7 traceability claim
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/space-compute-gantt-v3.xlsx
+++ b/docs/space-compute-gantt-v3.xlsx
@@ -600,7 +600,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE95"/>
+  <dimension ref="A1:AE96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -4823,7 +4823,7 @@
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>T8.6,T8.5,T9.5</t>
+          <t>T8.6,T8.5,T9.6</t>
         </is>
       </c>
       <c r="I88" s="4" t="n">
@@ -5076,36 +5076,36 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>T8.13</t>
+          <t>T9.6</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>P8</t>
+          <t>P9</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Custom domain + II alternative origins</t>
+          <t>Full-app screenshot grid: labeled Playwright con…</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>human</t>
+          <t>haiku-4.5</t>
         </is>
       </c>
       <c r="E94" s="3" t="n">
-        <v>46400</v>
+        <v>46414</v>
       </c>
       <c r="F94" s="3" t="n">
-        <v>46400</v>
+        <v>46414</v>
       </c>
       <c r="G94" t="n">
         <v>1</v>
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>T8.1</t>
+          <t>T9.5</t>
         </is>
       </c>
       <c r="I94" s="4" t="n">
@@ -5123,7 +5123,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>T8.15</t>
+          <t>T8.13</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -5133,7 +5133,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Owner review: discovery + peer-review agent proc…</t>
+          <t>Custom domain + II alternative origins</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -5142,17 +5142,17 @@
         </is>
       </c>
       <c r="E95" s="3" t="n">
-        <v>46296</v>
+        <v>46400</v>
       </c>
       <c r="F95" s="3" t="n">
-        <v>46296</v>
+        <v>46400</v>
       </c>
       <c r="G95" t="n">
         <v>1</v>
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>T0.4</t>
+          <t>T8.1</t>
         </is>
       </c>
       <c r="I95" s="4" t="n">
@@ -5167,8 +5167,55 @@
         <v/>
       </c>
     </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>T8.15</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>P8</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Owner review: discovery + peer-review agent proc…</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>human</t>
+        </is>
+      </c>
+      <c r="E96" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="F96" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="G96" t="n">
+        <v>1</v>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>T0.4</t>
+        </is>
+      </c>
+      <c r="I96" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J96">
+        <f>IF(I96&gt;=1,"Done",IF(TODAY()&gt;F96,"Late",IF(I96&gt;0,"In progress","Not started")))</f>
+        <v/>
+      </c>
+      <c r="K96">
+        <f>G96*I96</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="L2:AE95">
+  <conditionalFormatting sqref="L2:AE96">
     <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="1">
       <formula>AND(L$1+6&gt;=$E2,L$1&lt;=$F2,L$1&lt;=$E2+($F2-$E2)*$I2)</formula>
     </cfRule>
@@ -5206,7 +5253,7 @@
       <formula>AND(TODAY()&gt;=L$1,TODAY()&lt;L$1+7)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J2:J95">
+  <conditionalFormatting sqref="J2:J96">
     <cfRule type="expression" priority="13" dxfId="12">
       <formula>LEFT(J2,4)="Late"</formula>
     </cfRule>
@@ -5702,7 +5749,7 @@
         <v>46398</v>
       </c>
       <c r="I11" s="3" t="n">
-        <v>46413</v>
+        <v>46414</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
@@ -5737,7 +5784,7 @@
         <v/>
       </c>
       <c r="G12" s="17">
-        <f>IF(C12&gt;0,SUM(Gantt!K2:K95)/C12,0)</f>
+        <f>IF(C12&gt;0,SUM(Gantt!K2:K96)/C12,0)</f>
         <v/>
       </c>
       <c r="H12" s="18" t="n">
@@ -5904,7 +5951,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>T9.5</t>
+          <t>T9.6</t>
         </is>
       </c>
       <c r="C7" s="3">

</xml_diff>

<commit_message>
T4.10, T4.11 done: ledger entries
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/space-compute-gantt-v3.xlsx
+++ b/docs/space-compute-gantt-v3.xlsx
@@ -2806,7 +2806,7 @@
         </is>
       </c>
       <c r="I45" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J45">
         <f>IF(I45&gt;=1,"Done",IF(TODAY()&gt;F45,"Late",IF(I45&gt;0,"In progress","Not started")))</f>
@@ -2853,7 +2853,7 @@
         </is>
       </c>
       <c r="I46" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J46">
         <f>IF(I46&gt;=1,"Done",IF(TODAY()&gt;F46,"Late",IF(I46&gt;0,"In progress","Not started")))</f>

</xml_diff>

<commit_message>
T7.3 done; add T7.12 (storage per classification + indexed gold get_task) from T7.3 findings
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/space-compute-gantt-v3.xlsx
+++ b/docs/space-compute-gantt-v3.xlsx
@@ -600,7 +600,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE96"/>
+  <dimension ref="A1:AE97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -4075,7 +4075,7 @@
         </is>
       </c>
       <c r="I72" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J72">
         <f>IF(I72&gt;=1,"Done",IF(TODAY()&gt;F72,"Late",IF(I72&gt;0,"In progress","Not started")))</f>
@@ -4390,10 +4390,10 @@
         </is>
       </c>
       <c r="E79" s="3" t="n">
-        <v>46394</v>
+        <v>46395</v>
       </c>
       <c r="F79" s="3" t="n">
-        <v>46395</v>
+        <v>46398</v>
       </c>
       <c r="G79" t="n">
         <v>2</v>
@@ -4418,36 +4418,36 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>T8.14</t>
+          <t>T7.12</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>P8</t>
+          <t>P7</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Create Cloudflare R2 bucket + API token + custom…</t>
+          <t>Platform storage per classification (~44 KB → ≤1…</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>human</t>
+          <t>opus-5.5 (high)</t>
         </is>
       </c>
       <c r="E80" s="3" t="n">
-        <v>46316</v>
+        <v>46394</v>
       </c>
       <c r="F80" s="3" t="n">
-        <v>46316</v>
+        <v>46395</v>
       </c>
       <c r="G80" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>T1.7</t>
+          <t>T7.3</t>
         </is>
       </c>
       <c r="I80" s="4" t="n">
@@ -4465,7 +4465,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>T8.16</t>
+          <t>T8.14</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -4475,26 +4475,26 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Scale dataset to 20,000 subjects (R-62) and publ…</t>
+          <t>Create Cloudflare R2 bucket + API token + custom…</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>haiku-4.5</t>
+          <t>human</t>
         </is>
       </c>
       <c r="E81" s="3" t="n">
-        <v>46395</v>
+        <v>46316</v>
       </c>
       <c r="F81" s="3" t="n">
-        <v>46395</v>
+        <v>46316</v>
       </c>
       <c r="G81" t="n">
         <v>1</v>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>T8.14</t>
+          <t>T1.7</t>
         </is>
       </c>
       <c r="I81" s="4" t="n">
@@ -4512,7 +4512,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>T8.1</t>
+          <t>T8.16</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -4522,30 +4522,30 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Staging deploy, deploy workflow, snapshots, cycl…</t>
+          <t>Scale dataset to 20,000 subjects (R-62) and publ…</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>sonnet-5</t>
+          <t>haiku-4.5</t>
         </is>
       </c>
       <c r="E82" s="3" t="n">
         <v>46398</v>
       </c>
       <c r="F82" s="3" t="n">
-        <v>46399</v>
+        <v>46398</v>
       </c>
       <c r="G82" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>T7.1</t>
+          <t>T8.14</t>
         </is>
       </c>
       <c r="I82" s="4" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="J82">
         <f>IF(I82&gt;=1,"Done",IF(TODAY()&gt;F82,"Late",IF(I82&gt;0,"In progress","Not started")))</f>
@@ -4559,7 +4559,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>T8.2</t>
+          <t>T8.1</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -4569,30 +4569,30 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Upload subjects/protocol/honeypots to staging</t>
+          <t>Staging deploy, deploy workflow, snapshots, cycl…</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>haiku-4.5</t>
+          <t>sonnet-5</t>
         </is>
       </c>
       <c r="E83" s="3" t="n">
-        <v>46400</v>
+        <v>46399</v>
       </c>
       <c r="F83" s="3" t="n">
         <v>46400</v>
       </c>
       <c r="G83" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>T8.16,T8.1,T7.6</t>
+          <t>T7.1</t>
         </is>
       </c>
       <c r="I83" s="4" t="n">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="J83">
         <f>IF(I83&gt;=1,"Done",IF(TODAY()&gt;F83,"Late",IF(I83&gt;0,"In progress","Not started")))</f>
@@ -4606,7 +4606,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>T8.5</t>
+          <t>T8.2</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -4616,26 +4616,26 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Fund prod treasury with ICP float (10–20 ICP) + …</t>
+          <t>Upload subjects/protocol/honeypots to staging</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>human</t>
+          <t>haiku-4.5</t>
         </is>
       </c>
       <c r="E84" s="3" t="n">
-        <v>46419</v>
+        <v>46401</v>
       </c>
       <c r="F84" s="3" t="n">
-        <v>46419</v>
+        <v>46401</v>
       </c>
       <c r="G84" t="n">
         <v>1</v>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>T8.6</t>
+          <t>T8.16,T8.1,T7.6</t>
         </is>
       </c>
       <c r="I84" s="4" t="n">
@@ -4653,7 +4653,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>T8.3</t>
+          <t>T8.5</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -4663,7 +4663,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Closed beta (10-20 owners)</t>
+          <t>Fund prod treasury with ICP float (10–20 ICP) + …</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -4672,17 +4672,17 @@
         </is>
       </c>
       <c r="E85" s="3" t="n">
-        <v>46401</v>
+        <v>46420</v>
       </c>
       <c r="F85" s="3" t="n">
-        <v>46414</v>
+        <v>46420</v>
       </c>
       <c r="G85" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>T8.2,T6.10</t>
+          <t>T8.6</t>
         </is>
       </c>
       <c r="I85" s="4" t="n">
@@ -4700,7 +4700,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>T8.4</t>
+          <t>T8.3</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -4710,19 +4710,19 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Beta fixes &amp; tuning</t>
+          <t>Closed beta (10-20 owners)</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>sonnet-5</t>
+          <t>human</t>
         </is>
       </c>
       <c r="E86" s="3" t="n">
-        <v>46401</v>
+        <v>46402</v>
       </c>
       <c r="F86" s="3" t="n">
-        <v>46414</v>
+        <v>46415</v>
       </c>
       <c r="G86" t="n">
         <v>10</v>
@@ -4747,7 +4747,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>T8.6</t>
+          <t>T8.4</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -4757,7 +4757,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Production deploy, II metadata, treasury watch l…</t>
+          <t>Beta fixes &amp; tuning</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -4766,17 +4766,17 @@
         </is>
       </c>
       <c r="E87" s="3" t="n">
+        <v>46402</v>
+      </c>
+      <c r="F87" s="3" t="n">
         <v>46415</v>
       </c>
-      <c r="F87" s="3" t="n">
-        <v>46416</v>
-      </c>
       <c r="G87" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>T8.3,T8.4,T8.13</t>
+          <t>T8.2,T6.10</t>
         </is>
       </c>
       <c r="I87" s="4" t="n">
@@ -4794,7 +4794,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>T8.7</t>
+          <t>T8.6</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -4804,26 +4804,26 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Public launch</t>
+          <t>Production deploy, II metadata, treasury watch l…</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>human</t>
+          <t>sonnet-5</t>
         </is>
       </c>
       <c r="E88" s="3" t="n">
-        <v>46420</v>
+        <v>46416</v>
       </c>
       <c r="F88" s="3" t="n">
-        <v>46420</v>
+        <v>46419</v>
       </c>
       <c r="G88" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>T8.6,T8.5,T9.6</t>
+          <t>T8.3,T8.4,T8.13</t>
         </is>
       </c>
       <c r="I88" s="4" t="n">
@@ -4841,36 +4841,36 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>T9.1</t>
+          <t>T8.7</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>P9</t>
+          <t>P8</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Import mockups (Claude Design), reconcile, desig…</t>
+          <t>Public launch</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>sonnet-5</t>
+          <t>human</t>
         </is>
       </c>
       <c r="E89" s="3" t="n">
-        <v>46398</v>
+        <v>46421</v>
       </c>
       <c r="F89" s="3" t="n">
-        <v>46401</v>
+        <v>46421</v>
       </c>
       <c r="G89" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>T6.10</t>
+          <t>T8.6,T8.5,T9.6</t>
         </is>
       </c>
       <c r="I89" s="4" t="n">
@@ -4888,7 +4888,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>T9.2</t>
+          <t>T9.1</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -4898,7 +4898,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Style public pages: landing, museum, discovery, …</t>
+          <t>Import mockups (Claude Design), reconcile, desig…</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -4907,17 +4907,17 @@
         </is>
       </c>
       <c r="E90" s="3" t="n">
+        <v>46399</v>
+      </c>
+      <c r="F90" s="3" t="n">
         <v>46402</v>
-      </c>
-      <c r="F90" s="3" t="n">
-        <v>46407</v>
       </c>
       <c r="G90" t="n">
         <v>4</v>
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>T9.1</t>
+          <t>T6.10</t>
         </is>
       </c>
       <c r="I90" s="4" t="n">
@@ -4935,7 +4935,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>T9.3</t>
+          <t>T9.2</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -4945,7 +4945,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Style owner flows: spawn, dashboard, connect age…</t>
+          <t>Style public pages: landing, museum, discovery, …</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -4954,10 +4954,10 @@
         </is>
       </c>
       <c r="E91" s="3" t="n">
-        <v>46402</v>
+        <v>46405</v>
       </c>
       <c r="F91" s="3" t="n">
-        <v>46407</v>
+        <v>46408</v>
       </c>
       <c r="G91" t="n">
         <v>4</v>
@@ -4982,7 +4982,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>T9.4</t>
+          <t>T9.3</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -4992,22 +4992,22 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Style admin console + about/legal/practice pages</t>
+          <t>Style owner flows: spawn, dashboard, connect age…</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>haiku-4.5</t>
+          <t>sonnet-5</t>
         </is>
       </c>
       <c r="E92" s="3" t="n">
+        <v>46405</v>
+      </c>
+      <c r="F92" s="3" t="n">
         <v>46408</v>
       </c>
-      <c r="F92" s="3" t="n">
-        <v>46409</v>
-      </c>
       <c r="G92" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H92" t="inlineStr">
         <is>
@@ -5029,7 +5029,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>T9.5</t>
+          <t>T9.4</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -5039,7 +5039,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Responsive/mobile pass, visual-regression baseli…</t>
+          <t>Style admin console + about/legal/practice pages</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -5048,17 +5048,17 @@
         </is>
       </c>
       <c r="E93" s="3" t="n">
+        <v>46409</v>
+      </c>
+      <c r="F93" s="3" t="n">
         <v>46412</v>
-      </c>
-      <c r="F93" s="3" t="n">
-        <v>46413</v>
       </c>
       <c r="G93" t="n">
         <v>2</v>
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>T9.2,T9.3,T9.4</t>
+          <t>T9.1</t>
         </is>
       </c>
       <c r="I93" s="4" t="n">
@@ -5076,7 +5076,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>T9.6</t>
+          <t>T9.5</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -5086,7 +5086,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Full-app screenshot grid: labeled Playwright con…</t>
+          <t>Responsive/mobile pass, visual-regression baseli…</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -5095,17 +5095,17 @@
         </is>
       </c>
       <c r="E94" s="3" t="n">
-        <v>46414</v>
+        <v>46413</v>
       </c>
       <c r="F94" s="3" t="n">
         <v>46414</v>
       </c>
       <c r="G94" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>T9.5</t>
+          <t>T9.2,T9.3,T9.4</t>
         </is>
       </c>
       <c r="I94" s="4" t="n">
@@ -5123,36 +5123,36 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>T8.13</t>
+          <t>T9.6</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>P8</t>
+          <t>P9</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Custom domain + II alternative origins</t>
+          <t>Full-app screenshot grid: labeled Playwright con…</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>human</t>
+          <t>haiku-4.5</t>
         </is>
       </c>
       <c r="E95" s="3" t="n">
-        <v>46400</v>
+        <v>46415</v>
       </c>
       <c r="F95" s="3" t="n">
-        <v>46400</v>
+        <v>46415</v>
       </c>
       <c r="G95" t="n">
         <v>1</v>
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>T8.1</t>
+          <t>T9.5</t>
         </is>
       </c>
       <c r="I95" s="4" t="n">
@@ -5170,7 +5170,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>T8.15</t>
+          <t>T8.13</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -5180,7 +5180,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Owner review: discovery + peer-review agent proc…</t>
+          <t>Custom domain + II alternative origins</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -5189,17 +5189,17 @@
         </is>
       </c>
       <c r="E96" s="3" t="n">
-        <v>46296</v>
+        <v>46401</v>
       </c>
       <c r="F96" s="3" t="n">
-        <v>46296</v>
+        <v>46401</v>
       </c>
       <c r="G96" t="n">
         <v>1</v>
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>T0.4</t>
+          <t>T8.1</t>
         </is>
       </c>
       <c r="I96" s="4" t="n">
@@ -5214,8 +5214,55 @@
         <v/>
       </c>
     </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>T8.15</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>P8</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Owner review: discovery + peer-review agent proc…</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>human</t>
+        </is>
+      </c>
+      <c r="E97" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="F97" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="G97" t="n">
+        <v>1</v>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>T0.4</t>
+        </is>
+      </c>
+      <c r="I97" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J97">
+        <f>IF(I97&gt;=1,"Done",IF(TODAY()&gt;F97,"Late",IF(I97&gt;0,"In progress","Not started")))</f>
+        <v/>
+      </c>
+      <c r="K97">
+        <f>G97*I97</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="L2:AE96">
+  <conditionalFormatting sqref="L2:AE97">
     <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="1">
       <formula>AND(L$1+6&gt;=$E2,L$1&lt;=$F2,L$1&lt;=$E2+($F2-$E2)*$I2)</formula>
     </cfRule>
@@ -5253,7 +5300,7 @@
       <formula>AND(TODAY()&gt;=L$1,TODAY()&lt;L$1+7)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J2:J96">
+  <conditionalFormatting sqref="J2:J97">
     <cfRule type="expression" priority="13" dxfId="12">
       <formula>LEFT(J2,4)="Late"</formula>
     </cfRule>
@@ -5707,7 +5754,7 @@
         <v>46296</v>
       </c>
       <c r="I10" s="3" t="n">
-        <v>46420</v>
+        <v>46421</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
@@ -5746,10 +5793,10 @@
         <v/>
       </c>
       <c r="H11" s="3" t="n">
-        <v>46398</v>
+        <v>46399</v>
       </c>
       <c r="I11" s="3" t="n">
-        <v>46414</v>
+        <v>46415</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
@@ -5784,14 +5831,14 @@
         <v/>
       </c>
       <c r="G12" s="17">
-        <f>IF(C12&gt;0,SUM(Gantt!K2:K96)/C12,0)</f>
+        <f>IF(C12&gt;0,SUM(Gantt!K2:K97)/C12,0)</f>
         <v/>
       </c>
       <c r="H12" s="18" t="n">
         <v>46286</v>
       </c>
       <c r="I12" s="18" t="n">
-        <v>46420</v>
+        <v>46421</v>
       </c>
     </row>
     <row r="14">

</xml_diff>